<commit_message>
added more historic data, adapted scoring scheme for older leagues
</commit_message>
<xml_diff>
--- a/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
+++ b/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Dropbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5125C2A0-06AD-47D6-A430-EA2EE1CF2B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3938F41E-A811-4515-8485-EFC252B27397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D7BAE6BD-B2A4-4DD1-AF79-906BD29E778A}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
   <si>
     <t>Marco Hürdler</t>
   </si>
@@ -144,15 +144,28 @@
   <si>
     <t>Rang</t>
   </si>
+  <si>
+    <t>Donaubowler Clubmeisterschaft 2026 / Stand 19.05.26</t>
+  </si>
+  <si>
+    <t>Richard Zorzi</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -190,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -213,11 +226,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -248,6 +270,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -584,7 +609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{171CD03C-3231-415F-B722-714CA0D22DE3}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:AQ33"/>
+  <dimension ref="A1:AQ34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
@@ -613,276 +638,191 @@
     <col min="42" max="43" width="6.5703125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="U1" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="V1" s="12"/>
-      <c r="W1" s="12"/>
-      <c r="X1" s="12"/>
-      <c r="Y1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA1" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB1" s="12"/>
-      <c r="AC1" s="12"/>
-      <c r="AD1" s="12"/>
-      <c r="AE1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="AF1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG1" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="AH1" s="12"/>
-      <c r="AI1" s="12"/>
-      <c r="AJ1" s="12"/>
-      <c r="AK1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="AL1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="AN1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>30</v>
-      </c>
+    <row r="1" spans="1:43" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="B1" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3">
-        <v>216</v>
-      </c>
-      <c r="D2" s="3">
-        <v>239</v>
-      </c>
-      <c r="E2" s="3">
-        <v>224</v>
-      </c>
-      <c r="F2" s="3">
-        <v>209</v>
-      </c>
-      <c r="G2" s="9">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4">
-        <f t="shared" ref="H2:H20" si="0">SUM(C2:G2)</f>
-        <v>888</v>
-      </c>
-      <c r="I2" s="3">
-        <v>245</v>
-      </c>
-      <c r="J2" s="3">
-        <v>194</v>
-      </c>
-      <c r="K2" s="3">
-        <v>190</v>
-      </c>
-      <c r="L2" s="3">
-        <v>216</v>
-      </c>
-      <c r="M2" s="9">
-        <v>0</v>
-      </c>
-      <c r="N2" s="4">
-        <f t="shared" ref="N2:N20" si="1">SUM(I2:L2)</f>
-        <v>845</v>
-      </c>
-      <c r="O2" s="3">
-        <v>215</v>
-      </c>
-      <c r="P2" s="3">
-        <v>179</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>217</v>
-      </c>
-      <c r="R2" s="3">
-        <v>192</v>
-      </c>
-      <c r="S2" s="9">
-        <v>0</v>
-      </c>
-      <c r="T2" s="4">
-        <f t="shared" ref="T2:T20" si="2">SUM(O2:R2)</f>
-        <v>803</v>
-      </c>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="9">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="4">
-        <f t="shared" ref="Z2:Z20" si="3">SUM(U2:X2)</f>
-        <v>0</v>
-      </c>
-      <c r="AA2" s="3"/>
-      <c r="AB2" s="3"/>
-      <c r="AC2" s="3"/>
-      <c r="AD2" s="3"/>
-      <c r="AE2" s="9">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="4">
-        <f t="shared" ref="AF2:AF20" si="4">SUM(AA2:AD2)</f>
-        <v>0</v>
-      </c>
-      <c r="AG2" s="3"/>
-      <c r="AH2" s="3"/>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-      <c r="AK2" s="9">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="4">
-        <f t="shared" ref="AL2:AL20" si="5">SUM(AG2:AJ2)</f>
-        <v>0</v>
-      </c>
-      <c r="AM2" s="6" cm="1">
-        <f t="array" ref="AM2">SUM(C2:F2+I2:L2+O2:R2+U2:X2+AA2:AD2+AG2:AJ2)</f>
-        <v>2536</v>
-      </c>
-      <c r="AN2" s="8">
-        <f t="shared" ref="AN2:AN20" si="6">SUM(H2+N2+T2+Z2+AF2+AL2)</f>
-        <v>2536</v>
-      </c>
-      <c r="AO2">
-        <v>200</v>
-      </c>
-      <c r="AP2" s="11">
-        <v>207</v>
-      </c>
-      <c r="AQ2" s="11">
-        <f t="shared" ref="AQ2:AQ20" si="7">SUM((AO2-AP2)*0.7)</f>
-        <v>-4.8999999999999995</v>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AA2" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB2" s="12"/>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="12"/>
+      <c r="AE2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AF2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AG2" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="AH2" s="12"/>
+      <c r="AI2" s="12"/>
+      <c r="AJ2" s="12"/>
+      <c r="AK2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AL2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AN2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AP2" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D3" s="3">
-        <v>193</v>
+        <v>227</v>
       </c>
       <c r="E3" s="3">
         <v>205</v>
       </c>
       <c r="F3" s="3">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="G3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H3" s="4">
-        <f t="shared" si="0"/>
-        <v>815</v>
+        <f>SUM(C3:G3)</f>
+        <v>843</v>
       </c>
       <c r="I3" s="3">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="J3" s="3">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K3" s="3">
+        <v>183</v>
+      </c>
+      <c r="L3" s="3">
         <v>224</v>
       </c>
-      <c r="L3" s="3">
-        <v>189</v>
-      </c>
       <c r="M3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="N3" s="4">
-        <f t="shared" si="1"/>
-        <v>880</v>
-      </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+        <f>SUM(I3:L3)</f>
+        <v>830</v>
+      </c>
+      <c r="O3" s="3">
+        <v>214</v>
+      </c>
+      <c r="P3" s="3">
+        <v>203</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>219</v>
+      </c>
+      <c r="R3" s="3">
+        <v>239</v>
+      </c>
       <c r="S3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="T3" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>SUM(O3:R3)</f>
+        <v>875</v>
       </c>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Z3" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U3:X3)</f>
         <v>0</v>
       </c>
       <c r="AA3" s="3"/>
@@ -890,10 +830,10 @@
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AF3" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA3:AD3)</f>
         <v>0</v>
       </c>
       <c r="AG3" s="3"/>
@@ -901,96 +841,104 @@
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AL3" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG3:AJ3)</f>
         <v>0</v>
       </c>
       <c r="AM3" s="6" cm="1">
         <f t="array" ref="AM3">SUM(C3:F3+I3:L3+O3:R3+U3:X3+AA3:AD3+AG3:AJ3)</f>
-        <v>1675</v>
+        <v>2532</v>
       </c>
       <c r="AN3" s="8">
-        <f t="shared" si="6"/>
-        <v>1695</v>
+        <f>SUM(H3+N3+T3+Z3+AF3+AL3)</f>
+        <v>2548</v>
       </c>
       <c r="AO3">
         <v>200</v>
       </c>
       <c r="AP3" s="11">
-        <v>193.33</v>
+        <v>193.83</v>
       </c>
       <c r="AQ3" s="11">
-        <f t="shared" si="7"/>
-        <v>4.6689999999999907</v>
+        <f>SUM((AO3-AP3)*0.7)</f>
+        <v>4.3189999999999911</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="D4" s="3">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E4" s="3">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="F4" s="3">
+        <v>209</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <f>SUM(C4:G4)</f>
+        <v>888</v>
+      </c>
+      <c r="I4" s="3">
+        <v>245</v>
+      </c>
+      <c r="J4" s="3">
+        <v>194</v>
+      </c>
+      <c r="K4" s="3">
         <v>190</v>
       </c>
-      <c r="G4" s="9">
-        <v>16</v>
-      </c>
-      <c r="H4" s="4">
-        <f t="shared" si="0"/>
-        <v>843</v>
-      </c>
-      <c r="I4" s="3">
-        <v>191</v>
-      </c>
-      <c r="J4" s="3">
-        <v>232</v>
-      </c>
-      <c r="K4" s="3">
-        <v>183</v>
-      </c>
       <c r="L4" s="3">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="M4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N4" s="4">
-        <f t="shared" si="1"/>
-        <v>830</v>
-      </c>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+        <f>SUM(I4:L4)</f>
+        <v>845</v>
+      </c>
+      <c r="O4" s="3">
+        <v>215</v>
+      </c>
+      <c r="P4" s="3">
+        <v>179</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>217</v>
+      </c>
+      <c r="R4" s="3">
+        <v>192</v>
+      </c>
       <c r="S4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="T4" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>SUM(O4:R4)</f>
+        <v>803</v>
       </c>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U4:X4)</f>
         <v>0</v>
       </c>
       <c r="AA4" s="3"/>
@@ -998,10 +946,10 @@
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AF4" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA4:AD4)</f>
         <v>0</v>
       </c>
       <c r="AG4" s="3"/>
@@ -1009,34 +957,34 @@
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AL4" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG4:AJ4)</f>
         <v>0</v>
       </c>
       <c r="AM4" s="6" cm="1">
         <f t="array" ref="AM4">SUM(C4:F4+I4:L4+O4:R4+U4:X4+AA4:AD4+AG4:AJ4)</f>
-        <v>1657</v>
+        <v>2536</v>
       </c>
       <c r="AN4" s="8">
-        <f t="shared" si="6"/>
-        <v>1673</v>
+        <f>SUM(H4+N4+T4+Z4+AF4+AL4)</f>
+        <v>2536</v>
       </c>
       <c r="AO4">
         <v>200</v>
       </c>
       <c r="AP4" s="11">
-        <v>193.83</v>
+        <v>207</v>
       </c>
       <c r="AQ4" s="11">
-        <f t="shared" si="7"/>
-        <v>4.3189999999999911</v>
+        <f>SUM((AO4-AP4)*0.7)</f>
+        <v>-4.8999999999999995</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
@@ -1057,7 +1005,7 @@
         <v>76</v>
       </c>
       <c r="H5" s="4">
-        <f t="shared" si="0"/>
+        <f>SUM(C5:G5)</f>
         <v>823</v>
       </c>
       <c r="I5" s="3">
@@ -1076,19 +1024,27 @@
         <v>76</v>
       </c>
       <c r="N5" s="4">
-        <f t="shared" si="1"/>
+        <f>SUM(I5:L5)</f>
         <v>781</v>
       </c>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
+      <c r="O5" s="3">
+        <v>148</v>
+      </c>
+      <c r="P5" s="3">
+        <v>149</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>177</v>
+      </c>
+      <c r="R5" s="3">
+        <v>182</v>
+      </c>
       <c r="S5" s="9">
         <v>76</v>
       </c>
       <c r="T5" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>SUM(O5:R5)</f>
+        <v>656</v>
       </c>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
@@ -1098,7 +1054,7 @@
         <v>76</v>
       </c>
       <c r="Z5" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U5:X5)</f>
         <v>0</v>
       </c>
       <c r="AA5" s="3"/>
@@ -1109,7 +1065,7 @@
         <v>76</v>
       </c>
       <c r="AF5" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA5:AD5)</f>
         <v>0</v>
       </c>
       <c r="AG5" s="3"/>
@@ -1120,16 +1076,16 @@
         <v>76</v>
       </c>
       <c r="AL5" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG5:AJ5)</f>
         <v>0</v>
       </c>
       <c r="AM5" s="6" cm="1">
         <f t="array" ref="AM5">SUM(C5:F5+I5:L5+O5:R5+U5:X5+AA5:AD5+AG5:AJ5)</f>
-        <v>1528</v>
+        <v>2184</v>
       </c>
       <c r="AN5" s="8">
-        <f t="shared" si="6"/>
-        <v>1604</v>
+        <f>SUM(H5+N5+T5+Z5+AF5+AL5)</f>
+        <v>2260</v>
       </c>
       <c r="AO5">
         <v>200</v>
@@ -1138,75 +1094,83 @@
         <v>173.04</v>
       </c>
       <c r="AQ5" s="11">
-        <f t="shared" si="7"/>
+        <f>SUM((AO5-AP5)*0.7)</f>
         <v>18.872000000000003</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C6" s="3">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="D6" s="3">
-        <v>176</v>
+        <v>205</v>
       </c>
       <c r="E6" s="3">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="F6" s="3">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="G6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="H6" s="4">
-        <f t="shared" si="0"/>
-        <v>801</v>
+        <f>SUM(C6:G6)</f>
+        <v>825</v>
       </c>
       <c r="I6" s="3">
+        <v>174</v>
+      </c>
+      <c r="J6" s="3">
         <v>200</v>
       </c>
-      <c r="J6" s="3">
-        <v>191</v>
-      </c>
       <c r="K6" s="3">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="L6" s="3">
-        <v>204</v>
+        <v>147</v>
       </c>
       <c r="M6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="N6" s="4">
-        <f t="shared" si="1"/>
-        <v>789</v>
-      </c>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
+        <f>SUM(I6:L6)</f>
+        <v>710</v>
+      </c>
+      <c r="O6" s="3">
+        <v>185</v>
+      </c>
+      <c r="P6" s="3">
+        <v>149</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>167</v>
+      </c>
+      <c r="R6" s="3">
+        <v>213</v>
+      </c>
       <c r="S6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="T6" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>SUM(O6:R6)</f>
+        <v>714</v>
       </c>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="Z6" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U6:X6)</f>
         <v>0</v>
       </c>
       <c r="AA6" s="3"/>
@@ -1214,10 +1178,10 @@
       <c r="AC6" s="3"/>
       <c r="AD6" s="3"/>
       <c r="AE6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="AF6" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA6:AD6)</f>
         <v>0</v>
       </c>
       <c r="AG6" s="3"/>
@@ -1225,96 +1189,104 @@
       <c r="AI6" s="3"/>
       <c r="AJ6" s="3"/>
       <c r="AK6" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="AL6" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG6:AJ6)</f>
         <v>0</v>
       </c>
       <c r="AM6" s="6" cm="1">
         <f t="array" ref="AM6">SUM(C6:F6+I6:L6+O6:R6+U6:X6+AA6:AD6+AG6:AJ6)</f>
-        <v>1494</v>
+        <v>2205</v>
       </c>
       <c r="AN6" s="8">
-        <f t="shared" si="6"/>
-        <v>1590</v>
+        <f>SUM(H6+N6+T6+Z6+AF6+AL6)</f>
+        <v>2249</v>
       </c>
       <c r="AO6">
         <v>200</v>
       </c>
       <c r="AP6" s="11">
-        <v>166.35</v>
+        <v>184.5</v>
       </c>
       <c r="AQ6" s="11">
-        <f t="shared" si="7"/>
-        <v>23.555000000000003</v>
+        <f>SUM((AO6-AP6)*0.7)</f>
+        <v>10.85</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C7" s="3">
+        <v>157</v>
+      </c>
+      <c r="D7" s="3">
+        <v>176</v>
+      </c>
+      <c r="E7" s="3">
+        <v>180</v>
+      </c>
+      <c r="F7" s="3">
+        <v>192</v>
+      </c>
+      <c r="G7" s="9">
+        <v>96</v>
+      </c>
+      <c r="H7" s="4">
+        <f>SUM(C7:G7)</f>
+        <v>801</v>
+      </c>
+      <c r="I7" s="3">
         <v>200</v>
       </c>
-      <c r="D7" s="3">
-        <v>205</v>
-      </c>
-      <c r="E7" s="3">
-        <v>192</v>
-      </c>
-      <c r="F7" s="3">
-        <v>184</v>
-      </c>
-      <c r="G7" s="9">
-        <v>44</v>
-      </c>
-      <c r="H7" s="4">
-        <f t="shared" si="0"/>
-        <v>825</v>
-      </c>
-      <c r="I7" s="3">
-        <v>174</v>
-      </c>
       <c r="J7" s="3">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="K7" s="3">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="L7" s="3">
-        <v>147</v>
+        <v>204</v>
       </c>
       <c r="M7" s="9">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="N7" s="4">
-        <f t="shared" si="1"/>
-        <v>710</v>
-      </c>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
+        <f>SUM(I7:L7)</f>
+        <v>789</v>
+      </c>
+      <c r="O7" s="3">
+        <v>131</v>
+      </c>
+      <c r="P7" s="3">
+        <v>142</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>152</v>
+      </c>
+      <c r="R7" s="3">
+        <v>163</v>
+      </c>
       <c r="S7" s="9">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="T7" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f>SUM(O7:R7)</f>
+        <v>588</v>
       </c>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
       <c r="Y7" s="9">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="Z7" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U7:X7)</f>
         <v>0</v>
       </c>
       <c r="AA7" s="3"/>
@@ -1322,10 +1294,10 @@
       <c r="AC7" s="3"/>
       <c r="AD7" s="3"/>
       <c r="AE7" s="9">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="AF7" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA7:AD7)</f>
         <v>0</v>
       </c>
       <c r="AG7" s="3"/>
@@ -1333,134 +1305,142 @@
       <c r="AI7" s="3"/>
       <c r="AJ7" s="3"/>
       <c r="AK7" s="9">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="AL7" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG7:AJ7)</f>
         <v>0</v>
       </c>
       <c r="AM7" s="6" cm="1">
         <f t="array" ref="AM7">SUM(C7:F7+I7:L7+O7:R7+U7:X7+AA7:AD7+AG7:AJ7)</f>
-        <v>1491</v>
+        <v>2082</v>
       </c>
       <c r="AN7" s="8">
-        <f t="shared" si="6"/>
-        <v>1535</v>
+        <f>SUM(H7+N7+T7+Z7+AF7+AL7)</f>
+        <v>2178</v>
       </c>
       <c r="AO7">
         <v>200</v>
       </c>
       <c r="AP7" s="11">
-        <v>184.5</v>
+        <v>166.35</v>
       </c>
       <c r="AQ7" s="11">
-        <f t="shared" si="7"/>
-        <v>10.85</v>
+        <f>SUM((AO7-AP7)*0.7)</f>
+        <v>23.555000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="2">
-        <v>246</v>
-      </c>
-      <c r="D8" s="2">
-        <v>192</v>
-      </c>
-      <c r="E8" s="2">
-        <v>176</v>
-      </c>
-      <c r="F8" s="2">
-        <v>199</v>
+        <v>2</v>
+      </c>
+      <c r="C8" s="3">
+        <v>190</v>
+      </c>
+      <c r="D8" s="3">
+        <v>193</v>
+      </c>
+      <c r="E8" s="3">
+        <v>205</v>
+      </c>
+      <c r="F8" s="3">
+        <v>207</v>
       </c>
       <c r="G8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="H8" s="4">
-        <f t="shared" si="0"/>
-        <v>857</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+        <f>SUM(C8:G8)</f>
+        <v>815</v>
+      </c>
+      <c r="I8" s="3">
+        <v>225</v>
+      </c>
+      <c r="J8" s="3">
+        <v>242</v>
+      </c>
+      <c r="K8" s="3">
+        <v>224</v>
+      </c>
+      <c r="L8" s="3">
+        <v>189</v>
+      </c>
       <c r="M8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="N8" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
+        <f>SUM(I8:L8)</f>
+        <v>880</v>
+      </c>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
       <c r="S8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="T8" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
+        <f>SUM(O8:R8)</f>
+        <v>0</v>
+      </c>
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
       <c r="Y8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="Z8" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
-      <c r="AC8" s="2"/>
-      <c r="AD8" s="2"/>
+        <f>SUM(U8:X8)</f>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
       <c r="AE8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AF8" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG8" s="2"/>
-      <c r="AH8" s="2"/>
-      <c r="AI8" s="2"/>
-      <c r="AJ8" s="2"/>
+        <f>SUM(AA8:AD8)</f>
+        <v>0</v>
+      </c>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+      <c r="AJ8" s="3"/>
       <c r="AK8" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AL8" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG8:AJ8)</f>
         <v>0</v>
       </c>
       <c r="AM8" s="6" cm="1">
         <f t="array" ref="AM8">SUM(C8:F8+I8:L8+O8:R8+U8:X8+AA8:AD8+AG8:AJ8)</f>
-        <v>813</v>
+        <v>1675</v>
       </c>
       <c r="AN8" s="8">
-        <f t="shared" si="6"/>
-        <v>857</v>
+        <f>SUM(H8+N8+T8+Z8+AF8+AL8)</f>
+        <v>1695</v>
       </c>
       <c r="AO8">
         <v>200</v>
       </c>
       <c r="AP8" s="11">
-        <v>185</v>
+        <v>193.33</v>
       </c>
       <c r="AQ8" s="11">
-        <f t="shared" si="7"/>
-        <v>10.5</v>
+        <f>SUM((AO8-AP8)*0.7)</f>
+        <v>4.6689999999999907</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>26</v>
@@ -1481,19 +1461,27 @@
         <v>40</v>
       </c>
       <c r="H9" s="4">
-        <f t="shared" si="0"/>
+        <f>SUM(C9:G9)</f>
         <v>840</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
+      <c r="I9" s="2">
+        <v>213</v>
+      </c>
+      <c r="J9" s="2">
+        <v>242</v>
+      </c>
+      <c r="K9" s="2">
+        <v>177</v>
+      </c>
+      <c r="L9" s="2">
+        <v>185</v>
+      </c>
       <c r="M9" s="9">
         <v>40</v>
       </c>
       <c r="N9" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM(I9:L9)</f>
+        <v>817</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
@@ -1503,7 +1491,7 @@
         <v>40</v>
       </c>
       <c r="T9" s="4">
-        <f t="shared" si="2"/>
+        <f>SUM(O9:R9)</f>
         <v>0</v>
       </c>
       <c r="U9" s="2"/>
@@ -1514,7 +1502,7 @@
         <v>40</v>
       </c>
       <c r="Z9" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U9:X9)</f>
         <v>0</v>
       </c>
       <c r="AA9" s="2"/>
@@ -1525,7 +1513,7 @@
         <v>40</v>
       </c>
       <c r="AF9" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA9:AD9)</f>
         <v>0</v>
       </c>
       <c r="AG9" s="2"/>
@@ -1536,16 +1524,16 @@
         <v>40</v>
       </c>
       <c r="AL9" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG9:AJ9)</f>
         <v>0</v>
       </c>
       <c r="AM9" s="6" cm="1">
         <f t="array" ref="AM9">SUM(C9:F9+I9:L9+O9:R9+U9:X9+AA9:AD9+AG9:AJ9)</f>
-        <v>800</v>
+        <v>1617</v>
       </c>
       <c r="AN9" s="8">
-        <f t="shared" si="6"/>
-        <v>840</v>
+        <f>SUM(H9+N9+T9+Z9+AF9+AL9)</f>
+        <v>1657</v>
       </c>
       <c r="AO9">
         <v>200</v>
@@ -1554,156 +1542,172 @@
         <v>185.77</v>
       </c>
       <c r="AQ9" s="11">
-        <f t="shared" si="7"/>
+        <f>SUM((AO9-AP9)*0.7)</f>
         <v>9.9609999999999914</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="3">
-        <v>183</v>
-      </c>
-      <c r="D10" s="3">
-        <v>174</v>
-      </c>
-      <c r="E10" s="3">
-        <v>207</v>
-      </c>
-      <c r="F10" s="3">
-        <v>216</v>
+        <v>29</v>
+      </c>
+      <c r="C10" s="2">
+        <v>246</v>
+      </c>
+      <c r="D10" s="2">
+        <v>192</v>
+      </c>
+      <c r="E10" s="2">
+        <v>176</v>
+      </c>
+      <c r="F10" s="2">
+        <v>199</v>
       </c>
       <c r="G10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" si="0"/>
-        <v>800</v>
-      </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+        <f>SUM(C10:G10)</f>
+        <v>857</v>
+      </c>
+      <c r="I10" s="2">
+        <v>177</v>
+      </c>
+      <c r="J10" s="2">
+        <v>146</v>
+      </c>
+      <c r="K10" s="2">
+        <v>224</v>
+      </c>
+      <c r="L10" s="2">
+        <v>178</v>
+      </c>
       <c r="M10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="N10" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
+        <f>SUM(I10:L10)</f>
+        <v>725</v>
+      </c>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
       <c r="S10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="T10" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
+        <f>SUM(O10:R10)</f>
+        <v>0</v>
+      </c>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
       <c r="Y10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="Z10" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA10" s="3"/>
-      <c r="AB10" s="3"/>
-      <c r="AC10" s="3"/>
-      <c r="AD10" s="3"/>
+        <f>SUM(U10:X10)</f>
+        <v>0</v>
+      </c>
+      <c r="AA10" s="2"/>
+      <c r="AB10" s="2"/>
+      <c r="AC10" s="2"/>
+      <c r="AD10" s="2"/>
       <c r="AE10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="AF10" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG10" s="3"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
+        <f>SUM(AA10:AD10)</f>
+        <v>0</v>
+      </c>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="2"/>
+      <c r="AI10" s="2"/>
+      <c r="AJ10" s="2"/>
       <c r="AK10" s="9">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="AL10" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG10:AJ10)</f>
         <v>0</v>
       </c>
       <c r="AM10" s="6" cm="1">
         <f t="array" ref="AM10">SUM(C10:F10+I10:L10+O10:R10+U10:X10+AA10:AD10+AG10:AJ10)</f>
-        <v>780</v>
+        <v>1538</v>
       </c>
       <c r="AN10" s="8">
-        <f t="shared" si="6"/>
-        <v>800</v>
+        <f>SUM(H10+N10+T10+Z10+AF10+AL10)</f>
+        <v>1582</v>
       </c>
       <c r="AO10">
         <v>200</v>
       </c>
       <c r="AP10" s="11">
-        <v>192.5</v>
+        <v>185</v>
       </c>
       <c r="AQ10" s="11">
-        <f t="shared" si="7"/>
-        <v>5.25</v>
+        <f>SUM((AO10-AP10)*0.7)</f>
+        <v>10.5</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C11" s="3">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="D11" s="3">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="E11" s="3">
-        <v>140</v>
+        <v>207</v>
       </c>
       <c r="F11" s="3">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="G11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="H11" s="4">
-        <f t="shared" si="0"/>
-        <v>780</v>
-      </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
+        <f>SUM(C11:G11)</f>
+        <v>800</v>
+      </c>
+      <c r="I11" s="3">
+        <v>174</v>
+      </c>
+      <c r="J11" s="3">
+        <v>190</v>
+      </c>
+      <c r="K11" s="3">
+        <v>146</v>
+      </c>
+      <c r="L11" s="3">
+        <v>136</v>
+      </c>
       <c r="M11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="N11" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM(I11:L11)</f>
+        <v>646</v>
       </c>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="S11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="T11" s="4">
-        <f t="shared" si="2"/>
+        <f>SUM(O11:R11)</f>
         <v>0</v>
       </c>
       <c r="U11" s="3"/>
@@ -1711,10 +1715,10 @@
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
       <c r="Y11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="Z11" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U11:X11)</f>
         <v>0</v>
       </c>
       <c r="AA11" s="3"/>
@@ -1722,10 +1726,10 @@
       <c r="AC11" s="3"/>
       <c r="AD11" s="3"/>
       <c r="AE11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="AF11" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA11:AD11)</f>
         <v>0</v>
       </c>
       <c r="AG11" s="3"/>
@@ -1733,277 +1737,301 @@
       <c r="AI11" s="3"/>
       <c r="AJ11" s="3"/>
       <c r="AK11" s="9">
-        <v>132</v>
+        <v>20</v>
       </c>
       <c r="AL11" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG11:AJ11)</f>
         <v>0</v>
       </c>
       <c r="AM11" s="6" cm="1">
         <f t="array" ref="AM11">SUM(C11:F11+I11:L11+O11:R11+U11:X11+AA11:AD11+AG11:AJ11)</f>
-        <v>648</v>
+        <v>1426</v>
       </c>
       <c r="AN11" s="8">
-        <f t="shared" si="6"/>
-        <v>780</v>
+        <f>SUM(H11+N11+T11+Z11+AF11+AL11)</f>
+        <v>1446</v>
       </c>
       <c r="AO11">
         <v>200</v>
       </c>
       <c r="AP11" s="11">
-        <v>153</v>
+        <v>192.5</v>
       </c>
       <c r="AQ11" s="11">
-        <f t="shared" si="7"/>
-        <v>32.9</v>
+        <f>SUM((AO11-AP11)*0.7)</f>
+        <v>5.25</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="3">
-        <v>179</v>
-      </c>
-      <c r="D12" s="3">
-        <v>183</v>
-      </c>
-      <c r="E12" s="3">
-        <v>144</v>
-      </c>
-      <c r="F12" s="3">
-        <v>164</v>
+        <v>24</v>
+      </c>
+      <c r="C12" s="2">
+        <v>172</v>
+      </c>
+      <c r="D12" s="2">
+        <v>174</v>
+      </c>
+      <c r="E12" s="2">
+        <v>154</v>
+      </c>
+      <c r="F12" s="2">
+        <v>162</v>
       </c>
       <c r="G12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="H12" s="4">
-        <f t="shared" si="0"/>
-        <v>762</v>
-      </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
+        <f>SUM(C12:G12)</f>
+        <v>746</v>
+      </c>
+      <c r="I12" s="2">
+        <v>178</v>
+      </c>
+      <c r="J12" s="2">
+        <v>178</v>
+      </c>
+      <c r="K12" s="2">
+        <v>132</v>
+      </c>
+      <c r="L12" s="2">
+        <v>169</v>
+      </c>
       <c r="M12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="N12" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
+        <f>SUM(I12:L12)</f>
+        <v>657</v>
+      </c>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
       <c r="S12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="T12" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
+        <f>SUM(O12:R12)</f>
+        <v>0</v>
+      </c>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
       <c r="Y12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="Z12" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA12" s="3"/>
-      <c r="AB12" s="3"/>
-      <c r="AC12" s="3"/>
-      <c r="AD12" s="3"/>
+        <f>SUM(U12:X12)</f>
+        <v>0</v>
+      </c>
+      <c r="AA12" s="2"/>
+      <c r="AB12" s="2"/>
+      <c r="AC12" s="2"/>
+      <c r="AD12" s="2"/>
       <c r="AE12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="AF12" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG12" s="3"/>
-      <c r="AH12" s="3"/>
-      <c r="AI12" s="3"/>
-      <c r="AJ12" s="3"/>
+        <f>SUM(AA12:AD12)</f>
+        <v>0</v>
+      </c>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="2"/>
+      <c r="AI12" s="2"/>
+      <c r="AJ12" s="2"/>
       <c r="AK12" s="9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="AL12" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG12:AJ12)</f>
         <v>0</v>
       </c>
       <c r="AM12" s="6" cm="1">
         <f t="array" ref="AM12">SUM(C12:F12+I12:L12+O12:R12+U12:X12+AA12:AD12+AG12:AJ12)</f>
-        <v>670</v>
+        <v>1319</v>
       </c>
       <c r="AN12" s="8">
-        <f t="shared" si="6"/>
-        <v>762</v>
+        <f>SUM(H12+N12+T12+Z12+AF12+AL12)</f>
+        <v>1403</v>
       </c>
       <c r="AO12">
         <v>200</v>
       </c>
       <c r="AP12" s="11">
-        <v>167</v>
+        <v>169.44</v>
       </c>
       <c r="AQ12" s="11">
-        <f t="shared" si="7"/>
-        <v>23.099999999999998</v>
+        <f>SUM((AO12-AP12)*0.7)</f>
+        <v>21.391999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="2">
-        <v>172</v>
-      </c>
-      <c r="D13" s="2">
-        <v>174</v>
-      </c>
-      <c r="E13" s="2">
-        <v>154</v>
-      </c>
-      <c r="F13" s="2">
+        <v>13</v>
+      </c>
+      <c r="C13" s="3">
+        <v>152</v>
+      </c>
+      <c r="D13" s="3">
+        <v>160</v>
+      </c>
+      <c r="E13" s="3">
+        <v>198</v>
+      </c>
+      <c r="F13" s="3">
+        <v>136</v>
+      </c>
+      <c r="G13" s="9">
+        <v>68</v>
+      </c>
+      <c r="H13" s="4">
+        <f>SUM(C13:G13)</f>
+        <v>714</v>
+      </c>
+      <c r="I13" s="3">
+        <v>163</v>
+      </c>
+      <c r="J13" s="3">
+        <v>171</v>
+      </c>
+      <c r="K13" s="3">
+        <v>189</v>
+      </c>
+      <c r="L13" s="3">
         <v>162</v>
       </c>
-      <c r="G13" s="9">
-        <v>84</v>
-      </c>
-      <c r="H13" s="4">
-        <f t="shared" si="0"/>
-        <v>746</v>
-      </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
       <c r="M13" s="9">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="N13" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
+        <f>SUM(I13:L13)</f>
+        <v>685</v>
+      </c>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
       <c r="S13" s="9">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="T13" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
+        <f>SUM(O13:R13)</f>
+        <v>0</v>
+      </c>
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
       <c r="Y13" s="9">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="Z13" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA13" s="2"/>
-      <c r="AB13" s="2"/>
-      <c r="AC13" s="2"/>
-      <c r="AD13" s="2"/>
+        <f>SUM(U13:X13)</f>
+        <v>0</v>
+      </c>
+      <c r="AA13" s="3"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+      <c r="AD13" s="3"/>
       <c r="AE13" s="9">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="AF13" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG13" s="2"/>
-      <c r="AH13" s="2"/>
-      <c r="AI13" s="2"/>
-      <c r="AJ13" s="2"/>
+        <f>SUM(AA13:AD13)</f>
+        <v>0</v>
+      </c>
+      <c r="AG13" s="3"/>
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="3"/>
+      <c r="AJ13" s="3"/>
       <c r="AK13" s="9">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="AL13" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG13:AJ13)</f>
         <v>0</v>
       </c>
       <c r="AM13" s="6" cm="1">
         <f t="array" ref="AM13">SUM(C13:F13+I13:L13+O13:R13+U13:X13+AA13:AD13+AG13:AJ13)</f>
-        <v>662</v>
+        <v>1331</v>
       </c>
       <c r="AN13" s="8">
-        <f t="shared" si="6"/>
-        <v>746</v>
+        <f>SUM(H13+N13+T13+Z13+AF13+AL13)</f>
+        <v>1399</v>
       </c>
       <c r="AO13">
         <v>200</v>
       </c>
       <c r="AP13" s="11">
-        <v>169.44</v>
+        <v>175.62</v>
       </c>
       <c r="AQ13" s="11">
-        <f t="shared" si="7"/>
-        <v>21.391999999999999</v>
+        <f>SUM((AO13-AP13)*0.7)</f>
+        <v>17.065999999999995</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C14" s="3">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D14" s="3">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E14" s="3">
-        <v>198</v>
+        <v>140</v>
       </c>
       <c r="F14" s="3">
-        <v>136</v>
+        <v>195</v>
       </c>
       <c r="G14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="H14" s="4">
-        <f t="shared" si="0"/>
-        <v>714</v>
-      </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
+        <f>SUM(C14:G14)</f>
+        <v>780</v>
+      </c>
+      <c r="I14" s="3">
+        <v>145</v>
+      </c>
+      <c r="J14" s="3">
+        <v>100</v>
+      </c>
+      <c r="K14" s="3">
+        <v>150</v>
+      </c>
+      <c r="L14" s="3">
+        <v>191</v>
+      </c>
       <c r="M14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="N14" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>SUM(I14:L14)</f>
+        <v>586</v>
       </c>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
       <c r="S14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="T14" s="4">
-        <f t="shared" si="2"/>
+        <f>SUM(O14:R14)</f>
         <v>0</v>
       </c>
       <c r="U14" s="3"/>
@@ -2011,10 +2039,10 @@
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="Z14" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U14:X14)</f>
         <v>0</v>
       </c>
       <c r="AA14" s="3"/>
@@ -2022,10 +2050,10 @@
       <c r="AC14" s="3"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="AF14" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA14:AD14)</f>
         <v>0</v>
       </c>
       <c r="AG14" s="3"/>
@@ -2033,66 +2061,66 @@
       <c r="AI14" s="3"/>
       <c r="AJ14" s="3"/>
       <c r="AK14" s="9">
-        <v>68</v>
+        <v>132</v>
       </c>
       <c r="AL14" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG14:AJ14)</f>
         <v>0</v>
       </c>
       <c r="AM14" s="6" cm="1">
         <f t="array" ref="AM14">SUM(C14:F14+I14:L14+O14:R14+U14:X14+AA14:AD14+AG14:AJ14)</f>
-        <v>646</v>
+        <v>1234</v>
       </c>
       <c r="AN14" s="8">
-        <f t="shared" si="6"/>
-        <v>714</v>
+        <f>SUM(H14+N14+T14+Z14+AF14+AL14)</f>
+        <v>1366</v>
       </c>
       <c r="AO14">
         <v>200</v>
       </c>
       <c r="AP14" s="11">
-        <v>175.62</v>
+        <v>153</v>
       </c>
       <c r="AQ14" s="11">
-        <f t="shared" si="7"/>
-        <v>17.065999999999995</v>
+        <f>SUM((AO14-AP14)*0.7)</f>
+        <v>32.9</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C15" s="3">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="D15" s="3">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="E15" s="3">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="F15" s="3">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="H15" s="4">
-        <f t="shared" si="0"/>
-        <v>712</v>
+        <f>SUM(C15:G15)</f>
+        <v>762</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="N15" s="4">
-        <f t="shared" si="1"/>
+        <f>SUM(I15:L15)</f>
         <v>0</v>
       </c>
       <c r="O15" s="3"/>
@@ -2100,10 +2128,10 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
       <c r="S15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="T15" s="4">
-        <f t="shared" si="2"/>
+        <f>SUM(O15:R15)</f>
         <v>0</v>
       </c>
       <c r="U15" s="3"/>
@@ -2111,10 +2139,10 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
       <c r="Y15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="Z15" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U15:X15)</f>
         <v>0</v>
       </c>
       <c r="AA15" s="3"/>
@@ -2122,10 +2150,10 @@
       <c r="AC15" s="3"/>
       <c r="AD15" s="3"/>
       <c r="AE15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="AF15" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA15:AD15)</f>
         <v>0</v>
       </c>
       <c r="AG15" s="3"/>
@@ -2133,250 +2161,266 @@
       <c r="AI15" s="3"/>
       <c r="AJ15" s="3"/>
       <c r="AK15" s="9">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="AL15" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG15:AJ15)</f>
         <v>0</v>
       </c>
       <c r="AM15" s="6" cm="1">
         <f t="array" ref="AM15">SUM(C15:F15+I15:L15+O15:R15+U15:X15+AA15:AD15+AG15:AJ15)</f>
-        <v>604</v>
+        <v>670</v>
       </c>
       <c r="AN15" s="8">
-        <f t="shared" si="6"/>
-        <v>712</v>
+        <f>SUM(H15+N15+T15+Z15+AF15+AL15)</f>
+        <v>762</v>
       </c>
       <c r="AO15">
         <v>200</v>
       </c>
       <c r="AP15" s="11">
-        <v>161.46</v>
+        <v>167</v>
       </c>
       <c r="AQ15" s="11">
-        <f t="shared" si="7"/>
-        <v>26.977999999999994</v>
+        <f>SUM((AO15-AP15)*0.7)</f>
+        <v>23.099999999999998</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="2">
-        <v>151</v>
-      </c>
-      <c r="D16" s="2">
-        <v>182</v>
-      </c>
-      <c r="E16" s="2">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3">
         <v>177</v>
       </c>
-      <c r="F16" s="2">
-        <v>147</v>
+      <c r="D16" s="3">
+        <v>199</v>
+      </c>
+      <c r="E16" s="3">
+        <v>134</v>
+      </c>
+      <c r="F16" s="3">
+        <v>211</v>
       </c>
       <c r="G16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="H16" s="4">
-        <f t="shared" si="0"/>
-        <v>693</v>
-      </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
+        <f>SUM(C16:G16)</f>
+        <v>737</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
       <c r="M16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="N16" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
+        <f>SUM(I16:L16)</f>
+        <v>0</v>
+      </c>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
       <c r="S16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="T16" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
+        <f>SUM(O16:R16)</f>
+        <v>0</v>
+      </c>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
       <c r="Y16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="Z16" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA16" s="2"/>
-      <c r="AB16" s="2"/>
-      <c r="AC16" s="2"/>
-      <c r="AD16" s="2"/>
+        <f>SUM(U16:X16)</f>
+        <v>0</v>
+      </c>
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="3"/>
+      <c r="AC16" s="3"/>
+      <c r="AD16" s="3"/>
       <c r="AE16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="AF16" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG16" s="2"/>
-      <c r="AH16" s="2"/>
-      <c r="AI16" s="2"/>
-      <c r="AJ16" s="2"/>
+        <f>SUM(AA16:AD16)</f>
+        <v>0</v>
+      </c>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3"/>
       <c r="AK16" s="9">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="AL16" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG16:AJ16)</f>
         <v>0</v>
       </c>
       <c r="AM16" s="6" cm="1">
         <f t="array" ref="AM16">SUM(C16:F16+I16:L16+O16:R16+U16:X16+AA16:AD16+AG16:AJ16)</f>
-        <v>657</v>
+        <v>721</v>
       </c>
       <c r="AN16" s="8">
-        <f t="shared" si="6"/>
-        <v>693</v>
+        <f>SUM(H16+N16+T16+Z16+AF16+AL16)</f>
+        <v>737</v>
       </c>
       <c r="AO16">
         <v>200</v>
       </c>
       <c r="AP16" s="11">
-        <v>187.47</v>
+        <v>194.7</v>
       </c>
       <c r="AQ16" s="11">
-        <f t="shared" si="7"/>
-        <v>8.7710000000000008</v>
+        <f>SUM((AO16-AP16)*0.7)</f>
+        <v>3.7100000000000075</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="C17" s="3">
+        <v>149</v>
+      </c>
+      <c r="D17" s="3">
+        <v>166</v>
+      </c>
+      <c r="E17" s="3">
+        <v>126</v>
+      </c>
+      <c r="F17" s="3">
+        <v>163</v>
+      </c>
       <c r="G17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="H17" s="4">
-        <f t="shared" si="0"/>
-        <v>84</v>
-      </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
+        <f>SUM(C17:G17)</f>
+        <v>712</v>
+      </c>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
       <c r="M17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="N17" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
+        <f>SUM(I17:L17)</f>
+        <v>0</v>
+      </c>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="3"/>
       <c r="S17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="T17" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
+        <f>SUM(O17:R17)</f>
+        <v>0</v>
+      </c>
+      <c r="U17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
       <c r="Y17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="Z17" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA17" s="2"/>
-      <c r="AB17" s="2"/>
-      <c r="AC17" s="2"/>
-      <c r="AD17" s="2"/>
+        <f>SUM(U17:X17)</f>
+        <v>0</v>
+      </c>
+      <c r="AA17" s="3"/>
+      <c r="AB17" s="3"/>
+      <c r="AC17" s="3"/>
+      <c r="AD17" s="3"/>
       <c r="AE17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="AF17" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG17" s="2"/>
-      <c r="AH17" s="2"/>
-      <c r="AI17" s="2"/>
-      <c r="AJ17" s="2"/>
+        <f>SUM(AA17:AD17)</f>
+        <v>0</v>
+      </c>
+      <c r="AG17" s="3"/>
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="3"/>
+      <c r="AJ17" s="3"/>
       <c r="AK17" s="9">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="AL17" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG17:AJ17)</f>
         <v>0</v>
       </c>
       <c r="AM17" s="6" cm="1">
         <f t="array" ref="AM17">SUM(C17:F17+I17:L17+O17:R17+U17:X17+AA17:AD17+AG17:AJ17)</f>
-        <v>0</v>
+        <v>604</v>
       </c>
       <c r="AN17" s="8">
-        <f t="shared" si="6"/>
-        <v>84</v>
+        <f>SUM(H17+N17+T17+Z17+AF17+AL17)</f>
+        <v>712</v>
       </c>
       <c r="AO17">
         <v>200</v>
       </c>
       <c r="AP17" s="11">
-        <v>169.88</v>
+        <v>161.46</v>
       </c>
       <c r="AQ17" s="11">
-        <f t="shared" si="7"/>
-        <v>21.084000000000003</v>
+        <f>SUM((AO17-AP17)*0.7)</f>
+        <v>26.977999999999994</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+        <v>33</v>
+      </c>
+      <c r="C18" s="2">
+        <v>148</v>
+      </c>
+      <c r="D18" s="2">
+        <v>134</v>
+      </c>
+      <c r="E18" s="2">
+        <v>164</v>
+      </c>
+      <c r="F18" s="2">
+        <v>178</v>
+      </c>
       <c r="G18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H18" s="4">
-        <f t="shared" si="0"/>
-        <v>68</v>
+        <f>SUM(C18:G18)</f>
+        <v>700</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="N18" s="4">
-        <f t="shared" si="1"/>
+        <f>SUM(I18:L18)</f>
         <v>0</v>
       </c>
       <c r="O18" s="2"/>
@@ -2384,10 +2428,10 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
       <c r="S18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T18" s="4">
-        <f t="shared" si="2"/>
+        <f>SUM(O18:R18)</f>
         <v>0</v>
       </c>
       <c r="U18" s="2"/>
@@ -2395,10 +2439,10 @@
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="Z18" s="4">
-        <f t="shared" si="3"/>
+        <f>SUM(U18:X18)</f>
         <v>0</v>
       </c>
       <c r="AA18" s="2"/>
@@ -2406,10 +2450,10 @@
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
       <c r="AE18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="AF18" s="4">
-        <f t="shared" si="4"/>
+        <f>SUM(AA18:AD18)</f>
         <v>0</v>
       </c>
       <c r="AG18" s="2"/>
@@ -2417,194 +2461,202 @@
       <c r="AI18" s="2"/>
       <c r="AJ18" s="2"/>
       <c r="AK18" s="9">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="AL18" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG18:AJ18)</f>
         <v>0</v>
       </c>
       <c r="AM18" s="6" cm="1">
         <f t="array" ref="AM18">SUM(C18:F18+I18:L18+O18:R18+U18:X18+AA18:AD18+AG18:AJ18)</f>
-        <v>0</v>
+        <v>624</v>
       </c>
       <c r="AN18" s="8">
-        <f t="shared" si="6"/>
-        <v>68</v>
+        <f>SUM(H18+N18+T18+Z18+AF18+AL18)</f>
+        <v>700</v>
       </c>
       <c r="AO18">
         <v>200</v>
       </c>
       <c r="AP18" s="11">
-        <v>175.36</v>
+        <v>173.14</v>
       </c>
       <c r="AQ18" s="11">
-        <f t="shared" si="7"/>
-        <v>17.24799999999999</v>
+        <f>SUM((AO18-AP18)*0.7)</f>
+        <v>18.802000000000007</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="C19" s="2">
+        <v>151</v>
+      </c>
+      <c r="D19" s="2">
+        <v>182</v>
+      </c>
+      <c r="E19" s="2">
+        <v>177</v>
+      </c>
+      <c r="F19" s="2">
+        <v>147</v>
+      </c>
       <c r="G19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H19" s="4">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
+        <f>SUM(C19:G19)</f>
+        <v>693</v>
+      </c>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
       <c r="M19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="N19" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
+        <f>SUM(I19:L19)</f>
+        <v>0</v>
+      </c>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
       <c r="S19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="T19" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
+        <f>SUM(O19:R19)</f>
+        <v>0</v>
+      </c>
+      <c r="U19" s="2"/>
+      <c r="V19" s="2"/>
+      <c r="W19" s="2"/>
+      <c r="X19" s="2"/>
       <c r="Y19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="Z19" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA19" s="3"/>
-      <c r="AB19" s="3"/>
-      <c r="AC19" s="3"/>
-      <c r="AD19" s="3"/>
+        <f>SUM(U19:X19)</f>
+        <v>0</v>
+      </c>
+      <c r="AA19" s="2"/>
+      <c r="AB19" s="2"/>
+      <c r="AC19" s="2"/>
+      <c r="AD19" s="2"/>
       <c r="AE19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="AF19" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG19" s="3"/>
-      <c r="AH19" s="3"/>
-      <c r="AI19" s="3"/>
-      <c r="AJ19" s="3"/>
+        <f>SUM(AA19:AD19)</f>
+        <v>0</v>
+      </c>
+      <c r="AG19" s="2"/>
+      <c r="AH19" s="2"/>
+      <c r="AI19" s="2"/>
+      <c r="AJ19" s="2"/>
       <c r="AK19" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="AL19" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG19:AJ19)</f>
         <v>0</v>
       </c>
       <c r="AM19" s="6" cm="1">
         <f t="array" ref="AM19">SUM(C19:F19+I19:L19+O19:R19+U19:X19+AA19:AD19+AG19:AJ19)</f>
-        <v>0</v>
+        <v>657</v>
       </c>
       <c r="AN19" s="8">
-        <f t="shared" si="6"/>
-        <v>16</v>
+        <f>SUM(H19+N19+T19+Z19+AF19+AL19)</f>
+        <v>693</v>
       </c>
       <c r="AO19">
         <v>200</v>
       </c>
       <c r="AP19" s="11">
-        <v>194.7</v>
+        <v>187.47</v>
       </c>
       <c r="AQ19" s="11">
-        <f t="shared" si="7"/>
-        <v>3.7100000000000075</v>
+        <f>SUM((AO19-AP19)*0.7)</f>
+        <v>8.7710000000000008</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+        <v>25</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
       <c r="G20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="H20" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
+        <f>SUM(C20:G20)</f>
+        <v>84</v>
+      </c>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
       <c r="M20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="N20" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
+        <f>SUM(I20:L20)</f>
+        <v>0</v>
+      </c>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
       <c r="S20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="T20" s="4">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
+        <f>SUM(O20:R20)</f>
+        <v>0</v>
+      </c>
+      <c r="U20" s="2"/>
+      <c r="V20" s="2"/>
+      <c r="W20" s="2"/>
+      <c r="X20" s="2"/>
       <c r="Y20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="Z20" s="4">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AA20" s="3"/>
-      <c r="AB20" s="3"/>
-      <c r="AC20" s="3"/>
-      <c r="AD20" s="3"/>
+        <f>SUM(U20:X20)</f>
+        <v>0</v>
+      </c>
+      <c r="AA20" s="2"/>
+      <c r="AB20" s="2"/>
+      <c r="AC20" s="2"/>
+      <c r="AD20" s="2"/>
       <c r="AE20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="AF20" s="4">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AG20" s="3"/>
-      <c r="AH20" s="3"/>
-      <c r="AI20" s="3"/>
-      <c r="AJ20" s="3"/>
+        <f>SUM(AA20:AD20)</f>
+        <v>0</v>
+      </c>
+      <c r="AG20" s="2"/>
+      <c r="AH20" s="2"/>
+      <c r="AI20" s="2"/>
+      <c r="AJ20" s="2"/>
       <c r="AK20" s="9">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="AL20" s="4">
-        <f t="shared" si="5"/>
+        <f>SUM(AG20:AJ20)</f>
         <v>0</v>
       </c>
       <c r="AM20" s="6" cm="1">
@@ -2612,74 +2664,91 @@
         <v>0</v>
       </c>
       <c r="AN20" s="8">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f>SUM(H20+N20+T20+Z20+AF20+AL20)</f>
+        <v>84</v>
       </c>
       <c r="AO20">
         <v>200</v>
       </c>
       <c r="AP20" s="11">
-        <v>202.46</v>
+        <v>169.88</v>
       </c>
       <c r="AQ20" s="11">
-        <f t="shared" si="7"/>
-        <v>-1.7220000000000055</v>
+        <f>SUM((AO20-AP20)*0.7)</f>
+        <v>21.084000000000003</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="9"/>
+      <c r="G21" s="9">
+        <v>68</v>
+      </c>
       <c r="H21" s="4">
-        <f t="shared" ref="H21:H33" si="8">SUM(C21:G21)</f>
-        <v>0</v>
+        <f>SUM(C21:G21)</f>
+        <v>68</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
-      <c r="M21" s="9"/>
+      <c r="M21" s="9">
+        <v>68</v>
+      </c>
       <c r="N21" s="4">
-        <f t="shared" ref="N21:N33" si="9">SUM(I21:L21)</f>
+        <f>SUM(I21:L21)</f>
         <v>0</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
-      <c r="S21" s="9"/>
+      <c r="S21" s="9">
+        <v>68</v>
+      </c>
       <c r="T21" s="4">
-        <f t="shared" ref="T21:T33" si="10">SUM(O21:R21)</f>
+        <f>SUM(O21:R21)</f>
         <v>0</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
       <c r="X21" s="2"/>
-      <c r="Y21" s="9"/>
+      <c r="Y21" s="9">
+        <v>68</v>
+      </c>
       <c r="Z21" s="4">
-        <f t="shared" ref="Z21:Z33" si="11">SUM(U21:X21)</f>
+        <f>SUM(U21:X21)</f>
         <v>0</v>
       </c>
       <c r="AA21" s="2"/>
       <c r="AB21" s="2"/>
       <c r="AC21" s="2"/>
       <c r="AD21" s="2"/>
-      <c r="AE21" s="9"/>
+      <c r="AE21" s="9">
+        <v>68</v>
+      </c>
       <c r="AF21" s="4">
-        <f t="shared" ref="AF21:AF33" si="12">SUM(AA21:AD21)</f>
+        <f>SUM(AA21:AD21)</f>
         <v>0</v>
       </c>
       <c r="AG21" s="2"/>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
       <c r="AJ21" s="2"/>
-      <c r="AK21" s="9"/>
+      <c r="AK21" s="9">
+        <v>68</v>
+      </c>
       <c r="AL21" s="4">
-        <f t="shared" ref="AL21:AL33" si="13">SUM(AG21:AJ21)</f>
+        <f>SUM(AG21:AJ21)</f>
         <v>0</v>
       </c>
       <c r="AM21" s="6" cm="1">
@@ -2687,72 +2756,91 @@
         <v>0</v>
       </c>
       <c r="AN21" s="8">
-        <f t="shared" ref="AN21:AN33" si="14">SUM(H21+N21+T21+Z21+AF21+AL21)</f>
-        <v>0</v>
+        <f>SUM(H21+N21+T21+Z21+AF21+AL21)</f>
+        <v>68</v>
       </c>
       <c r="AO21">
         <v>200</v>
       </c>
-      <c r="AP21" s="11"/>
+      <c r="AP21" s="11">
+        <v>175.36</v>
+      </c>
       <c r="AQ21" s="11">
-        <f t="shared" ref="AQ21:AQ33" si="15">SUM((AO21-AP21)*0.7)</f>
-        <v>140</v>
+        <f>SUM((AO21-AP21)*0.7)</f>
+        <v>17.24799999999999</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="9"/>
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="9">
+        <v>0</v>
+      </c>
       <c r="H22" s="4">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="9"/>
+        <f>SUM(C22:G22)</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="9">
+        <v>0</v>
+      </c>
       <c r="N22" s="4">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="9"/>
+        <f>SUM(I22:L22)</f>
+        <v>0</v>
+      </c>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="9">
+        <v>0</v>
+      </c>
       <c r="T22" s="4">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="U22" s="2"/>
-      <c r="V22" s="2"/>
-      <c r="W22" s="2"/>
-      <c r="X22" s="2"/>
-      <c r="Y22" s="9"/>
+        <f>SUM(O22:R22)</f>
+        <v>0</v>
+      </c>
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+      <c r="Y22" s="9">
+        <v>0</v>
+      </c>
       <c r="Z22" s="4">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="AA22" s="2"/>
-      <c r="AB22" s="2"/>
-      <c r="AC22" s="2"/>
-      <c r="AD22" s="2"/>
-      <c r="AE22" s="9"/>
+        <f>SUM(U22:X22)</f>
+        <v>0</v>
+      </c>
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3"/>
+      <c r="AC22" s="3"/>
+      <c r="AD22" s="3"/>
+      <c r="AE22" s="9">
+        <v>0</v>
+      </c>
       <c r="AF22" s="4">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="AG22" s="2"/>
-      <c r="AH22" s="2"/>
-      <c r="AI22" s="2"/>
-      <c r="AJ22" s="2"/>
-      <c r="AK22" s="9"/>
+        <f>SUM(AA22:AD22)</f>
+        <v>0</v>
+      </c>
+      <c r="AG22" s="3"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+      <c r="AJ22" s="3"/>
+      <c r="AK22" s="9">
+        <v>0</v>
+      </c>
       <c r="AL22" s="4">
-        <f t="shared" si="13"/>
+        <f>SUM(AG22:AJ22)</f>
         <v>0</v>
       </c>
       <c r="AM22" s="6" cm="1">
@@ -2760,16 +2848,18 @@
         <v>0</v>
       </c>
       <c r="AN22" s="8">
-        <f t="shared" si="14"/>
+        <f>SUM(H22+N22+T22+Z22+AF22+AL22)</f>
         <v>0</v>
       </c>
       <c r="AO22">
         <v>200</v>
       </c>
-      <c r="AP22" s="11"/>
+      <c r="AP22" s="11">
+        <v>202.46</v>
+      </c>
       <c r="AQ22" s="11">
-        <f t="shared" si="15"/>
-        <v>140</v>
+        <f>SUM((AO22-AP22)*0.7)</f>
+        <v>-1.7220000000000055</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -2780,7 +2870,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="9"/>
       <c r="H23" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="H22:H34" si="0">SUM(C23:G23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="2"/>
@@ -2789,7 +2879,7 @@
       <c r="L23" s="2"/>
       <c r="M23" s="9"/>
       <c r="N23" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="N22:N34" si="1">SUM(I23:L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="2"/>
@@ -2798,7 +2888,7 @@
       <c r="R23" s="2"/>
       <c r="S23" s="9"/>
       <c r="T23" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="T22:T34" si="2">SUM(O23:R23)</f>
         <v>0</v>
       </c>
       <c r="U23" s="2"/>
@@ -2807,7 +2897,7 @@
       <c r="X23" s="2"/>
       <c r="Y23" s="9"/>
       <c r="Z23" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="Z22:Z34" si="3">SUM(U23:X23)</f>
         <v>0</v>
       </c>
       <c r="AA23" s="2"/>
@@ -2816,7 +2906,7 @@
       <c r="AD23" s="2"/>
       <c r="AE23" s="9"/>
       <c r="AF23" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="AF22:AF34" si="4">SUM(AA23:AD23)</f>
         <v>0</v>
       </c>
       <c r="AG23" s="2"/>
@@ -2825,7 +2915,7 @@
       <c r="AJ23" s="2"/>
       <c r="AK23" s="9"/>
       <c r="AL23" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="AL22:AL34" si="5">SUM(AG23:AJ23)</f>
         <v>0</v>
       </c>
       <c r="AM23" s="6" cm="1">
@@ -2833,7 +2923,7 @@
         <v>0</v>
       </c>
       <c r="AN23" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="AN22:AN34" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
         <v>0</v>
       </c>
       <c r="AO23">
@@ -2841,7 +2931,7 @@
       </c>
       <c r="AP23" s="11"/>
       <c r="AQ23" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="AQ22:AQ34" si="7">SUM((AO23-AP23)*0.7)</f>
         <v>140</v>
       </c>
     </row>
@@ -2853,7 +2943,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="9"/>
       <c r="H24" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I24" s="2"/>
@@ -2862,7 +2952,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="9"/>
       <c r="N24" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O24" s="2"/>
@@ -2871,7 +2961,7 @@
       <c r="R24" s="2"/>
       <c r="S24" s="9"/>
       <c r="T24" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U24" s="2"/>
@@ -2880,7 +2970,7 @@
       <c r="X24" s="2"/>
       <c r="Y24" s="9"/>
       <c r="Z24" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA24" s="2"/>
@@ -2889,7 +2979,7 @@
       <c r="AD24" s="2"/>
       <c r="AE24" s="9"/>
       <c r="AF24" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG24" s="2"/>
@@ -2898,7 +2988,7 @@
       <c r="AJ24" s="2"/>
       <c r="AK24" s="9"/>
       <c r="AL24" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM24" s="6" cm="1">
@@ -2906,7 +2996,7 @@
         <v>0</v>
       </c>
       <c r="AN24" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO24">
@@ -2914,7 +3004,7 @@
       </c>
       <c r="AP24" s="11"/>
       <c r="AQ24" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -2926,7 +3016,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="9"/>
       <c r="H25" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I25" s="2"/>
@@ -2935,7 +3025,7 @@
       <c r="L25" s="2"/>
       <c r="M25" s="9"/>
       <c r="N25" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O25" s="2"/>
@@ -2944,7 +3034,7 @@
       <c r="R25" s="2"/>
       <c r="S25" s="9"/>
       <c r="T25" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U25" s="2"/>
@@ -2953,7 +3043,7 @@
       <c r="X25" s="2"/>
       <c r="Y25" s="9"/>
       <c r="Z25" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA25" s="2"/>
@@ -2962,7 +3052,7 @@
       <c r="AD25" s="2"/>
       <c r="AE25" s="9"/>
       <c r="AF25" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG25" s="2"/>
@@ -2971,7 +3061,7 @@
       <c r="AJ25" s="2"/>
       <c r="AK25" s="9"/>
       <c r="AL25" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM25" s="6" cm="1">
@@ -2979,7 +3069,7 @@
         <v>0</v>
       </c>
       <c r="AN25" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO25">
@@ -2987,7 +3077,7 @@
       </c>
       <c r="AP25" s="11"/>
       <c r="AQ25" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -2999,7 +3089,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="9"/>
       <c r="H26" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I26" s="2"/>
@@ -3008,7 +3098,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="9"/>
       <c r="N26" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O26" s="2"/>
@@ -3017,7 +3107,7 @@
       <c r="R26" s="2"/>
       <c r="S26" s="9"/>
       <c r="T26" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U26" s="2"/>
@@ -3026,7 +3116,7 @@
       <c r="X26" s="2"/>
       <c r="Y26" s="9"/>
       <c r="Z26" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA26" s="2"/>
@@ -3035,7 +3125,7 @@
       <c r="AD26" s="2"/>
       <c r="AE26" s="9"/>
       <c r="AF26" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG26" s="2"/>
@@ -3044,7 +3134,7 @@
       <c r="AJ26" s="2"/>
       <c r="AK26" s="9"/>
       <c r="AL26" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM26" s="6" cm="1">
@@ -3052,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="AN26" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO26">
@@ -3060,7 +3150,7 @@
       </c>
       <c r="AP26" s="11"/>
       <c r="AQ26" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3072,7 +3162,7 @@
       <c r="F27" s="2"/>
       <c r="G27" s="9"/>
       <c r="H27" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I27" s="2"/>
@@ -3081,7 +3171,7 @@
       <c r="L27" s="2"/>
       <c r="M27" s="9"/>
       <c r="N27" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O27" s="2"/>
@@ -3090,7 +3180,7 @@
       <c r="R27" s="2"/>
       <c r="S27" s="9"/>
       <c r="T27" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U27" s="2"/>
@@ -3099,7 +3189,7 @@
       <c r="X27" s="2"/>
       <c r="Y27" s="9"/>
       <c r="Z27" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA27" s="2"/>
@@ -3108,7 +3198,7 @@
       <c r="AD27" s="2"/>
       <c r="AE27" s="9"/>
       <c r="AF27" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG27" s="2"/>
@@ -3117,7 +3207,7 @@
       <c r="AJ27" s="2"/>
       <c r="AK27" s="9"/>
       <c r="AL27" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM27" s="6" cm="1">
@@ -3125,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="AN27" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO27">
@@ -3133,7 +3223,7 @@
       </c>
       <c r="AP27" s="11"/>
       <c r="AQ27" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3145,7 +3235,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="9"/>
       <c r="H28" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I28" s="2"/>
@@ -3154,7 +3244,7 @@
       <c r="L28" s="2"/>
       <c r="M28" s="9"/>
       <c r="N28" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O28" s="2"/>
@@ -3163,7 +3253,7 @@
       <c r="R28" s="2"/>
       <c r="S28" s="9"/>
       <c r="T28" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U28" s="2"/>
@@ -3172,7 +3262,7 @@
       <c r="X28" s="2"/>
       <c r="Y28" s="9"/>
       <c r="Z28" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA28" s="2"/>
@@ -3181,7 +3271,7 @@
       <c r="AD28" s="2"/>
       <c r="AE28" s="9"/>
       <c r="AF28" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG28" s="2"/>
@@ -3190,7 +3280,7 @@
       <c r="AJ28" s="2"/>
       <c r="AK28" s="9"/>
       <c r="AL28" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM28" s="6" cm="1">
@@ -3198,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="AN28" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO28">
@@ -3206,7 +3296,7 @@
       </c>
       <c r="AP28" s="11"/>
       <c r="AQ28" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3218,7 +3308,7 @@
       <c r="F29" s="2"/>
       <c r="G29" s="9"/>
       <c r="H29" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I29" s="2"/>
@@ -3227,7 +3317,7 @@
       <c r="L29" s="2"/>
       <c r="M29" s="9"/>
       <c r="N29" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O29" s="2"/>
@@ -3236,7 +3326,7 @@
       <c r="R29" s="2"/>
       <c r="S29" s="9"/>
       <c r="T29" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U29" s="2"/>
@@ -3245,7 +3335,7 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="9"/>
       <c r="Z29" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA29" s="2"/>
@@ -3254,7 +3344,7 @@
       <c r="AD29" s="2"/>
       <c r="AE29" s="9"/>
       <c r="AF29" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG29" s="2"/>
@@ -3263,7 +3353,7 @@
       <c r="AJ29" s="2"/>
       <c r="AK29" s="9"/>
       <c r="AL29" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM29" s="6" cm="1">
@@ -3271,7 +3361,7 @@
         <v>0</v>
       </c>
       <c r="AN29" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO29">
@@ -3279,7 +3369,7 @@
       </c>
       <c r="AP29" s="11"/>
       <c r="AQ29" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3291,7 +3381,7 @@
       <c r="F30" s="2"/>
       <c r="G30" s="9"/>
       <c r="H30" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I30" s="2"/>
@@ -3300,7 +3390,7 @@
       <c r="L30" s="2"/>
       <c r="M30" s="9"/>
       <c r="N30" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O30" s="2"/>
@@ -3309,7 +3399,7 @@
       <c r="R30" s="2"/>
       <c r="S30" s="9"/>
       <c r="T30" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U30" s="2"/>
@@ -3318,7 +3408,7 @@
       <c r="X30" s="2"/>
       <c r="Y30" s="9"/>
       <c r="Z30" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA30" s="2"/>
@@ -3327,7 +3417,7 @@
       <c r="AD30" s="2"/>
       <c r="AE30" s="9"/>
       <c r="AF30" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG30" s="2"/>
@@ -3336,7 +3426,7 @@
       <c r="AJ30" s="2"/>
       <c r="AK30" s="9"/>
       <c r="AL30" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM30" s="6" cm="1">
@@ -3344,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="AN30" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO30">
@@ -3352,7 +3442,7 @@
       </c>
       <c r="AP30" s="11"/>
       <c r="AQ30" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3364,7 +3454,7 @@
       <c r="F31" s="2"/>
       <c r="G31" s="9"/>
       <c r="H31" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I31" s="2"/>
@@ -3373,7 +3463,7 @@
       <c r="L31" s="2"/>
       <c r="M31" s="9"/>
       <c r="N31" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O31" s="2"/>
@@ -3382,7 +3472,7 @@
       <c r="R31" s="2"/>
       <c r="S31" s="9"/>
       <c r="T31" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U31" s="2"/>
@@ -3391,7 +3481,7 @@
       <c r="X31" s="2"/>
       <c r="Y31" s="9"/>
       <c r="Z31" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA31" s="2"/>
@@ -3400,7 +3490,7 @@
       <c r="AD31" s="2"/>
       <c r="AE31" s="9"/>
       <c r="AF31" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG31" s="2"/>
@@ -3409,7 +3499,7 @@
       <c r="AJ31" s="2"/>
       <c r="AK31" s="9"/>
       <c r="AL31" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM31" s="6" cm="1">
@@ -3417,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="AN31" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO31">
@@ -3425,7 +3515,7 @@
       </c>
       <c r="AP31" s="11"/>
       <c r="AQ31" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3437,7 +3527,7 @@
       <c r="F32" s="2"/>
       <c r="G32" s="9"/>
       <c r="H32" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I32" s="2"/>
@@ -3446,7 +3536,7 @@
       <c r="L32" s="2"/>
       <c r="M32" s="9"/>
       <c r="N32" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O32" s="2"/>
@@ -3455,7 +3545,7 @@
       <c r="R32" s="2"/>
       <c r="S32" s="9"/>
       <c r="T32" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U32" s="2"/>
@@ -3464,7 +3554,7 @@
       <c r="X32" s="2"/>
       <c r="Y32" s="9"/>
       <c r="Z32" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA32" s="2"/>
@@ -3473,7 +3563,7 @@
       <c r="AD32" s="2"/>
       <c r="AE32" s="9"/>
       <c r="AF32" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG32" s="2"/>
@@ -3482,7 +3572,7 @@
       <c r="AJ32" s="2"/>
       <c r="AK32" s="9"/>
       <c r="AL32" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM32" s="6" cm="1">
@@ -3490,7 +3580,7 @@
         <v>0</v>
       </c>
       <c r="AN32" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO32">
@@ -3498,7 +3588,7 @@
       </c>
       <c r="AP32" s="11"/>
       <c r="AQ32" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
@@ -3510,7 +3600,7 @@
       <c r="F33" s="2"/>
       <c r="G33" s="9"/>
       <c r="H33" s="4">
-        <f t="shared" si="8"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I33" s="2"/>
@@ -3519,7 +3609,7 @@
       <c r="L33" s="2"/>
       <c r="M33" s="9"/>
       <c r="N33" s="4">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O33" s="2"/>
@@ -3528,7 +3618,7 @@
       <c r="R33" s="2"/>
       <c r="S33" s="9"/>
       <c r="T33" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U33" s="2"/>
@@ -3537,7 +3627,7 @@
       <c r="X33" s="2"/>
       <c r="Y33" s="9"/>
       <c r="Z33" s="4">
-        <f t="shared" si="11"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA33" s="2"/>
@@ -3546,7 +3636,7 @@
       <c r="AD33" s="2"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="4">
-        <f t="shared" si="12"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG33" s="2"/>
@@ -3555,7 +3645,7 @@
       <c r="AJ33" s="2"/>
       <c r="AK33" s="9"/>
       <c r="AL33" s="4">
-        <f t="shared" si="13"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM33" s="6" cm="1">
@@ -3563,7 +3653,7 @@
         <v>0</v>
       </c>
       <c r="AN33" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AO33">
@@ -3571,21 +3661,95 @@
       </c>
       <c r="AP33" s="11"/>
       <c r="AQ33" s="11">
-        <f t="shared" si="15"/>
+        <f t="shared" si="7"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" spans="2:43" x14ac:dyDescent="0.25">
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="O34" s="2"/>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="2"/>
+      <c r="R34" s="2"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U34" s="2"/>
+      <c r="V34" s="2"/>
+      <c r="W34" s="2"/>
+      <c r="X34" s="2"/>
+      <c r="Y34" s="9"/>
+      <c r="Z34" s="4">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA34" s="2"/>
+      <c r="AB34" s="2"/>
+      <c r="AC34" s="2"/>
+      <c r="AD34" s="2"/>
+      <c r="AE34" s="9"/>
+      <c r="AF34" s="4">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34" s="2"/>
+      <c r="AJ34" s="2"/>
+      <c r="AK34" s="9"/>
+      <c r="AL34" s="4">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AM34" s="6" cm="1">
+        <f t="array" ref="AM34">SUM(C34:F34+I34:L34+O34:R34+U34:X34+AA34:AD34+AG34:AJ34)</f>
+        <v>0</v>
+      </c>
+      <c r="AN34" s="8">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AO34">
+        <v>200</v>
+      </c>
+      <c r="AP34" s="11"/>
+      <c r="AQ34" s="11">
+        <f t="shared" si="7"/>
         <v>140</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:AQ20">
-    <sortCondition descending="1" ref="AN2:AN20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:AQ22">
+    <sortCondition descending="1" ref="AN3:AN22"/>
   </sortState>
-  <mergeCells count="6">
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="O1:R1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="AA1:AD1"/>
+  <mergeCells count="7">
+    <mergeCell ref="B1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="O2:R2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="AA2:AD2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added latest donaubowler CM results, changed sorting
</commit_message>
<xml_diff>
--- a/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
+++ b/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="DieseArbeitsmappe"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Dropbox\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3938F41E-A811-4515-8485-EFC252B27397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C87C71-D6C6-43D8-89F6-A548A75A3B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D7BAE6BD-B2A4-4DD1-AF79-906BD29E778A}"/>
   </bookViews>
@@ -145,10 +145,10 @@
     <t>Rang</t>
   </si>
   <si>
-    <t>Donaubowler Clubmeisterschaft 2026 / Stand 19.05.26</t>
+    <t>Richard Zorzi</t>
   </si>
   <si>
-    <t>Richard Zorzi</t>
+    <t>Donaubowler Clubmeisterschaft 2026 / Stand 21.05.26</t>
   </si>
 </sst>
 </file>
@@ -268,11 +268,11 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -617,7 +617,9 @@
     <col min="3" max="6" width="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="12" width="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="18" width="4" bestFit="1" customWidth="1"/>
@@ -639,27 +641,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="B1" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
-      <c r="T1" s="13"/>
+      <c r="B1" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -668,72 +670,72 @@
       <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
       <c r="G2" s="9" t="s">
         <v>28</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
       <c r="M2" s="9" t="s">
         <v>28</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
       <c r="S2" s="9" t="s">
         <v>28</v>
       </c>
       <c r="T2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="U2" s="12" t="s">
+      <c r="U2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
       <c r="Y2" s="9" t="s">
         <v>28</v>
       </c>
       <c r="Z2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AA2" s="12" t="s">
+      <c r="AA2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="AB2" s="12"/>
-      <c r="AC2" s="12"/>
-      <c r="AD2" s="12"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
       <c r="AE2" s="9" t="s">
         <v>28</v>
       </c>
       <c r="AF2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="AG2" s="12" t="s">
+      <c r="AG2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="AH2" s="12"/>
-      <c r="AI2" s="12"/>
-      <c r="AJ2" s="12"/>
+      <c r="AH2" s="13"/>
+      <c r="AI2" s="13"/>
+      <c r="AJ2" s="13"/>
       <c r="AK2" s="9" t="s">
         <v>28</v>
       </c>
@@ -755,82 +757,90 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="D3" s="3">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E3" s="3">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="F3" s="3">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="G3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4">
         <f>SUM(C3:G3)</f>
-        <v>843</v>
+        <v>888</v>
       </c>
       <c r="I3" s="3">
-        <v>191</v>
+        <v>245</v>
       </c>
       <c r="J3" s="3">
-        <v>232</v>
+        <v>194</v>
       </c>
       <c r="K3" s="3">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="L3" s="3">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="M3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="N3" s="4">
         <f>SUM(I3:L3)</f>
-        <v>830</v>
+        <v>845</v>
       </c>
       <c r="O3" s="3">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P3" s="3">
-        <v>203</v>
+        <v>179</v>
       </c>
       <c r="Q3" s="3">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="R3" s="3">
-        <v>239</v>
+        <v>192</v>
       </c>
       <c r="S3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="T3" s="4">
         <f>SUM(O3:R3)</f>
-        <v>875</v>
-      </c>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
+        <v>803</v>
+      </c>
+      <c r="U3" s="3">
+        <v>214</v>
+      </c>
+      <c r="V3" s="3">
+        <v>227</v>
+      </c>
+      <c r="W3" s="3">
+        <v>224</v>
+      </c>
+      <c r="X3" s="3">
+        <v>185</v>
+      </c>
       <c r="Y3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="4">
         <f>SUM(U3:X3)</f>
-        <v>0</v>
+        <v>850</v>
       </c>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3"/>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AF3" s="4">
         <f>SUM(AA3:AD3)</f>
@@ -841,7 +851,7 @@
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AL3" s="4">
         <f>SUM(AG3:AJ3)</f>
@@ -849,21 +859,21 @@
       </c>
       <c r="AM3" s="6" cm="1">
         <f t="array" ref="AM3">SUM(C3:F3+I3:L3+O3:R3+U3:X3+AA3:AD3+AG3:AJ3)</f>
-        <v>2532</v>
+        <v>3386</v>
       </c>
       <c r="AN3" s="8">
         <f>SUM(H3+N3+T3+Z3+AF3+AL3)</f>
-        <v>2548</v>
+        <v>3386</v>
       </c>
       <c r="AO3">
         <v>200</v>
       </c>
       <c r="AP3" s="11">
-        <v>193.83</v>
+        <v>207</v>
       </c>
       <c r="AQ3" s="11">
         <f>SUM((AO3-AP3)*0.7)</f>
-        <v>4.3189999999999911</v>
+        <v>-4.8999999999999995</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -871,71 +881,71 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C4" s="3">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="D4" s="3">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="E4" s="3">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="F4" s="3">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="G4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H4" s="4">
         <f>SUM(C4:G4)</f>
-        <v>888</v>
+        <v>843</v>
       </c>
       <c r="I4" s="3">
-        <v>245</v>
+        <v>191</v>
       </c>
       <c r="J4" s="3">
-        <v>194</v>
+        <v>232</v>
       </c>
       <c r="K4" s="3">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="L4" s="3">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="M4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="N4" s="4">
         <f>SUM(I4:L4)</f>
-        <v>845</v>
+        <v>830</v>
       </c>
       <c r="O4" s="3">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P4" s="3">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="Q4" s="3">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="R4" s="3">
-        <v>192</v>
+        <v>239</v>
       </c>
       <c r="S4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="T4" s="4">
         <f>SUM(O4:R4)</f>
-        <v>803</v>
+        <v>875</v>
       </c>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Z4" s="4">
         <f>SUM(U4:X4)</f>
@@ -946,7 +956,7 @@
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="AF4" s="4">
         <f>SUM(AA4:AD4)</f>
@@ -957,7 +967,7 @@
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="9">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="AL4" s="4">
         <f>SUM(AG4:AJ4)</f>
@@ -965,21 +975,21 @@
       </c>
       <c r="AM4" s="6" cm="1">
         <f t="array" ref="AM4">SUM(C4:F4+I4:L4+O4:R4+U4:X4+AA4:AD4+AG4:AJ4)</f>
-        <v>2536</v>
+        <v>2532</v>
       </c>
       <c r="AN4" s="8">
         <f>SUM(H4+N4+T4+Z4+AF4+AL4)</f>
-        <v>2536</v>
+        <v>2548</v>
       </c>
       <c r="AO4">
         <v>200</v>
       </c>
       <c r="AP4" s="11">
-        <v>207</v>
+        <v>193.83</v>
       </c>
       <c r="AQ4" s="11">
         <f>SUM((AO4-AP4)*0.7)</f>
-        <v>-4.8999999999999995</v>
+        <v>4.3189999999999911</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -1335,63 +1345,71 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3">
-        <v>190</v>
+        <v>152</v>
       </c>
       <c r="D8" s="3">
-        <v>193</v>
+        <v>160</v>
       </c>
       <c r="E8" s="3">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="F8" s="3">
-        <v>207</v>
+        <v>136</v>
       </c>
       <c r="G8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="H8" s="4">
         <f>SUM(C8:G8)</f>
-        <v>815</v>
+        <v>714</v>
       </c>
       <c r="I8" s="3">
-        <v>225</v>
+        <v>163</v>
       </c>
       <c r="J8" s="3">
-        <v>242</v>
+        <v>171</v>
       </c>
       <c r="K8" s="3">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="L8" s="3">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="M8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="N8" s="4">
         <f>SUM(I8:L8)</f>
-        <v>880</v>
-      </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
+        <v>685</v>
+      </c>
+      <c r="O8" s="3">
+        <v>156</v>
+      </c>
+      <c r="P8" s="3">
+        <v>174</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>150</v>
+      </c>
+      <c r="R8" s="3">
+        <v>184</v>
+      </c>
       <c r="S8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="T8" s="4">
         <f>SUM(O8:R8)</f>
-        <v>0</v>
+        <v>664</v>
       </c>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
       <c r="Y8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="Z8" s="4">
         <f>SUM(U8:X8)</f>
@@ -1402,7 +1420,7 @@
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
       <c r="AE8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="AF8" s="4">
         <f>SUM(AA8:AD8)</f>
@@ -1413,7 +1431,7 @@
       <c r="AI8" s="3"/>
       <c r="AJ8" s="3"/>
       <c r="AK8" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="AL8" s="4">
         <f>SUM(AG8:AJ8)</f>
@@ -1421,21 +1439,21 @@
       </c>
       <c r="AM8" s="6" cm="1">
         <f t="array" ref="AM8">SUM(C8:F8+I8:L8+O8:R8+U8:X8+AA8:AD8+AG8:AJ8)</f>
-        <v>1675</v>
+        <v>1995</v>
       </c>
       <c r="AN8" s="8">
         <f>SUM(H8+N8+T8+Z8+AF8+AL8)</f>
-        <v>1695</v>
+        <v>2063</v>
       </c>
       <c r="AO8">
         <v>200</v>
       </c>
       <c r="AP8" s="11">
-        <v>193.33</v>
+        <v>175.62</v>
       </c>
       <c r="AQ8" s="11">
         <f>SUM((AO8-AP8)*0.7)</f>
-        <v>4.6689999999999907</v>
+        <v>17.065999999999995</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -1443,85 +1461,93 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="2">
-        <v>220</v>
-      </c>
-      <c r="D9" s="2">
-        <v>190</v>
-      </c>
-      <c r="E9" s="2">
-        <v>188</v>
-      </c>
-      <c r="F9" s="2">
-        <v>202</v>
+        <v>6</v>
+      </c>
+      <c r="C9" s="3">
+        <v>156</v>
+      </c>
+      <c r="D9" s="3">
+        <v>157</v>
+      </c>
+      <c r="E9" s="3">
+        <v>140</v>
+      </c>
+      <c r="F9" s="3">
+        <v>195</v>
       </c>
       <c r="G9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="H9" s="4">
         <f>SUM(C9:G9)</f>
-        <v>840</v>
-      </c>
-      <c r="I9" s="2">
-        <v>213</v>
-      </c>
-      <c r="J9" s="2">
-        <v>242</v>
-      </c>
-      <c r="K9" s="2">
-        <v>177</v>
-      </c>
-      <c r="L9" s="2">
-        <v>185</v>
+        <v>780</v>
+      </c>
+      <c r="I9" s="3">
+        <v>145</v>
+      </c>
+      <c r="J9" s="3">
+        <v>100</v>
+      </c>
+      <c r="K9" s="3">
+        <v>150</v>
+      </c>
+      <c r="L9" s="3">
+        <v>191</v>
       </c>
       <c r="M9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="N9" s="4">
         <f>SUM(I9:L9)</f>
-        <v>817</v>
-      </c>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
+        <v>586</v>
+      </c>
+      <c r="O9" s="3">
+        <v>163</v>
+      </c>
+      <c r="P9" s="3">
+        <v>204</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>163</v>
+      </c>
+      <c r="R9" s="3">
+        <v>156</v>
+      </c>
       <c r="S9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="T9" s="4">
         <f>SUM(O9:R9)</f>
-        <v>0</v>
-      </c>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
+        <v>686</v>
+      </c>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
       <c r="Y9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="Z9" s="4">
         <f>SUM(U9:X9)</f>
         <v>0</v>
       </c>
-      <c r="AA9" s="2"/>
-      <c r="AB9" s="2"/>
-      <c r="AC9" s="2"/>
-      <c r="AD9" s="2"/>
+      <c r="AA9" s="3"/>
+      <c r="AB9" s="3"/>
+      <c r="AC9" s="3"/>
+      <c r="AD9" s="3"/>
       <c r="AE9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="AF9" s="4">
         <f>SUM(AA9:AD9)</f>
         <v>0</v>
       </c>
-      <c r="AG9" s="2"/>
-      <c r="AH9" s="2"/>
-      <c r="AI9" s="2"/>
-      <c r="AJ9" s="2"/>
+      <c r="AG9" s="3"/>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="3"/>
+      <c r="AJ9" s="3"/>
       <c r="AK9" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="AL9" s="4">
         <f>SUM(AG9:AJ9)</f>
@@ -1529,21 +1555,21 @@
       </c>
       <c r="AM9" s="6" cm="1">
         <f t="array" ref="AM9">SUM(C9:F9+I9:L9+O9:R9+U9:X9+AA9:AD9+AG9:AJ9)</f>
-        <v>1617</v>
+        <v>1920</v>
       </c>
       <c r="AN9" s="8">
         <f>SUM(H9+N9+T9+Z9+AF9+AL9)</f>
-        <v>1657</v>
+        <v>2052</v>
       </c>
       <c r="AO9">
         <v>200</v>
       </c>
       <c r="AP9" s="11">
-        <v>185.77</v>
+        <v>153</v>
       </c>
       <c r="AQ9" s="11">
         <f>SUM((AO9-AP9)*0.7)</f>
-        <v>9.9609999999999914</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -1551,85 +1577,85 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="2">
-        <v>246</v>
-      </c>
-      <c r="D10" s="2">
-        <v>192</v>
-      </c>
-      <c r="E10" s="2">
-        <v>176</v>
-      </c>
-      <c r="F10" s="2">
-        <v>199</v>
+        <v>2</v>
+      </c>
+      <c r="C10" s="3">
+        <v>190</v>
+      </c>
+      <c r="D10" s="3">
+        <v>193</v>
+      </c>
+      <c r="E10" s="3">
+        <v>205</v>
+      </c>
+      <c r="F10" s="3">
+        <v>207</v>
       </c>
       <c r="G10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="H10" s="4">
         <f>SUM(C10:G10)</f>
-        <v>857</v>
-      </c>
-      <c r="I10" s="2">
-        <v>177</v>
-      </c>
-      <c r="J10" s="2">
-        <v>146</v>
-      </c>
-      <c r="K10" s="2">
+        <v>815</v>
+      </c>
+      <c r="I10" s="3">
+        <v>225</v>
+      </c>
+      <c r="J10" s="3">
+        <v>242</v>
+      </c>
+      <c r="K10" s="3">
         <v>224</v>
       </c>
-      <c r="L10" s="2">
-        <v>178</v>
+      <c r="L10" s="3">
+        <v>189</v>
       </c>
       <c r="M10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="N10" s="4">
         <f>SUM(I10:L10)</f>
-        <v>725</v>
-      </c>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
+        <v>880</v>
+      </c>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
       <c r="S10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="T10" s="4">
         <f>SUM(O10:R10)</f>
         <v>0</v>
       </c>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
       <c r="Y10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="Z10" s="4">
         <f>SUM(U10:X10)</f>
         <v>0</v>
       </c>
-      <c r="AA10" s="2"/>
-      <c r="AB10" s="2"/>
-      <c r="AC10" s="2"/>
-      <c r="AD10" s="2"/>
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="3"/>
+      <c r="AC10" s="3"/>
+      <c r="AD10" s="3"/>
       <c r="AE10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AF10" s="4">
         <f>SUM(AA10:AD10)</f>
         <v>0</v>
       </c>
-      <c r="AG10" s="2"/>
-      <c r="AH10" s="2"/>
-      <c r="AI10" s="2"/>
-      <c r="AJ10" s="2"/>
+      <c r="AG10" s="3"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="3"/>
+      <c r="AJ10" s="3"/>
       <c r="AK10" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AL10" s="4">
         <f>SUM(AG10:AJ10)</f>
@@ -1637,21 +1663,21 @@
       </c>
       <c r="AM10" s="6" cm="1">
         <f t="array" ref="AM10">SUM(C10:F10+I10:L10+O10:R10+U10:X10+AA10:AD10+AG10:AJ10)</f>
-        <v>1538</v>
+        <v>1675</v>
       </c>
       <c r="AN10" s="8">
         <f>SUM(H10+N10+T10+Z10+AF10+AL10)</f>
-        <v>1582</v>
+        <v>1695</v>
       </c>
       <c r="AO10">
         <v>200</v>
       </c>
       <c r="AP10" s="11">
-        <v>185</v>
+        <v>193.33</v>
       </c>
       <c r="AQ10" s="11">
         <f>SUM((AO10-AP10)*0.7)</f>
-        <v>10.5</v>
+        <v>4.6689999999999907</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -1659,85 +1685,85 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="3">
-        <v>183</v>
-      </c>
-      <c r="D11" s="3">
-        <v>174</v>
-      </c>
-      <c r="E11" s="3">
-        <v>207</v>
-      </c>
-      <c r="F11" s="3">
-        <v>216</v>
+        <v>26</v>
+      </c>
+      <c r="C11" s="2">
+        <v>220</v>
+      </c>
+      <c r="D11" s="2">
+        <v>190</v>
+      </c>
+      <c r="E11" s="2">
+        <v>188</v>
+      </c>
+      <c r="F11" s="2">
+        <v>202</v>
       </c>
       <c r="G11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H11" s="4">
         <f>SUM(C11:G11)</f>
-        <v>800</v>
-      </c>
-      <c r="I11" s="3">
-        <v>174</v>
-      </c>
-      <c r="J11" s="3">
-        <v>190</v>
-      </c>
-      <c r="K11" s="3">
-        <v>146</v>
-      </c>
-      <c r="L11" s="3">
-        <v>136</v>
+        <v>840</v>
+      </c>
+      <c r="I11" s="2">
+        <v>213</v>
+      </c>
+      <c r="J11" s="2">
+        <v>242</v>
+      </c>
+      <c r="K11" s="2">
+        <v>177</v>
+      </c>
+      <c r="L11" s="2">
+        <v>185</v>
       </c>
       <c r="M11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N11" s="4">
         <f>SUM(I11:L11)</f>
-        <v>646</v>
-      </c>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
+        <v>817</v>
+      </c>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
       <c r="S11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="T11" s="4">
         <f>SUM(O11:R11)</f>
         <v>0</v>
       </c>
-      <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
       <c r="Y11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="Z11" s="4">
         <f>SUM(U11:X11)</f>
         <v>0</v>
       </c>
-      <c r="AA11" s="3"/>
-      <c r="AB11" s="3"/>
-      <c r="AC11" s="3"/>
-      <c r="AD11" s="3"/>
+      <c r="AA11" s="2"/>
+      <c r="AB11" s="2"/>
+      <c r="AC11" s="2"/>
+      <c r="AD11" s="2"/>
       <c r="AE11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="AF11" s="4">
         <f>SUM(AA11:AD11)</f>
         <v>0</v>
       </c>
-      <c r="AG11" s="3"/>
-      <c r="AH11" s="3"/>
-      <c r="AI11" s="3"/>
-      <c r="AJ11" s="3"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11" s="2"/>
+      <c r="AJ11" s="2"/>
       <c r="AK11" s="9">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="AL11" s="4">
         <f>SUM(AG11:AJ11)</f>
@@ -1745,21 +1771,21 @@
       </c>
       <c r="AM11" s="6" cm="1">
         <f t="array" ref="AM11">SUM(C11:F11+I11:L11+O11:R11+U11:X11+AA11:AD11+AG11:AJ11)</f>
-        <v>1426</v>
+        <v>1617</v>
       </c>
       <c r="AN11" s="8">
         <f>SUM(H11+N11+T11+Z11+AF11+AL11)</f>
-        <v>1446</v>
+        <v>1657</v>
       </c>
       <c r="AO11">
         <v>200</v>
       </c>
       <c r="AP11" s="11">
-        <v>192.5</v>
+        <v>185.77</v>
       </c>
       <c r="AQ11" s="11">
         <f>SUM((AO11-AP11)*0.7)</f>
-        <v>5.25</v>
+        <v>9.9609999999999914</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -1767,52 +1793,52 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2">
-        <v>172</v>
+        <v>246</v>
       </c>
       <c r="D12" s="2">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="E12" s="2">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="F12" s="2">
-        <v>162</v>
+        <v>199</v>
       </c>
       <c r="G12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="H12" s="4">
         <f>SUM(C12:G12)</f>
-        <v>746</v>
+        <v>857</v>
       </c>
       <c r="I12" s="2">
+        <v>177</v>
+      </c>
+      <c r="J12" s="2">
+        <v>146</v>
+      </c>
+      <c r="K12" s="2">
+        <v>224</v>
+      </c>
+      <c r="L12" s="2">
         <v>178</v>
       </c>
-      <c r="J12" s="2">
-        <v>178</v>
-      </c>
-      <c r="K12" s="2">
-        <v>132</v>
-      </c>
-      <c r="L12" s="2">
-        <v>169</v>
-      </c>
       <c r="M12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="N12" s="4">
         <f>SUM(I12:L12)</f>
-        <v>657</v>
+        <v>725</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
       <c r="S12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="T12" s="4">
         <f>SUM(O12:R12)</f>
@@ -1823,7 +1849,7 @@
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
       <c r="Y12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="Z12" s="4">
         <f>SUM(U12:X12)</f>
@@ -1834,7 +1860,7 @@
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
       <c r="AE12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="AF12" s="4">
         <f>SUM(AA12:AD12)</f>
@@ -1845,7 +1871,7 @@
       <c r="AI12" s="2"/>
       <c r="AJ12" s="2"/>
       <c r="AK12" s="9">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="AL12" s="4">
         <f>SUM(AG12:AJ12)</f>
@@ -1853,21 +1879,21 @@
       </c>
       <c r="AM12" s="6" cm="1">
         <f t="array" ref="AM12">SUM(C12:F12+I12:L12+O12:R12+U12:X12+AA12:AD12+AG12:AJ12)</f>
-        <v>1319</v>
+        <v>1538</v>
       </c>
       <c r="AN12" s="8">
         <f>SUM(H12+N12+T12+Z12+AF12+AL12)</f>
-        <v>1403</v>
+        <v>1582</v>
       </c>
       <c r="AO12">
         <v>200</v>
       </c>
       <c r="AP12" s="11">
-        <v>169.44</v>
+        <v>185</v>
       </c>
       <c r="AQ12" s="11">
         <f>SUM((AO12-AP12)*0.7)</f>
-        <v>21.391999999999999</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -1875,52 +1901,52 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D13" s="3">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E13" s="3">
-        <v>198</v>
+        <v>126</v>
       </c>
       <c r="F13" s="3">
-        <v>136</v>
+        <v>163</v>
       </c>
       <c r="G13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="H13" s="4">
         <f>SUM(C13:G13)</f>
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="I13" s="3">
-        <v>163</v>
+        <v>226</v>
       </c>
       <c r="J13" s="3">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="K13" s="3">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="L13" s="3">
-        <v>162</v>
+        <v>204</v>
       </c>
       <c r="M13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="N13" s="4">
         <f>SUM(I13:L13)</f>
-        <v>685</v>
+        <v>813</v>
       </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
       <c r="S13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="T13" s="4">
         <f>SUM(O13:R13)</f>
@@ -1931,7 +1957,7 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="Z13" s="4">
         <f>SUM(U13:X13)</f>
@@ -1942,7 +1968,7 @@
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
       <c r="AE13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="AF13" s="4">
         <f>SUM(AA13:AD13)</f>
@@ -1953,7 +1979,7 @@
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
       <c r="AK13" s="9">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="AL13" s="4">
         <f>SUM(AG13:AJ13)</f>
@@ -1961,21 +1987,21 @@
       </c>
       <c r="AM13" s="6" cm="1">
         <f t="array" ref="AM13">SUM(C13:F13+I13:L13+O13:R13+U13:X13+AA13:AD13+AG13:AJ13)</f>
-        <v>1331</v>
+        <v>1417</v>
       </c>
       <c r="AN13" s="8">
         <f>SUM(H13+N13+T13+Z13+AF13+AL13)</f>
-        <v>1399</v>
+        <v>1525</v>
       </c>
       <c r="AO13">
         <v>200</v>
       </c>
       <c r="AP13" s="11">
-        <v>175.62</v>
+        <v>161.46</v>
       </c>
       <c r="AQ13" s="11">
         <f>SUM((AO13-AP13)*0.7)</f>
-        <v>17.065999999999995</v>
+        <v>26.977999999999994</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -1983,85 +2009,85 @@
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="3">
-        <v>156</v>
-      </c>
-      <c r="D14" s="3">
-        <v>157</v>
-      </c>
-      <c r="E14" s="3">
-        <v>140</v>
-      </c>
-      <c r="F14" s="3">
-        <v>195</v>
+        <v>32</v>
+      </c>
+      <c r="C14" s="2">
+        <v>148</v>
+      </c>
+      <c r="D14" s="2">
+        <v>134</v>
+      </c>
+      <c r="E14" s="2">
+        <v>164</v>
+      </c>
+      <c r="F14" s="2">
+        <v>178</v>
       </c>
       <c r="G14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="H14" s="4">
         <f>SUM(C14:G14)</f>
-        <v>780</v>
-      </c>
-      <c r="I14" s="3">
-        <v>145</v>
-      </c>
-      <c r="J14" s="3">
-        <v>100</v>
-      </c>
-      <c r="K14" s="3">
-        <v>150</v>
-      </c>
-      <c r="L14" s="3">
-        <v>191</v>
+        <v>700</v>
+      </c>
+      <c r="I14" s="2">
+        <v>203</v>
+      </c>
+      <c r="J14" s="2">
+        <v>176</v>
+      </c>
+      <c r="K14" s="2">
+        <v>183</v>
+      </c>
+      <c r="L14" s="2">
+        <v>223</v>
       </c>
       <c r="M14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="N14" s="4">
         <f>SUM(I14:L14)</f>
-        <v>586</v>
-      </c>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
+        <v>785</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
       <c r="S14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="T14" s="4">
         <f>SUM(O14:R14)</f>
         <v>0</v>
       </c>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
       <c r="Y14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="Z14" s="4">
         <f>SUM(U14:X14)</f>
         <v>0</v>
       </c>
-      <c r="AA14" s="3"/>
-      <c r="AB14" s="3"/>
-      <c r="AC14" s="3"/>
-      <c r="AD14" s="3"/>
+      <c r="AA14" s="2"/>
+      <c r="AB14" s="2"/>
+      <c r="AC14" s="2"/>
+      <c r="AD14" s="2"/>
       <c r="AE14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="AF14" s="4">
         <f>SUM(AA14:AD14)</f>
         <v>0</v>
       </c>
-      <c r="AG14" s="3"/>
-      <c r="AH14" s="3"/>
-      <c r="AI14" s="3"/>
-      <c r="AJ14" s="3"/>
+      <c r="AG14" s="2"/>
+      <c r="AH14" s="2"/>
+      <c r="AI14" s="2"/>
+      <c r="AJ14" s="2"/>
       <c r="AK14" s="9">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="AL14" s="4">
         <f>SUM(AG14:AJ14)</f>
@@ -2069,21 +2095,21 @@
       </c>
       <c r="AM14" s="6" cm="1">
         <f t="array" ref="AM14">SUM(C14:F14+I14:L14+O14:R14+U14:X14+AA14:AD14+AG14:AJ14)</f>
-        <v>1234</v>
+        <v>1409</v>
       </c>
       <c r="AN14" s="8">
         <f>SUM(H14+N14+T14+Z14+AF14+AL14)</f>
-        <v>1366</v>
+        <v>1485</v>
       </c>
       <c r="AO14">
         <v>200</v>
       </c>
       <c r="AP14" s="11">
-        <v>153</v>
+        <v>173.14</v>
       </c>
       <c r="AQ14" s="11">
         <f>SUM((AO14-AP14)*0.7)</f>
-        <v>32.9</v>
+        <v>18.802000000000007</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -2112,16 +2138,24 @@
         <f>SUM(C15:G15)</f>
         <v>762</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="I15" s="3">
+        <v>182</v>
+      </c>
+      <c r="J15" s="3">
+        <v>202</v>
+      </c>
+      <c r="K15" s="3">
+        <v>158</v>
+      </c>
+      <c r="L15" s="3">
+        <v>163</v>
+      </c>
       <c r="M15" s="9">
         <v>92</v>
       </c>
       <c r="N15" s="4">
         <f>SUM(I15:L15)</f>
-        <v>0</v>
+        <v>705</v>
       </c>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
@@ -2169,11 +2203,11 @@
       </c>
       <c r="AM15" s="6" cm="1">
         <f t="array" ref="AM15">SUM(C15:F15+I15:L15+O15:R15+U15:X15+AA15:AD15+AG15:AJ15)</f>
-        <v>670</v>
+        <v>1375</v>
       </c>
       <c r="AN15" s="8">
         <f>SUM(H15+N15+T15+Z15+AF15+AL15)</f>
-        <v>762</v>
+        <v>1467</v>
       </c>
       <c r="AO15">
         <v>200</v>
@@ -2191,44 +2225,52 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="3">
+        <v>183</v>
+      </c>
+      <c r="D16" s="3">
+        <v>174</v>
+      </c>
+      <c r="E16" s="3">
+        <v>207</v>
+      </c>
+      <c r="F16" s="3">
+        <v>216</v>
+      </c>
+      <c r="G16" s="9">
         <v>20</v>
-      </c>
-      <c r="C16" s="3">
-        <v>177</v>
-      </c>
-      <c r="D16" s="3">
-        <v>199</v>
-      </c>
-      <c r="E16" s="3">
-        <v>134</v>
-      </c>
-      <c r="F16" s="3">
-        <v>211</v>
-      </c>
-      <c r="G16" s="9">
-        <v>16</v>
       </c>
       <c r="H16" s="4">
         <f>SUM(C16:G16)</f>
-        <v>737</v>
-      </c>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
+        <v>800</v>
+      </c>
+      <c r="I16" s="3">
+        <v>174</v>
+      </c>
+      <c r="J16" s="3">
+        <v>190</v>
+      </c>
+      <c r="K16" s="3">
+        <v>146</v>
+      </c>
+      <c r="L16" s="3">
+        <v>136</v>
+      </c>
       <c r="M16" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N16" s="4">
         <f>SUM(I16:L16)</f>
-        <v>0</v>
+        <v>646</v>
       </c>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
       <c r="S16" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="T16" s="4">
         <f>SUM(O16:R16)</f>
@@ -2239,7 +2281,7 @@
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
       <c r="Y16" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="Z16" s="4">
         <f>SUM(U16:X16)</f>
@@ -2250,7 +2292,7 @@
       <c r="AC16" s="3"/>
       <c r="AD16" s="3"/>
       <c r="AE16" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AF16" s="4">
         <f>SUM(AA16:AD16)</f>
@@ -2261,7 +2303,7 @@
       <c r="AI16" s="3"/>
       <c r="AJ16" s="3"/>
       <c r="AK16" s="9">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AL16" s="4">
         <f>SUM(AG16:AJ16)</f>
@@ -2269,21 +2311,21 @@
       </c>
       <c r="AM16" s="6" cm="1">
         <f t="array" ref="AM16">SUM(C16:F16+I16:L16+O16:R16+U16:X16+AA16:AD16+AG16:AJ16)</f>
-        <v>721</v>
+        <v>1426</v>
       </c>
       <c r="AN16" s="8">
         <f>SUM(H16+N16+T16+Z16+AF16+AL16)</f>
-        <v>737</v>
+        <v>1446</v>
       </c>
       <c r="AO16">
         <v>200</v>
       </c>
       <c r="AP16" s="11">
-        <v>194.7</v>
+        <v>192.5</v>
       </c>
       <c r="AQ16" s="11">
         <f>SUM((AO16-AP16)*0.7)</f>
-        <v>3.7100000000000075</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -2291,77 +2333,85 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="3">
-        <v>149</v>
-      </c>
-      <c r="D17" s="3">
-        <v>166</v>
-      </c>
-      <c r="E17" s="3">
-        <v>126</v>
-      </c>
-      <c r="F17" s="3">
-        <v>163</v>
+        <v>24</v>
+      </c>
+      <c r="C17" s="2">
+        <v>172</v>
+      </c>
+      <c r="D17" s="2">
+        <v>174</v>
+      </c>
+      <c r="E17" s="2">
+        <v>154</v>
+      </c>
+      <c r="F17" s="2">
+        <v>162</v>
       </c>
       <c r="G17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="H17" s="4">
         <f>SUM(C17:G17)</f>
-        <v>712</v>
-      </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+        <v>746</v>
+      </c>
+      <c r="I17" s="2">
+        <v>178</v>
+      </c>
+      <c r="J17" s="2">
+        <v>178</v>
+      </c>
+      <c r="K17" s="2">
+        <v>132</v>
+      </c>
+      <c r="L17" s="2">
+        <v>169</v>
+      </c>
       <c r="M17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="N17" s="4">
         <f>SUM(I17:L17)</f>
-        <v>0</v>
-      </c>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
+        <v>657</v>
+      </c>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
       <c r="S17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="T17" s="4">
         <f>SUM(O17:R17)</f>
         <v>0</v>
       </c>
-      <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
-      <c r="X17" s="3"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="2"/>
+      <c r="W17" s="2"/>
+      <c r="X17" s="2"/>
       <c r="Y17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="Z17" s="4">
         <f>SUM(U17:X17)</f>
         <v>0</v>
       </c>
-      <c r="AA17" s="3"/>
-      <c r="AB17" s="3"/>
-      <c r="AC17" s="3"/>
-      <c r="AD17" s="3"/>
+      <c r="AA17" s="2"/>
+      <c r="AB17" s="2"/>
+      <c r="AC17" s="2"/>
+      <c r="AD17" s="2"/>
       <c r="AE17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="AF17" s="4">
         <f>SUM(AA17:AD17)</f>
         <v>0</v>
       </c>
-      <c r="AG17" s="3"/>
-      <c r="AH17" s="3"/>
-      <c r="AI17" s="3"/>
-      <c r="AJ17" s="3"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="2"/>
+      <c r="AI17" s="2"/>
+      <c r="AJ17" s="2"/>
       <c r="AK17" s="9">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="AL17" s="4">
         <f>SUM(AG17:AJ17)</f>
@@ -2369,21 +2419,21 @@
       </c>
       <c r="AM17" s="6" cm="1">
         <f t="array" ref="AM17">SUM(C17:F17+I17:L17+O17:R17+U17:X17+AA17:AD17+AG17:AJ17)</f>
-        <v>604</v>
+        <v>1319</v>
       </c>
       <c r="AN17" s="8">
         <f>SUM(H17+N17+T17+Z17+AF17+AL17)</f>
-        <v>712</v>
+        <v>1403</v>
       </c>
       <c r="AO17">
         <v>200</v>
       </c>
       <c r="AP17" s="11">
-        <v>161.46</v>
+        <v>169.44</v>
       </c>
       <c r="AQ17" s="11">
         <f>SUM((AO17-AP17)*0.7)</f>
-        <v>26.977999999999994</v>
+        <v>21.391999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -2391,77 +2441,77 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="2">
-        <v>148</v>
-      </c>
-      <c r="D18" s="2">
+        <v>20</v>
+      </c>
+      <c r="C18" s="3">
+        <v>177</v>
+      </c>
+      <c r="D18" s="3">
+        <v>199</v>
+      </c>
+      <c r="E18" s="3">
         <v>134</v>
       </c>
-      <c r="E18" s="2">
-        <v>164</v>
-      </c>
-      <c r="F18" s="2">
-        <v>178</v>
+      <c r="F18" s="3">
+        <v>211</v>
       </c>
       <c r="G18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="H18" s="4">
         <f>SUM(C18:G18)</f>
-        <v>700</v>
-      </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
+        <v>737</v>
+      </c>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
       <c r="M18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="N18" s="4">
         <f>SUM(I18:L18)</f>
         <v>0</v>
       </c>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
       <c r="S18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="T18" s="4">
         <f>SUM(O18:R18)</f>
         <v>0</v>
       </c>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
       <c r="Y18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="Z18" s="4">
         <f>SUM(U18:X18)</f>
         <v>0</v>
       </c>
-      <c r="AA18" s="2"/>
-      <c r="AB18" s="2"/>
-      <c r="AC18" s="2"/>
-      <c r="AD18" s="2"/>
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3"/>
+      <c r="AC18" s="3"/>
+      <c r="AD18" s="3"/>
       <c r="AE18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="AF18" s="4">
         <f>SUM(AA18:AD18)</f>
         <v>0</v>
       </c>
-      <c r="AG18" s="2"/>
-      <c r="AH18" s="2"/>
-      <c r="AI18" s="2"/>
-      <c r="AJ18" s="2"/>
+      <c r="AG18" s="3"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="3"/>
       <c r="AK18" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="AL18" s="4">
         <f>SUM(AG18:AJ18)</f>
@@ -2469,21 +2519,21 @@
       </c>
       <c r="AM18" s="6" cm="1">
         <f t="array" ref="AM18">SUM(C18:F18+I18:L18+O18:R18+U18:X18+AA18:AD18+AG18:AJ18)</f>
-        <v>624</v>
+        <v>721</v>
       </c>
       <c r="AN18" s="8">
         <f>SUM(H18+N18+T18+Z18+AF18+AL18)</f>
-        <v>700</v>
+        <v>737</v>
       </c>
       <c r="AO18">
         <v>200</v>
       </c>
       <c r="AP18" s="11">
-        <v>173.14</v>
+        <v>194.7</v>
       </c>
       <c r="AQ18" s="11">
         <f>SUM((AO18-AP18)*0.7)</f>
-        <v>18.802000000000007</v>
+        <v>3.7100000000000075</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -2870,7 +2920,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="9"/>
       <c r="H23" s="4">
-        <f t="shared" ref="H22:H34" si="0">SUM(C23:G23)</f>
+        <f t="shared" ref="H23:H34" si="0">SUM(C23:G23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="2"/>
@@ -2879,7 +2929,7 @@
       <c r="L23" s="2"/>
       <c r="M23" s="9"/>
       <c r="N23" s="4">
-        <f t="shared" ref="N22:N34" si="1">SUM(I23:L23)</f>
+        <f t="shared" ref="N23:N34" si="1">SUM(I23:L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="2"/>
@@ -2888,7 +2938,7 @@
       <c r="R23" s="2"/>
       <c r="S23" s="9"/>
       <c r="T23" s="4">
-        <f t="shared" ref="T22:T34" si="2">SUM(O23:R23)</f>
+        <f t="shared" ref="T23:T34" si="2">SUM(O23:R23)</f>
         <v>0</v>
       </c>
       <c r="U23" s="2"/>
@@ -2897,7 +2947,7 @@
       <c r="X23" s="2"/>
       <c r="Y23" s="9"/>
       <c r="Z23" s="4">
-        <f t="shared" ref="Z22:Z34" si="3">SUM(U23:X23)</f>
+        <f t="shared" ref="Z23:Z34" si="3">SUM(U23:X23)</f>
         <v>0</v>
       </c>
       <c r="AA23" s="2"/>
@@ -2906,7 +2956,7 @@
       <c r="AD23" s="2"/>
       <c r="AE23" s="9"/>
       <c r="AF23" s="4">
-        <f t="shared" ref="AF22:AF34" si="4">SUM(AA23:AD23)</f>
+        <f t="shared" ref="AF23:AF34" si="4">SUM(AA23:AD23)</f>
         <v>0</v>
       </c>
       <c r="AG23" s="2"/>
@@ -2915,7 +2965,7 @@
       <c r="AJ23" s="2"/>
       <c r="AK23" s="9"/>
       <c r="AL23" s="4">
-        <f t="shared" ref="AL22:AL34" si="5">SUM(AG23:AJ23)</f>
+        <f t="shared" ref="AL23:AL34" si="5">SUM(AG23:AJ23)</f>
         <v>0</v>
       </c>
       <c r="AM23" s="6" cm="1">
@@ -2923,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="AN23" s="8">
-        <f t="shared" ref="AN22:AN34" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
+        <f t="shared" ref="AN23:AN34" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
         <v>0</v>
       </c>
       <c r="AO23">
@@ -2931,7 +2981,7 @@
       </c>
       <c r="AP23" s="11"/>
       <c r="AQ23" s="11">
-        <f t="shared" ref="AQ22:AQ34" si="7">SUM((AO23-AP23)*0.7)</f>
+        <f t="shared" ref="AQ23:AQ34" si="7">SUM((AO23-AP23)*0.7)</f>
         <v>140</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(data): publish merged league history and parquet-first loading
Add build_published_dataset pipeline, merged league/tournament parquets, path layout docs, and data-access/metadata support for ~15 seasons of published results.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
+++ b/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C87C71-D6C6-43D8-89F6-A548A75A3B60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED689F11-B6CF-4BAC-A24F-3B33287BCD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D7BAE6BD-B2A4-4DD1-AF79-906BD29E778A}"/>
   </bookViews>
@@ -148,7 +148,7 @@
     <t>Richard Zorzi</t>
   </si>
   <si>
-    <t>Donaubowler Clubmeisterschaft 2026 / Stand 21.05.26</t>
+    <t>Donaubowler Clubmeisterschaft 2026 / Stand 02.06.26</t>
   </si>
 </sst>
 </file>
@@ -757,123 +757,131 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="D3" s="3">
-        <v>239</v>
+        <v>214</v>
       </c>
       <c r="E3" s="3">
-        <v>224</v>
+        <v>167</v>
       </c>
       <c r="F3" s="3">
-        <v>209</v>
+        <v>171</v>
       </c>
       <c r="G3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="H3" s="4">
-        <f>SUM(C3:G3)</f>
-        <v>888</v>
+        <f t="shared" ref="H3:H22" si="0">SUM(C3:G3)</f>
+        <v>823</v>
       </c>
       <c r="I3" s="3">
-        <v>245</v>
+        <v>179</v>
       </c>
       <c r="J3" s="3">
+        <v>215</v>
+      </c>
+      <c r="K3" s="3">
+        <v>193</v>
+      </c>
+      <c r="L3" s="3">
         <v>194</v>
       </c>
-      <c r="K3" s="3">
-        <v>190</v>
-      </c>
-      <c r="L3" s="3">
-        <v>216</v>
-      </c>
       <c r="M3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="N3" s="4">
-        <f>SUM(I3:L3)</f>
-        <v>845</v>
+        <f t="shared" ref="N3:N22" si="1">SUM(I3:L3)</f>
+        <v>781</v>
       </c>
       <c r="O3" s="3">
-        <v>215</v>
+        <v>148</v>
       </c>
       <c r="P3" s="3">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="Q3" s="3">
-        <v>217</v>
+        <v>177</v>
       </c>
       <c r="R3" s="3">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="S3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="T3" s="4">
-        <f>SUM(O3:R3)</f>
-        <v>803</v>
+        <f t="shared" ref="T3:T22" si="2">SUM(O3:R3)</f>
+        <v>656</v>
       </c>
       <c r="U3" s="3">
+        <v>148</v>
+      </c>
+      <c r="V3" s="3">
+        <v>156</v>
+      </c>
+      <c r="W3" s="3">
         <v>214</v>
       </c>
-      <c r="V3" s="3">
-        <v>227</v>
-      </c>
-      <c r="W3" s="3">
-        <v>224</v>
-      </c>
       <c r="X3" s="3">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="Y3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="Z3" s="4">
-        <f>SUM(U3:X3)</f>
-        <v>850</v>
-      </c>
-      <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
+        <f t="shared" ref="Z3:Z22" si="3">SUM(U3:X3)</f>
+        <v>719</v>
+      </c>
+      <c r="AA3" s="3">
+        <v>123</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>203</v>
+      </c>
+      <c r="AC3" s="3">
+        <v>168</v>
+      </c>
+      <c r="AD3" s="3">
+        <v>181</v>
+      </c>
       <c r="AE3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="AF3" s="4">
-        <f>SUM(AA3:AD3)</f>
-        <v>0</v>
+        <f t="shared" ref="AF3:AF22" si="4">SUM(AA3:AD3)</f>
+        <v>675</v>
       </c>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="9">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="AL3" s="4">
-        <f>SUM(AG3:AJ3)</f>
+        <f t="shared" ref="AL3:AL22" si="5">SUM(AG3:AJ3)</f>
         <v>0</v>
       </c>
       <c r="AM3" s="6" cm="1">
         <f t="array" ref="AM3">SUM(C3:F3+I3:L3+O3:R3+U3:X3+AA3:AD3+AG3:AJ3)</f>
-        <v>3386</v>
+        <v>3578</v>
       </c>
       <c r="AN3" s="8">
-        <f>SUM(H3+N3+T3+Z3+AF3+AL3)</f>
-        <v>3386</v>
+        <f t="shared" ref="AN3:AN22" si="6">SUM(H3+N3+T3+Z3+AF3+AL3)</f>
+        <v>3654</v>
       </c>
       <c r="AO3">
         <v>200</v>
       </c>
       <c r="AP3" s="11">
-        <v>207</v>
+        <v>173.04</v>
       </c>
       <c r="AQ3" s="11">
-        <f>SUM((AO3-AP3)*0.7)</f>
-        <v>-4.8999999999999995</v>
+        <f t="shared" ref="AQ3:AQ22" si="7">SUM((AO3-AP3)*0.7)</f>
+        <v>18.872000000000003</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -881,85 +889,93 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="D4" s="3">
+        <v>239</v>
+      </c>
+      <c r="E4" s="3">
+        <v>224</v>
+      </c>
+      <c r="F4" s="3">
+        <v>209</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <f t="shared" si="0"/>
+        <v>888</v>
+      </c>
+      <c r="I4" s="3">
+        <v>245</v>
+      </c>
+      <c r="J4" s="3">
+        <v>194</v>
+      </c>
+      <c r="K4" s="3">
+        <v>190</v>
+      </c>
+      <c r="L4" s="3">
+        <v>216</v>
+      </c>
+      <c r="M4" s="9">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4">
+        <f t="shared" si="1"/>
+        <v>845</v>
+      </c>
+      <c r="O4" s="3">
+        <v>215</v>
+      </c>
+      <c r="P4" s="3">
+        <v>179</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>217</v>
+      </c>
+      <c r="R4" s="3">
+        <v>192</v>
+      </c>
+      <c r="S4" s="9">
+        <v>0</v>
+      </c>
+      <c r="T4" s="4">
+        <f t="shared" si="2"/>
+        <v>803</v>
+      </c>
+      <c r="U4" s="3">
+        <v>214</v>
+      </c>
+      <c r="V4" s="3">
         <v>227</v>
       </c>
-      <c r="E4" s="3">
-        <v>205</v>
-      </c>
-      <c r="F4" s="3">
-        <v>190</v>
-      </c>
-      <c r="G4" s="9">
-        <v>16</v>
-      </c>
-      <c r="H4" s="4">
-        <f>SUM(C4:G4)</f>
-        <v>843</v>
-      </c>
-      <c r="I4" s="3">
-        <v>191</v>
-      </c>
-      <c r="J4" s="3">
-        <v>232</v>
-      </c>
-      <c r="K4" s="3">
-        <v>183</v>
-      </c>
-      <c r="L4" s="3">
+      <c r="W4" s="3">
         <v>224</v>
       </c>
-      <c r="M4" s="9">
-        <v>16</v>
-      </c>
-      <c r="N4" s="4">
-        <f>SUM(I4:L4)</f>
-        <v>830</v>
-      </c>
-      <c r="O4" s="3">
-        <v>214</v>
-      </c>
-      <c r="P4" s="3">
-        <v>203</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>219</v>
-      </c>
-      <c r="R4" s="3">
-        <v>239</v>
-      </c>
-      <c r="S4" s="9">
-        <v>16</v>
-      </c>
-      <c r="T4" s="4">
-        <f>SUM(O4:R4)</f>
-        <v>875</v>
-      </c>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
+      <c r="X4" s="3">
+        <v>185</v>
+      </c>
       <c r="Y4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="4">
-        <f>SUM(U4:X4)</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>850</v>
       </c>
       <c r="AA4" s="3"/>
       <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AF4" s="4">
-        <f>SUM(AA4:AD4)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG4" s="3"/>
@@ -967,29 +983,29 @@
       <c r="AI4" s="3"/>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="9">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="AL4" s="4">
-        <f>SUM(AG4:AJ4)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM4" s="6" cm="1">
         <f t="array" ref="AM4">SUM(C4:F4+I4:L4+O4:R4+U4:X4+AA4:AD4+AG4:AJ4)</f>
-        <v>2532</v>
+        <v>3386</v>
       </c>
       <c r="AN4" s="8">
-        <f>SUM(H4+N4+T4+Z4+AF4+AL4)</f>
-        <v>2548</v>
+        <f t="shared" si="6"/>
+        <v>3386</v>
       </c>
       <c r="AO4">
         <v>200</v>
       </c>
       <c r="AP4" s="11">
-        <v>193.83</v>
+        <v>200</v>
       </c>
       <c r="AQ4" s="11">
-        <f>SUM((AO4-AP4)*0.7)</f>
-        <v>4.3189999999999911</v>
+        <f t="shared" si="7"/>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -997,85 +1013,93 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="D5" s="3">
+        <v>227</v>
+      </c>
+      <c r="E5" s="3">
+        <v>205</v>
+      </c>
+      <c r="F5" s="3">
+        <v>190</v>
+      </c>
+      <c r="G5" s="9">
+        <v>16</v>
+      </c>
+      <c r="H5" s="4">
+        <f t="shared" si="0"/>
+        <v>843</v>
+      </c>
+      <c r="I5" s="3">
+        <v>191</v>
+      </c>
+      <c r="J5" s="3">
+        <v>232</v>
+      </c>
+      <c r="K5" s="3">
+        <v>183</v>
+      </c>
+      <c r="L5" s="3">
+        <v>224</v>
+      </c>
+      <c r="M5" s="9">
+        <v>16</v>
+      </c>
+      <c r="N5" s="4">
+        <f t="shared" si="1"/>
+        <v>830</v>
+      </c>
+      <c r="O5" s="3">
         <v>214</v>
       </c>
-      <c r="E5" s="3">
-        <v>167</v>
-      </c>
-      <c r="F5" s="3">
-        <v>171</v>
-      </c>
-      <c r="G5" s="9">
-        <v>76</v>
-      </c>
-      <c r="H5" s="4">
-        <f>SUM(C5:G5)</f>
-        <v>823</v>
-      </c>
-      <c r="I5" s="3">
-        <v>179</v>
-      </c>
-      <c r="J5" s="3">
-        <v>215</v>
-      </c>
-      <c r="K5" s="3">
+      <c r="P5" s="3">
+        <v>203</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>219</v>
+      </c>
+      <c r="R5" s="3">
+        <v>239</v>
+      </c>
+      <c r="S5" s="9">
+        <v>16</v>
+      </c>
+      <c r="T5" s="4">
+        <f t="shared" si="2"/>
+        <v>875</v>
+      </c>
+      <c r="U5" s="3">
+        <v>204</v>
+      </c>
+      <c r="V5" s="3">
+        <v>203</v>
+      </c>
+      <c r="W5" s="3">
         <v>193</v>
       </c>
-      <c r="L5" s="3">
-        <v>194</v>
-      </c>
-      <c r="M5" s="9">
-        <v>76</v>
-      </c>
-      <c r="N5" s="4">
-        <f>SUM(I5:L5)</f>
-        <v>781</v>
-      </c>
-      <c r="O5" s="3">
-        <v>148</v>
-      </c>
-      <c r="P5" s="3">
-        <v>149</v>
-      </c>
-      <c r="Q5" s="3">
-        <v>177</v>
-      </c>
-      <c r="R5" s="3">
-        <v>182</v>
-      </c>
-      <c r="S5" s="9">
-        <v>76</v>
-      </c>
-      <c r="T5" s="4">
-        <f>SUM(O5:R5)</f>
-        <v>656</v>
-      </c>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
+      <c r="X5" s="3">
+        <v>176</v>
+      </c>
       <c r="Y5" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="Z5" s="4">
-        <f>SUM(U5:X5)</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>776</v>
       </c>
       <c r="AA5" s="3"/>
       <c r="AB5" s="3"/>
       <c r="AC5" s="3"/>
       <c r="AD5" s="3"/>
       <c r="AE5" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="AF5" s="4">
-        <f>SUM(AA5:AD5)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG5" s="3"/>
@@ -1083,29 +1107,29 @@
       <c r="AI5" s="3"/>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="9">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="AL5" s="4">
-        <f>SUM(AG5:AJ5)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM5" s="6" cm="1">
         <f t="array" ref="AM5">SUM(C5:F5+I5:L5+O5:R5+U5:X5+AA5:AD5+AG5:AJ5)</f>
-        <v>2184</v>
+        <v>3308</v>
       </c>
       <c r="AN5" s="8">
-        <f>SUM(H5+N5+T5+Z5+AF5+AL5)</f>
-        <v>2260</v>
+        <f t="shared" si="6"/>
+        <v>3324</v>
       </c>
       <c r="AO5">
         <v>200</v>
       </c>
       <c r="AP5" s="11">
-        <v>173.04</v>
+        <v>193.83</v>
       </c>
       <c r="AQ5" s="11">
-        <f>SUM((AO5-AP5)*0.7)</f>
-        <v>18.872000000000003</v>
+        <f t="shared" si="7"/>
+        <v>4.3189999999999911</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -1113,115 +1137,123 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2">
+        <v>220</v>
+      </c>
+      <c r="D6" s="2">
+        <v>190</v>
+      </c>
+      <c r="E6" s="2">
+        <v>188</v>
+      </c>
+      <c r="F6" s="2">
+        <v>202</v>
+      </c>
+      <c r="G6" s="9">
+        <v>40</v>
+      </c>
+      <c r="H6" s="4">
+        <f t="shared" si="0"/>
+        <v>840</v>
+      </c>
+      <c r="I6" s="2">
+        <v>213</v>
+      </c>
+      <c r="J6" s="2">
+        <v>242</v>
+      </c>
+      <c r="K6" s="2">
+        <v>177</v>
+      </c>
+      <c r="L6" s="2">
+        <v>185</v>
+      </c>
+      <c r="M6" s="9">
+        <v>40</v>
+      </c>
+      <c r="N6" s="4">
+        <f t="shared" si="1"/>
+        <v>817</v>
+      </c>
+      <c r="O6" s="2">
+        <v>194</v>
+      </c>
+      <c r="P6" s="2">
+        <v>148</v>
+      </c>
+      <c r="Q6" s="2">
         <v>200</v>
       </c>
-      <c r="D6" s="3">
-        <v>205</v>
-      </c>
-      <c r="E6" s="3">
-        <v>192</v>
-      </c>
-      <c r="F6" s="3">
-        <v>184</v>
-      </c>
-      <c r="G6" s="9">
-        <v>44</v>
-      </c>
-      <c r="H6" s="4">
-        <f>SUM(C6:G6)</f>
-        <v>825</v>
-      </c>
-      <c r="I6" s="3">
-        <v>174</v>
-      </c>
-      <c r="J6" s="3">
-        <v>200</v>
-      </c>
-      <c r="K6" s="3">
-        <v>189</v>
-      </c>
-      <c r="L6" s="3">
-        <v>147</v>
-      </c>
-      <c r="M6" s="9">
-        <v>44</v>
-      </c>
-      <c r="N6" s="4">
-        <f>SUM(I6:L6)</f>
-        <v>710</v>
-      </c>
-      <c r="O6" s="3">
-        <v>185</v>
-      </c>
-      <c r="P6" s="3">
-        <v>149</v>
-      </c>
-      <c r="Q6" s="3">
-        <v>167</v>
-      </c>
-      <c r="R6" s="3">
-        <v>213</v>
+      <c r="R6" s="2">
+        <v>259</v>
       </c>
       <c r="S6" s="9">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="T6" s="4">
-        <f>SUM(O6:R6)</f>
-        <v>714</v>
-      </c>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
+        <f t="shared" si="2"/>
+        <v>801</v>
+      </c>
+      <c r="U6" s="2">
+        <v>170</v>
+      </c>
+      <c r="V6" s="2">
+        <v>225</v>
+      </c>
+      <c r="W6" s="2">
+        <v>191</v>
+      </c>
+      <c r="X6" s="2">
+        <v>202</v>
+      </c>
       <c r="Y6" s="9">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="Z6" s="4">
-        <f>SUM(U6:X6)</f>
-        <v>0</v>
-      </c>
-      <c r="AA6" s="3"/>
-      <c r="AB6" s="3"/>
-      <c r="AC6" s="3"/>
-      <c r="AD6" s="3"/>
+        <f t="shared" si="3"/>
+        <v>788</v>
+      </c>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
       <c r="AE6" s="9">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="AF6" s="4">
-        <f>SUM(AA6:AD6)</f>
-        <v>0</v>
-      </c>
-      <c r="AG6" s="3"/>
-      <c r="AH6" s="3"/>
-      <c r="AI6" s="3"/>
-      <c r="AJ6" s="3"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
       <c r="AK6" s="9">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="AL6" s="4">
-        <f>SUM(AG6:AJ6)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM6" s="6" cm="1">
         <f t="array" ref="AM6">SUM(C6:F6+I6:L6+O6:R6+U6:X6+AA6:AD6+AG6:AJ6)</f>
-        <v>2205</v>
+        <v>3206</v>
       </c>
       <c r="AN6" s="8">
-        <f>SUM(H6+N6+T6+Z6+AF6+AL6)</f>
-        <v>2249</v>
+        <f t="shared" si="6"/>
+        <v>3246</v>
       </c>
       <c r="AO6">
         <v>200</v>
       </c>
       <c r="AP6" s="11">
-        <v>184.5</v>
+        <v>185.77</v>
       </c>
       <c r="AQ6" s="11">
-        <f>SUM((AO6-AP6)*0.7)</f>
-        <v>10.85</v>
+        <f t="shared" si="7"/>
+        <v>9.9609999999999914</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -1229,115 +1261,123 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="3">
-        <v>157</v>
-      </c>
-      <c r="D7" s="3">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2">
+        <v>246</v>
+      </c>
+      <c r="D7" s="2">
+        <v>192</v>
+      </c>
+      <c r="E7" s="2">
         <v>176</v>
       </c>
-      <c r="E7" s="3">
-        <v>180</v>
-      </c>
-      <c r="F7" s="3">
-        <v>192</v>
+      <c r="F7" s="2">
+        <v>199</v>
       </c>
       <c r="G7" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="H7" s="4">
-        <f>SUM(C7:G7)</f>
-        <v>801</v>
-      </c>
-      <c r="I7" s="3">
-        <v>200</v>
-      </c>
-      <c r="J7" s="3">
+        <f t="shared" si="0"/>
+        <v>857</v>
+      </c>
+      <c r="I7" s="2">
+        <v>177</v>
+      </c>
+      <c r="J7" s="2">
+        <v>146</v>
+      </c>
+      <c r="K7" s="2">
+        <v>224</v>
+      </c>
+      <c r="L7" s="2">
+        <v>178</v>
+      </c>
+      <c r="M7" s="9">
+        <v>44</v>
+      </c>
+      <c r="N7" s="4">
+        <f t="shared" si="1"/>
+        <v>725</v>
+      </c>
+      <c r="O7" s="2">
         <v>191</v>
       </c>
-      <c r="K7" s="3">
-        <v>194</v>
-      </c>
-      <c r="L7" s="3">
-        <v>204</v>
-      </c>
-      <c r="M7" s="9">
-        <v>96</v>
-      </c>
-      <c r="N7" s="4">
-        <f>SUM(I7:L7)</f>
-        <v>789</v>
-      </c>
-      <c r="O7" s="3">
-        <v>131</v>
-      </c>
-      <c r="P7" s="3">
-        <v>142</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>152</v>
-      </c>
-      <c r="R7" s="3">
-        <v>163</v>
+      <c r="P7" s="2">
+        <v>181</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>198</v>
+      </c>
+      <c r="R7" s="2">
+        <v>205</v>
       </c>
       <c r="S7" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="T7" s="4">
-        <f>SUM(O7:R7)</f>
-        <v>588</v>
-      </c>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
+        <f t="shared" si="2"/>
+        <v>775</v>
+      </c>
+      <c r="U7" s="2">
+        <v>198</v>
+      </c>
+      <c r="V7" s="2">
+        <v>171</v>
+      </c>
+      <c r="W7" s="2">
+        <v>156</v>
+      </c>
+      <c r="X7" s="2">
+        <v>173</v>
+      </c>
       <c r="Y7" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="Z7" s="4">
-        <f>SUM(U7:X7)</f>
-        <v>0</v>
-      </c>
-      <c r="AA7" s="3"/>
-      <c r="AB7" s="3"/>
-      <c r="AC7" s="3"/>
-      <c r="AD7" s="3"/>
+        <f t="shared" si="3"/>
+        <v>698</v>
+      </c>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
       <c r="AE7" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="AF7" s="4">
-        <f>SUM(AA7:AD7)</f>
-        <v>0</v>
-      </c>
-      <c r="AG7" s="3"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
       <c r="AK7" s="9">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="AL7" s="4">
-        <f>SUM(AG7:AJ7)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM7" s="6" cm="1">
         <f t="array" ref="AM7">SUM(C7:F7+I7:L7+O7:R7+U7:X7+AA7:AD7+AG7:AJ7)</f>
-        <v>2082</v>
+        <v>3011</v>
       </c>
       <c r="AN7" s="8">
-        <f>SUM(H7+N7+T7+Z7+AF7+AL7)</f>
-        <v>2178</v>
+        <f t="shared" si="6"/>
+        <v>3055</v>
       </c>
       <c r="AO7">
         <v>200</v>
       </c>
       <c r="AP7" s="11">
-        <v>166.35</v>
+        <v>185</v>
       </c>
       <c r="AQ7" s="11">
-        <f>SUM((AO7-AP7)*0.7)</f>
-        <v>23.555000000000003</v>
+        <f t="shared" si="7"/>
+        <v>10.5</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -1345,85 +1385,93 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C8" s="3">
+        <v>157</v>
+      </c>
+      <c r="D8" s="3">
+        <v>176</v>
+      </c>
+      <c r="E8" s="3">
+        <v>180</v>
+      </c>
+      <c r="F8" s="3">
+        <v>192</v>
+      </c>
+      <c r="G8" s="9">
+        <v>96</v>
+      </c>
+      <c r="H8" s="4">
+        <f t="shared" si="0"/>
+        <v>801</v>
+      </c>
+      <c r="I8" s="3">
+        <v>200</v>
+      </c>
+      <c r="J8" s="3">
+        <v>191</v>
+      </c>
+      <c r="K8" s="3">
+        <v>194</v>
+      </c>
+      <c r="L8" s="3">
+        <v>204</v>
+      </c>
+      <c r="M8" s="9">
+        <v>96</v>
+      </c>
+      <c r="N8" s="4">
+        <f t="shared" si="1"/>
+        <v>789</v>
+      </c>
+      <c r="O8" s="3">
+        <v>131</v>
+      </c>
+      <c r="P8" s="3">
+        <v>142</v>
+      </c>
+      <c r="Q8" s="3">
         <v>152</v>
       </c>
-      <c r="D8" s="3">
-        <v>160</v>
-      </c>
-      <c r="E8" s="3">
-        <v>198</v>
-      </c>
-      <c r="F8" s="3">
-        <v>136</v>
-      </c>
-      <c r="G8" s="9">
-        <v>68</v>
-      </c>
-      <c r="H8" s="4">
-        <f>SUM(C8:G8)</f>
-        <v>714</v>
-      </c>
-      <c r="I8" s="3">
+      <c r="R8" s="3">
         <v>163</v>
       </c>
-      <c r="J8" s="3">
-        <v>171</v>
-      </c>
-      <c r="K8" s="3">
-        <v>189</v>
-      </c>
-      <c r="L8" s="3">
-        <v>162</v>
-      </c>
-      <c r="M8" s="9">
-        <v>68</v>
-      </c>
-      <c r="N8" s="4">
-        <f>SUM(I8:L8)</f>
-        <v>685</v>
-      </c>
-      <c r="O8" s="3">
-        <v>156</v>
-      </c>
-      <c r="P8" s="3">
-        <v>174</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>150</v>
-      </c>
-      <c r="R8" s="3">
-        <v>184</v>
-      </c>
       <c r="S8" s="9">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="T8" s="4">
-        <f>SUM(O8:R8)</f>
-        <v>664</v>
-      </c>
-      <c r="U8" s="3"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
+        <f t="shared" si="2"/>
+        <v>588</v>
+      </c>
+      <c r="U8" s="3">
+        <v>192</v>
+      </c>
+      <c r="V8" s="3">
+        <v>168</v>
+      </c>
+      <c r="W8" s="3">
+        <v>157</v>
+      </c>
+      <c r="X8" s="3">
+        <v>210</v>
+      </c>
       <c r="Y8" s="9">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="Z8" s="4">
-        <f>SUM(U8:X8)</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>727</v>
       </c>
       <c r="AA8" s="3"/>
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
       <c r="AD8" s="3"/>
       <c r="AE8" s="9">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="AF8" s="4">
-        <f>SUM(AA8:AD8)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG8" s="3"/>
@@ -1431,29 +1479,29 @@
       <c r="AI8" s="3"/>
       <c r="AJ8" s="3"/>
       <c r="AK8" s="9">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="AL8" s="4">
-        <f>SUM(AG8:AJ8)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM8" s="6" cm="1">
         <f t="array" ref="AM8">SUM(C8:F8+I8:L8+O8:R8+U8:X8+AA8:AD8+AG8:AJ8)</f>
-        <v>1995</v>
+        <v>2809</v>
       </c>
       <c r="AN8" s="8">
-        <f>SUM(H8+N8+T8+Z8+AF8+AL8)</f>
-        <v>2063</v>
+        <f t="shared" si="6"/>
+        <v>2905</v>
       </c>
       <c r="AO8">
         <v>200</v>
       </c>
       <c r="AP8" s="11">
-        <v>175.62</v>
+        <v>166.36</v>
       </c>
       <c r="AQ8" s="11">
-        <f>SUM((AO8-AP8)*0.7)</f>
-        <v>17.065999999999995</v>
+        <f t="shared" si="7"/>
+        <v>23.547999999999988</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -1461,115 +1509,123 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="3">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2">
+        <v>172</v>
+      </c>
+      <c r="D9" s="2">
+        <v>174</v>
+      </c>
+      <c r="E9" s="2">
+        <v>154</v>
+      </c>
+      <c r="F9" s="2">
+        <v>162</v>
+      </c>
+      <c r="G9" s="9">
+        <v>84</v>
+      </c>
+      <c r="H9" s="4">
+        <f t="shared" si="0"/>
+        <v>746</v>
+      </c>
+      <c r="I9" s="2">
+        <v>178</v>
+      </c>
+      <c r="J9" s="2">
+        <v>178</v>
+      </c>
+      <c r="K9" s="2">
+        <v>132</v>
+      </c>
+      <c r="L9" s="2">
+        <v>169</v>
+      </c>
+      <c r="M9" s="9">
+        <v>84</v>
+      </c>
+      <c r="N9" s="4">
+        <f t="shared" si="1"/>
+        <v>657</v>
+      </c>
+      <c r="O9" s="2">
+        <v>179</v>
+      </c>
+      <c r="P9" s="2">
+        <v>173</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>169</v>
+      </c>
+      <c r="R9" s="2">
         <v>156</v>
       </c>
-      <c r="D9" s="3">
-        <v>157</v>
-      </c>
-      <c r="E9" s="3">
-        <v>140</v>
-      </c>
-      <c r="F9" s="3">
-        <v>195</v>
-      </c>
-      <c r="G9" s="9">
-        <v>132</v>
-      </c>
-      <c r="H9" s="4">
-        <f>SUM(C9:G9)</f>
-        <v>780</v>
-      </c>
-      <c r="I9" s="3">
-        <v>145</v>
-      </c>
-      <c r="J9" s="3">
-        <v>100</v>
-      </c>
-      <c r="K9" s="3">
-        <v>150</v>
-      </c>
-      <c r="L9" s="3">
+      <c r="S9" s="9">
+        <v>84</v>
+      </c>
+      <c r="T9" s="4">
+        <f t="shared" si="2"/>
+        <v>677</v>
+      </c>
+      <c r="U9" s="2">
         <v>191</v>
       </c>
-      <c r="M9" s="9">
-        <v>132</v>
-      </c>
-      <c r="N9" s="4">
-        <f>SUM(I9:L9)</f>
-        <v>586</v>
-      </c>
-      <c r="O9" s="3">
-        <v>163</v>
-      </c>
-      <c r="P9" s="3">
-        <v>204</v>
-      </c>
-      <c r="Q9" s="3">
-        <v>163</v>
-      </c>
-      <c r="R9" s="3">
-        <v>156</v>
-      </c>
-      <c r="S9" s="9">
-        <v>132</v>
-      </c>
-      <c r="T9" s="4">
-        <f>SUM(O9:R9)</f>
-        <v>686</v>
-      </c>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
+      <c r="V9" s="2">
+        <v>173</v>
+      </c>
+      <c r="W9" s="2">
+        <v>200</v>
+      </c>
+      <c r="X9" s="2">
+        <v>182</v>
+      </c>
       <c r="Y9" s="9">
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="Z9" s="4">
-        <f>SUM(U9:X9)</f>
-        <v>0</v>
-      </c>
-      <c r="AA9" s="3"/>
-      <c r="AB9" s="3"/>
-      <c r="AC9" s="3"/>
-      <c r="AD9" s="3"/>
+        <f t="shared" si="3"/>
+        <v>746</v>
+      </c>
+      <c r="AA9" s="2"/>
+      <c r="AB9" s="2"/>
+      <c r="AC9" s="2"/>
+      <c r="AD9" s="2"/>
       <c r="AE9" s="9">
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="AF9" s="4">
-        <f>SUM(AA9:AD9)</f>
-        <v>0</v>
-      </c>
-      <c r="AG9" s="3"/>
-      <c r="AH9" s="3"/>
-      <c r="AI9" s="3"/>
-      <c r="AJ9" s="3"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
+      <c r="AJ9" s="2"/>
       <c r="AK9" s="9">
-        <v>132</v>
+        <v>84</v>
       </c>
       <c r="AL9" s="4">
-        <f>SUM(AG9:AJ9)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM9" s="6" cm="1">
         <f t="array" ref="AM9">SUM(C9:F9+I9:L9+O9:R9+U9:X9+AA9:AD9+AG9:AJ9)</f>
-        <v>1920</v>
+        <v>2742</v>
       </c>
       <c r="AN9" s="8">
-        <f>SUM(H9+N9+T9+Z9+AF9+AL9)</f>
-        <v>2052</v>
+        <f t="shared" si="6"/>
+        <v>2826</v>
       </c>
       <c r="AO9">
         <v>200</v>
       </c>
       <c r="AP9" s="11">
-        <v>153</v>
+        <v>169.44</v>
       </c>
       <c r="AQ9" s="11">
-        <f>SUM((AO9-AP9)*0.7)</f>
-        <v>32.9</v>
+        <f t="shared" si="7"/>
+        <v>21.391999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -1577,77 +1633,93 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3">
-        <v>190</v>
+        <v>152</v>
       </c>
       <c r="D10" s="3">
-        <v>193</v>
+        <v>160</v>
       </c>
       <c r="E10" s="3">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="F10" s="3">
-        <v>207</v>
+        <v>136</v>
       </c>
       <c r="G10" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="H10" s="4">
-        <f>SUM(C10:G10)</f>
-        <v>815</v>
+        <f t="shared" si="0"/>
+        <v>714</v>
       </c>
       <c r="I10" s="3">
-        <v>225</v>
+        <v>163</v>
       </c>
       <c r="J10" s="3">
-        <v>242</v>
+        <v>171</v>
       </c>
       <c r="K10" s="3">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="L10" s="3">
+        <v>162</v>
+      </c>
+      <c r="M10" s="9">
+        <v>68</v>
+      </c>
+      <c r="N10" s="4">
+        <f t="shared" si="1"/>
+        <v>685</v>
+      </c>
+      <c r="O10" s="3">
+        <v>156</v>
+      </c>
+      <c r="P10" s="3">
+        <v>174</v>
+      </c>
+      <c r="Q10" s="3">
+        <v>150</v>
+      </c>
+      <c r="R10" s="3">
+        <v>184</v>
+      </c>
+      <c r="S10" s="9">
+        <v>68</v>
+      </c>
+      <c r="T10" s="4">
+        <f t="shared" si="2"/>
+        <v>664</v>
+      </c>
+      <c r="U10" s="3">
+        <v>178</v>
+      </c>
+      <c r="V10" s="3">
+        <v>161</v>
+      </c>
+      <c r="W10" s="3">
+        <v>212</v>
+      </c>
+      <c r="X10" s="3">
         <v>189</v>
       </c>
-      <c r="M10" s="9">
-        <v>20</v>
-      </c>
-      <c r="N10" s="4">
-        <f>SUM(I10:L10)</f>
-        <v>880</v>
-      </c>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="9">
-        <v>20</v>
-      </c>
-      <c r="T10" s="4">
-        <f>SUM(O10:R10)</f>
-        <v>0</v>
-      </c>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
       <c r="Y10" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="Z10" s="4">
-        <f>SUM(U10:X10)</f>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>740</v>
       </c>
       <c r="AA10" s="3"/>
       <c r="AB10" s="3"/>
       <c r="AC10" s="3"/>
       <c r="AD10" s="3"/>
       <c r="AE10" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="AF10" s="4">
-        <f>SUM(AA10:AD10)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG10" s="3"/>
@@ -1655,29 +1727,29 @@
       <c r="AI10" s="3"/>
       <c r="AJ10" s="3"/>
       <c r="AK10" s="9">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="AL10" s="4">
-        <f>SUM(AG10:AJ10)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM10" s="6" cm="1">
         <f t="array" ref="AM10">SUM(C10:F10+I10:L10+O10:R10+U10:X10+AA10:AD10+AG10:AJ10)</f>
-        <v>1675</v>
+        <v>2735</v>
       </c>
       <c r="AN10" s="8">
-        <f>SUM(H10+N10+T10+Z10+AF10+AL10)</f>
-        <v>1695</v>
+        <f t="shared" si="6"/>
+        <v>2803</v>
       </c>
       <c r="AO10">
         <v>200</v>
       </c>
       <c r="AP10" s="11">
-        <v>193.33</v>
+        <v>175.62</v>
       </c>
       <c r="AQ10" s="11">
-        <f>SUM((AO10-AP10)*0.7)</f>
-        <v>4.6689999999999907</v>
+        <f t="shared" si="7"/>
+        <v>17.065999999999995</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -1685,107 +1757,123 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="2">
-        <v>220</v>
-      </c>
-      <c r="D11" s="2">
-        <v>190</v>
-      </c>
-      <c r="E11" s="2">
-        <v>188</v>
-      </c>
-      <c r="F11" s="2">
-        <v>202</v>
+        <v>6</v>
+      </c>
+      <c r="C11" s="3">
+        <v>156</v>
+      </c>
+      <c r="D11" s="3">
+        <v>157</v>
+      </c>
+      <c r="E11" s="3">
+        <v>140</v>
+      </c>
+      <c r="F11" s="3">
+        <v>195</v>
       </c>
       <c r="G11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="H11" s="4">
-        <f>SUM(C11:G11)</f>
-        <v>840</v>
-      </c>
-      <c r="I11" s="2">
-        <v>213</v>
-      </c>
-      <c r="J11" s="2">
-        <v>242</v>
-      </c>
-      <c r="K11" s="2">
-        <v>177</v>
-      </c>
-      <c r="L11" s="2">
-        <v>185</v>
+        <f t="shared" si="0"/>
+        <v>780</v>
+      </c>
+      <c r="I11" s="3">
+        <v>145</v>
+      </c>
+      <c r="J11" s="3">
+        <v>100</v>
+      </c>
+      <c r="K11" s="3">
+        <v>150</v>
+      </c>
+      <c r="L11" s="3">
+        <v>191</v>
       </c>
       <c r="M11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="N11" s="4">
-        <f>SUM(I11:L11)</f>
-        <v>817</v>
-      </c>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
+        <f t="shared" si="1"/>
+        <v>586</v>
+      </c>
+      <c r="O11" s="3">
+        <v>163</v>
+      </c>
+      <c r="P11" s="3">
+        <v>204</v>
+      </c>
+      <c r="Q11" s="3">
+        <v>163</v>
+      </c>
+      <c r="R11" s="3">
+        <v>156</v>
+      </c>
       <c r="S11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="T11" s="4">
-        <f>SUM(O11:R11)</f>
-        <v>0</v>
-      </c>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
+        <f t="shared" si="2"/>
+        <v>686</v>
+      </c>
+      <c r="U11" s="3">
+        <v>135</v>
+      </c>
+      <c r="V11" s="3">
+        <v>136</v>
+      </c>
+      <c r="W11" s="3">
+        <v>147</v>
+      </c>
+      <c r="X11" s="3">
+        <v>178</v>
+      </c>
       <c r="Y11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="Z11" s="4">
-        <f>SUM(U11:X11)</f>
-        <v>0</v>
-      </c>
-      <c r="AA11" s="2"/>
-      <c r="AB11" s="2"/>
-      <c r="AC11" s="2"/>
-      <c r="AD11" s="2"/>
+        <f t="shared" si="3"/>
+        <v>596</v>
+      </c>
+      <c r="AA11" s="3"/>
+      <c r="AB11" s="3"/>
+      <c r="AC11" s="3"/>
+      <c r="AD11" s="3"/>
       <c r="AE11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="AF11" s="4">
-        <f>SUM(AA11:AD11)</f>
-        <v>0</v>
-      </c>
-      <c r="AG11" s="2"/>
-      <c r="AH11" s="2"/>
-      <c r="AI11" s="2"/>
-      <c r="AJ11" s="2"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG11" s="3"/>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
+      <c r="AJ11" s="3"/>
       <c r="AK11" s="9">
-        <v>40</v>
+        <v>132</v>
       </c>
       <c r="AL11" s="4">
-        <f>SUM(AG11:AJ11)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM11" s="6" cm="1">
         <f t="array" ref="AM11">SUM(C11:F11+I11:L11+O11:R11+U11:X11+AA11:AD11+AG11:AJ11)</f>
-        <v>1617</v>
+        <v>2516</v>
       </c>
       <c r="AN11" s="8">
-        <f>SUM(H11+N11+T11+Z11+AF11+AL11)</f>
-        <v>1657</v>
+        <f t="shared" si="6"/>
+        <v>2648</v>
       </c>
       <c r="AO11">
         <v>200</v>
       </c>
       <c r="AP11" s="11">
-        <v>185.77</v>
+        <v>152.86000000000001</v>
       </c>
       <c r="AQ11" s="11">
-        <f>SUM((AO11-AP11)*0.7)</f>
-        <v>9.9609999999999914</v>
+        <f t="shared" si="7"/>
+        <v>32.99799999999999</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -1793,107 +1881,115 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="2">
-        <v>246</v>
-      </c>
-      <c r="D12" s="2">
-        <v>192</v>
-      </c>
-      <c r="E12" s="2">
-        <v>176</v>
-      </c>
-      <c r="F12" s="2">
-        <v>199</v>
+        <v>2</v>
+      </c>
+      <c r="C12" s="3">
+        <v>190</v>
+      </c>
+      <c r="D12" s="3">
+        <v>193</v>
+      </c>
+      <c r="E12" s="3">
+        <v>205</v>
+      </c>
+      <c r="F12" s="3">
+        <v>207</v>
       </c>
       <c r="G12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="H12" s="4">
-        <f>SUM(C12:G12)</f>
-        <v>857</v>
-      </c>
-      <c r="I12" s="2">
-        <v>177</v>
-      </c>
-      <c r="J12" s="2">
-        <v>146</v>
-      </c>
-      <c r="K12" s="2">
+        <f t="shared" si="0"/>
+        <v>815</v>
+      </c>
+      <c r="I12" s="3">
+        <v>225</v>
+      </c>
+      <c r="J12" s="3">
+        <v>242</v>
+      </c>
+      <c r="K12" s="3">
         <v>224</v>
       </c>
-      <c r="L12" s="2">
-        <v>178</v>
+      <c r="L12" s="3">
+        <v>189</v>
       </c>
       <c r="M12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="N12" s="4">
-        <f>SUM(I12:L12)</f>
-        <v>725</v>
-      </c>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
+        <f t="shared" si="1"/>
+        <v>880</v>
+      </c>
+      <c r="O12" s="3">
+        <v>226</v>
+      </c>
+      <c r="P12" s="3">
+        <v>218</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>204</v>
+      </c>
+      <c r="R12" s="3">
+        <v>233</v>
+      </c>
       <c r="S12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="T12" s="4">
-        <f>SUM(O12:R12)</f>
-        <v>0</v>
-      </c>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
+        <f t="shared" si="2"/>
+        <v>881</v>
+      </c>
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
       <c r="Y12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="Z12" s="4">
-        <f>SUM(U12:X12)</f>
-        <v>0</v>
-      </c>
-      <c r="AA12" s="2"/>
-      <c r="AB12" s="2"/>
-      <c r="AC12" s="2"/>
-      <c r="AD12" s="2"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="3"/>
+      <c r="AC12" s="3"/>
+      <c r="AD12" s="3"/>
       <c r="AE12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AF12" s="4">
-        <f>SUM(AA12:AD12)</f>
-        <v>0</v>
-      </c>
-      <c r="AG12" s="2"/>
-      <c r="AH12" s="2"/>
-      <c r="AI12" s="2"/>
-      <c r="AJ12" s="2"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG12" s="3"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
+      <c r="AJ12" s="3"/>
       <c r="AK12" s="9">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="AL12" s="4">
-        <f>SUM(AG12:AJ12)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM12" s="6" cm="1">
         <f t="array" ref="AM12">SUM(C12:F12+I12:L12+O12:R12+U12:X12+AA12:AD12+AG12:AJ12)</f>
-        <v>1538</v>
+        <v>2556</v>
       </c>
       <c r="AN12" s="8">
-        <f>SUM(H12+N12+T12+Z12+AF12+AL12)</f>
-        <v>1582</v>
+        <f t="shared" si="6"/>
+        <v>2576</v>
       </c>
       <c r="AO12">
         <v>200</v>
       </c>
       <c r="AP12" s="11">
-        <v>185</v>
+        <v>193.33</v>
       </c>
       <c r="AQ12" s="11">
-        <f>SUM((AO12-AP12)*0.7)</f>
-        <v>10.5</v>
+        <f t="shared" si="7"/>
+        <v>4.6689999999999907</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -1901,66 +1997,74 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="D13" s="3">
-        <v>166</v>
+        <v>199</v>
       </c>
       <c r="E13" s="3">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F13" s="3">
-        <v>163</v>
+        <v>211</v>
       </c>
       <c r="G13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="H13" s="4">
-        <f>SUM(C13:G13)</f>
-        <v>712</v>
+        <f t="shared" si="0"/>
+        <v>737</v>
       </c>
       <c r="I13" s="3">
-        <v>226</v>
+        <v>200</v>
       </c>
       <c r="J13" s="3">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="K13" s="3">
+        <v>220</v>
+      </c>
+      <c r="L13" s="3">
         <v>203</v>
       </c>
-      <c r="L13" s="3">
-        <v>204</v>
-      </c>
       <c r="M13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="N13" s="4">
-        <f>SUM(I13:L13)</f>
+        <f t="shared" si="1"/>
         <v>813</v>
       </c>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
+      <c r="O13" s="3">
+        <v>222</v>
+      </c>
+      <c r="P13" s="3">
+        <v>227</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>228</v>
+      </c>
+      <c r="R13" s="3">
+        <v>201</v>
+      </c>
       <c r="S13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="T13" s="4">
-        <f>SUM(O13:R13)</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>878</v>
       </c>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
       <c r="Y13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="Z13" s="4">
-        <f>SUM(U13:X13)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA13" s="3"/>
@@ -1968,10 +2072,10 @@
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
       <c r="AE13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="AF13" s="4">
-        <f>SUM(AA13:AD13)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG13" s="3"/>
@@ -1979,29 +2083,29 @@
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
       <c r="AK13" s="9">
-        <v>108</v>
+        <v>16</v>
       </c>
       <c r="AL13" s="4">
-        <f>SUM(AG13:AJ13)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM13" s="6" cm="1">
         <f t="array" ref="AM13">SUM(C13:F13+I13:L13+O13:R13+U13:X13+AA13:AD13+AG13:AJ13)</f>
-        <v>1417</v>
+        <v>2412</v>
       </c>
       <c r="AN13" s="8">
-        <f>SUM(H13+N13+T13+Z13+AF13+AL13)</f>
-        <v>1525</v>
+        <f t="shared" si="6"/>
+        <v>2428</v>
       </c>
       <c r="AO13">
         <v>200</v>
       </c>
       <c r="AP13" s="11">
-        <v>161.46</v>
+        <v>194.71</v>
       </c>
       <c r="AQ13" s="11">
-        <f>SUM((AO13-AP13)*0.7)</f>
-        <v>26.977999999999994</v>
+        <f t="shared" si="7"/>
+        <v>3.7029999999999941</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -2009,107 +2113,115 @@
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="2">
-        <v>148</v>
-      </c>
-      <c r="D14" s="2">
-        <v>134</v>
-      </c>
-      <c r="E14" s="2">
-        <v>164</v>
-      </c>
-      <c r="F14" s="2">
-        <v>178</v>
+        <v>4</v>
+      </c>
+      <c r="C14" s="3">
+        <v>200</v>
+      </c>
+      <c r="D14" s="3">
+        <v>205</v>
+      </c>
+      <c r="E14" s="3">
+        <v>192</v>
+      </c>
+      <c r="F14" s="3">
+        <v>184</v>
       </c>
       <c r="G14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="H14" s="4">
-        <f>SUM(C14:G14)</f>
-        <v>700</v>
-      </c>
-      <c r="I14" s="2">
-        <v>203</v>
-      </c>
-      <c r="J14" s="2">
-        <v>176</v>
-      </c>
-      <c r="K14" s="2">
-        <v>183</v>
-      </c>
-      <c r="L14" s="2">
-        <v>223</v>
+        <f t="shared" si="0"/>
+        <v>825</v>
+      </c>
+      <c r="I14" s="3">
+        <v>174</v>
+      </c>
+      <c r="J14" s="3">
+        <v>200</v>
+      </c>
+      <c r="K14" s="3">
+        <v>189</v>
+      </c>
+      <c r="L14" s="3">
+        <v>147</v>
       </c>
       <c r="M14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="N14" s="4">
-        <f>SUM(I14:L14)</f>
-        <v>785</v>
-      </c>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
+        <f t="shared" si="1"/>
+        <v>710</v>
+      </c>
+      <c r="O14" s="3">
+        <v>185</v>
+      </c>
+      <c r="P14" s="3">
+        <v>149</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>167</v>
+      </c>
+      <c r="R14" s="3">
+        <v>213</v>
+      </c>
       <c r="S14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="T14" s="4">
-        <f>SUM(O14:R14)</f>
-        <v>0</v>
-      </c>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
+        <f t="shared" si="2"/>
+        <v>714</v>
+      </c>
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
       <c r="Y14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="Z14" s="4">
-        <f>SUM(U14:X14)</f>
-        <v>0</v>
-      </c>
-      <c r="AA14" s="2"/>
-      <c r="AB14" s="2"/>
-      <c r="AC14" s="2"/>
-      <c r="AD14" s="2"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+      <c r="AD14" s="3"/>
       <c r="AE14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="AF14" s="4">
-        <f>SUM(AA14:AD14)</f>
-        <v>0</v>
-      </c>
-      <c r="AG14" s="2"/>
-      <c r="AH14" s="2"/>
-      <c r="AI14" s="2"/>
-      <c r="AJ14" s="2"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG14" s="3"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="3"/>
       <c r="AK14" s="9">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="AL14" s="4">
-        <f>SUM(AG14:AJ14)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM14" s="6" cm="1">
         <f t="array" ref="AM14">SUM(C14:F14+I14:L14+O14:R14+U14:X14+AA14:AD14+AG14:AJ14)</f>
-        <v>1409</v>
+        <v>2205</v>
       </c>
       <c r="AN14" s="8">
-        <f>SUM(H14+N14+T14+Z14+AF14+AL14)</f>
-        <v>1485</v>
+        <f t="shared" si="6"/>
+        <v>2249</v>
       </c>
       <c r="AO14">
         <v>200</v>
       </c>
       <c r="AP14" s="11">
-        <v>173.14</v>
+        <v>184.5</v>
       </c>
       <c r="AQ14" s="11">
-        <f>SUM((AO14-AP14)*0.7)</f>
-        <v>18.802000000000007</v>
+        <f t="shared" si="7"/>
+        <v>10.85</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -2117,66 +2229,74 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C15" s="3">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="D15" s="3">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="E15" s="3">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="F15" s="3">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="H15" s="4">
-        <f>SUM(C15:G15)</f>
-        <v>762</v>
+        <f t="shared" si="0"/>
+        <v>712</v>
       </c>
       <c r="I15" s="3">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="J15" s="3">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="K15" s="3">
-        <v>158</v>
+        <v>203</v>
       </c>
       <c r="L15" s="3">
-        <v>163</v>
+        <v>204</v>
       </c>
       <c r="M15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="N15" s="4">
-        <f>SUM(I15:L15)</f>
-        <v>705</v>
-      </c>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
+        <f t="shared" si="1"/>
+        <v>813</v>
+      </c>
+      <c r="O15" s="3">
+        <v>148</v>
+      </c>
+      <c r="P15" s="3">
+        <v>192</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>156</v>
+      </c>
+      <c r="R15" s="3">
+        <v>190</v>
+      </c>
       <c r="S15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="T15" s="4">
-        <f>SUM(O15:R15)</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>686</v>
       </c>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
       <c r="Y15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="Z15" s="4">
-        <f>SUM(U15:X15)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA15" s="3"/>
@@ -2184,10 +2304,10 @@
       <c r="AC15" s="3"/>
       <c r="AD15" s="3"/>
       <c r="AE15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="AF15" s="4">
-        <f>SUM(AA15:AD15)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG15" s="3"/>
@@ -2195,29 +2315,29 @@
       <c r="AI15" s="3"/>
       <c r="AJ15" s="3"/>
       <c r="AK15" s="9">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="AL15" s="4">
-        <f>SUM(AG15:AJ15)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM15" s="6" cm="1">
         <f t="array" ref="AM15">SUM(C15:F15+I15:L15+O15:R15+U15:X15+AA15:AD15+AG15:AJ15)</f>
-        <v>1375</v>
+        <v>2103</v>
       </c>
       <c r="AN15" s="8">
-        <f>SUM(H15+N15+T15+Z15+AF15+AL15)</f>
-        <v>1467</v>
+        <f t="shared" si="6"/>
+        <v>2211</v>
       </c>
       <c r="AO15">
         <v>200</v>
       </c>
       <c r="AP15" s="11">
-        <v>167</v>
+        <v>161.47</v>
       </c>
       <c r="AQ15" s="11">
-        <f>SUM((AO15-AP15)*0.7)</f>
-        <v>23.099999999999998</v>
+        <f t="shared" si="7"/>
+        <v>26.971</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -2225,66 +2345,74 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="C16" s="3">
+        <v>179</v>
+      </c>
+      <c r="D16" s="3">
         <v>183</v>
       </c>
-      <c r="D16" s="3">
+      <c r="E16" s="3">
+        <v>144</v>
+      </c>
+      <c r="F16" s="3">
+        <v>164</v>
+      </c>
+      <c r="G16" s="9">
+        <v>92</v>
+      </c>
+      <c r="H16" s="4">
+        <f t="shared" si="0"/>
+        <v>762</v>
+      </c>
+      <c r="I16" s="3">
+        <v>182</v>
+      </c>
+      <c r="J16" s="3">
+        <v>202</v>
+      </c>
+      <c r="K16" s="3">
+        <v>158</v>
+      </c>
+      <c r="L16" s="3">
+        <v>163</v>
+      </c>
+      <c r="M16" s="9">
+        <v>92</v>
+      </c>
+      <c r="N16" s="4">
+        <f t="shared" si="1"/>
+        <v>705</v>
+      </c>
+      <c r="O16" s="3">
+        <v>155</v>
+      </c>
+      <c r="P16" s="3">
         <v>174</v>
       </c>
-      <c r="E16" s="3">
-        <v>207</v>
-      </c>
-      <c r="F16" s="3">
-        <v>216</v>
-      </c>
-      <c r="G16" s="9">
-        <v>20</v>
-      </c>
-      <c r="H16" s="4">
-        <f>SUM(C16:G16)</f>
-        <v>800</v>
-      </c>
-      <c r="I16" s="3">
-        <v>174</v>
-      </c>
-      <c r="J16" s="3">
-        <v>190</v>
-      </c>
-      <c r="K16" s="3">
-        <v>146</v>
-      </c>
-      <c r="L16" s="3">
-        <v>136</v>
-      </c>
-      <c r="M16" s="9">
-        <v>20</v>
-      </c>
-      <c r="N16" s="4">
-        <f>SUM(I16:L16)</f>
-        <v>646</v>
-      </c>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
+      <c r="Q16" s="3">
+        <v>180</v>
+      </c>
+      <c r="R16" s="3">
+        <v>203</v>
+      </c>
       <c r="S16" s="9">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="T16" s="4">
-        <f>SUM(O16:R16)</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>712</v>
       </c>
       <c r="U16" s="3"/>
       <c r="V16" s="3"/>
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
       <c r="Y16" s="9">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="Z16" s="4">
-        <f>SUM(U16:X16)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA16" s="3"/>
@@ -2292,10 +2420,10 @@
       <c r="AC16" s="3"/>
       <c r="AD16" s="3"/>
       <c r="AE16" s="9">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="AF16" s="4">
-        <f>SUM(AA16:AD16)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG16" s="3"/>
@@ -2303,29 +2431,29 @@
       <c r="AI16" s="3"/>
       <c r="AJ16" s="3"/>
       <c r="AK16" s="9">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="AL16" s="4">
-        <f>SUM(AG16:AJ16)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM16" s="6" cm="1">
         <f t="array" ref="AM16">SUM(C16:F16+I16:L16+O16:R16+U16:X16+AA16:AD16+AG16:AJ16)</f>
-        <v>1426</v>
+        <v>2087</v>
       </c>
       <c r="AN16" s="8">
-        <f>SUM(H16+N16+T16+Z16+AF16+AL16)</f>
-        <v>1446</v>
+        <f t="shared" si="6"/>
+        <v>2179</v>
       </c>
       <c r="AO16">
         <v>200</v>
       </c>
       <c r="AP16" s="11">
-        <v>192.5</v>
+        <v>167</v>
       </c>
       <c r="AQ16" s="11">
-        <f>SUM((AO16-AP16)*0.7)</f>
-        <v>5.25</v>
+        <f t="shared" si="7"/>
+        <v>23.099999999999998</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -2333,66 +2461,74 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2">
+        <v>148</v>
+      </c>
+      <c r="D17" s="2">
+        <v>134</v>
+      </c>
+      <c r="E17" s="2">
+        <v>164</v>
+      </c>
+      <c r="F17" s="2">
+        <v>178</v>
+      </c>
+      <c r="G17" s="9">
+        <v>76</v>
+      </c>
+      <c r="H17" s="4">
+        <f t="shared" si="0"/>
+        <v>700</v>
+      </c>
+      <c r="I17" s="2">
+        <v>203</v>
+      </c>
+      <c r="J17" s="2">
+        <v>176</v>
+      </c>
+      <c r="K17" s="2">
+        <v>183</v>
+      </c>
+      <c r="L17" s="2">
+        <v>223</v>
+      </c>
+      <c r="M17" s="9">
+        <v>76</v>
+      </c>
+      <c r="N17" s="4">
+        <f t="shared" si="1"/>
+        <v>785</v>
+      </c>
+      <c r="O17" s="2">
+        <v>164</v>
+      </c>
+      <c r="P17" s="2">
+        <v>160</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>169</v>
+      </c>
+      <c r="R17" s="2">
         <v>172</v>
       </c>
-      <c r="D17" s="2">
-        <v>174</v>
-      </c>
-      <c r="E17" s="2">
-        <v>154</v>
-      </c>
-      <c r="F17" s="2">
-        <v>162</v>
-      </c>
-      <c r="G17" s="9">
-        <v>84</v>
-      </c>
-      <c r="H17" s="4">
-        <f>SUM(C17:G17)</f>
-        <v>746</v>
-      </c>
-      <c r="I17" s="2">
-        <v>178</v>
-      </c>
-      <c r="J17" s="2">
-        <v>178</v>
-      </c>
-      <c r="K17" s="2">
-        <v>132</v>
-      </c>
-      <c r="L17" s="2">
-        <v>169</v>
-      </c>
-      <c r="M17" s="9">
-        <v>84</v>
-      </c>
-      <c r="N17" s="4">
-        <f>SUM(I17:L17)</f>
-        <v>657</v>
-      </c>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
       <c r="S17" s="9">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="T17" s="4">
-        <f>SUM(O17:R17)</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>665</v>
       </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
       <c r="Y17" s="9">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="Z17" s="4">
-        <f>SUM(U17:X17)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA17" s="2"/>
@@ -2400,10 +2536,10 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="9">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AF17" s="4">
-        <f>SUM(AA17:AD17)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG17" s="2"/>
@@ -2411,29 +2547,29 @@
       <c r="AI17" s="2"/>
       <c r="AJ17" s="2"/>
       <c r="AK17" s="9">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="AL17" s="4">
-        <f>SUM(AG17:AJ17)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM17" s="6" cm="1">
         <f t="array" ref="AM17">SUM(C17:F17+I17:L17+O17:R17+U17:X17+AA17:AD17+AG17:AJ17)</f>
-        <v>1319</v>
+        <v>2074</v>
       </c>
       <c r="AN17" s="8">
-        <f>SUM(H17+N17+T17+Z17+AF17+AL17)</f>
-        <v>1403</v>
+        <f t="shared" si="6"/>
+        <v>2150</v>
       </c>
       <c r="AO17">
         <v>200</v>
       </c>
       <c r="AP17" s="11">
-        <v>169.44</v>
+        <v>173.14</v>
       </c>
       <c r="AQ17" s="11">
-        <f>SUM((AO17-AP17)*0.7)</f>
-        <v>21.391999999999999</v>
+        <f t="shared" si="7"/>
+        <v>18.802000000000007</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -2441,99 +2577,107 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="3">
+        <v>23</v>
+      </c>
+      <c r="C18" s="2">
+        <v>151</v>
+      </c>
+      <c r="D18" s="2">
+        <v>182</v>
+      </c>
+      <c r="E18" s="2">
         <v>177</v>
       </c>
-      <c r="D18" s="3">
-        <v>199</v>
-      </c>
-      <c r="E18" s="3">
-        <v>134</v>
-      </c>
-      <c r="F18" s="3">
-        <v>211</v>
+      <c r="F18" s="2">
+        <v>147</v>
       </c>
       <c r="G18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H18" s="4">
-        <f>SUM(C18:G18)</f>
-        <v>737</v>
-      </c>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+        <f t="shared" si="0"/>
+        <v>693</v>
+      </c>
+      <c r="I18" s="2">
+        <v>192</v>
+      </c>
+      <c r="J18" s="2">
+        <v>208</v>
+      </c>
+      <c r="K18" s="2">
+        <v>188</v>
+      </c>
+      <c r="L18" s="2">
+        <v>218</v>
+      </c>
       <c r="M18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="N18" s="4">
-        <f>SUM(I18:L18)</f>
-        <v>0</v>
-      </c>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
+        <f t="shared" si="1"/>
+        <v>806</v>
+      </c>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
       <c r="S18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="T18" s="4">
-        <f>SUM(O18:R18)</f>
-        <v>0</v>
-      </c>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
+      <c r="X18" s="2"/>
       <c r="Y18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="Z18" s="4">
-        <f>SUM(U18:X18)</f>
-        <v>0</v>
-      </c>
-      <c r="AA18" s="3"/>
-      <c r="AB18" s="3"/>
-      <c r="AC18" s="3"/>
-      <c r="AD18" s="3"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA18" s="2"/>
+      <c r="AB18" s="2"/>
+      <c r="AC18" s="2"/>
+      <c r="AD18" s="2"/>
       <c r="AE18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="AF18" s="4">
-        <f>SUM(AA18:AD18)</f>
-        <v>0</v>
-      </c>
-      <c r="AG18" s="3"/>
-      <c r="AH18" s="3"/>
-      <c r="AI18" s="3"/>
-      <c r="AJ18" s="3"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG18" s="2"/>
+      <c r="AH18" s="2"/>
+      <c r="AI18" s="2"/>
+      <c r="AJ18" s="2"/>
       <c r="AK18" s="9">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="AL18" s="4">
-        <f>SUM(AG18:AJ18)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM18" s="6" cm="1">
         <f t="array" ref="AM18">SUM(C18:F18+I18:L18+O18:R18+U18:X18+AA18:AD18+AG18:AJ18)</f>
-        <v>721</v>
+        <v>1463</v>
       </c>
       <c r="AN18" s="8">
-        <f>SUM(H18+N18+T18+Z18+AF18+AL18)</f>
-        <v>737</v>
+        <f t="shared" si="6"/>
+        <v>1499</v>
       </c>
       <c r="AO18">
         <v>200</v>
       </c>
       <c r="AP18" s="11">
-        <v>194.7</v>
+        <v>187.48</v>
       </c>
       <c r="AQ18" s="11">
-        <f>SUM((AO18-AP18)*0.7)</f>
-        <v>3.7100000000000075</v>
+        <f t="shared" si="7"/>
+        <v>8.7640000000000065</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -2541,99 +2685,107 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="2">
-        <v>151</v>
-      </c>
-      <c r="D19" s="2">
-        <v>182</v>
-      </c>
-      <c r="E19" s="2">
-        <v>177</v>
-      </c>
-      <c r="F19" s="2">
-        <v>147</v>
+        <v>22</v>
+      </c>
+      <c r="C19" s="3">
+        <v>183</v>
+      </c>
+      <c r="D19" s="3">
+        <v>174</v>
+      </c>
+      <c r="E19" s="3">
+        <v>207</v>
+      </c>
+      <c r="F19" s="3">
+        <v>216</v>
       </c>
       <c r="G19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="H19" s="4">
-        <f>SUM(C19:G19)</f>
-        <v>693</v>
-      </c>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="I19" s="3">
+        <v>174</v>
+      </c>
+      <c r="J19" s="3">
+        <v>190</v>
+      </c>
+      <c r="K19" s="3">
+        <v>146</v>
+      </c>
+      <c r="L19" s="3">
+        <v>136</v>
+      </c>
       <c r="M19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="N19" s="4">
-        <f>SUM(I19:L19)</f>
-        <v>0</v>
-      </c>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
+        <f t="shared" si="1"/>
+        <v>646</v>
+      </c>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="3"/>
       <c r="S19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="T19" s="4">
-        <f>SUM(O19:R19)</f>
-        <v>0</v>
-      </c>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
-      <c r="X19" s="2"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
       <c r="Y19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="Z19" s="4">
-        <f>SUM(U19:X19)</f>
-        <v>0</v>
-      </c>
-      <c r="AA19" s="2"/>
-      <c r="AB19" s="2"/>
-      <c r="AC19" s="2"/>
-      <c r="AD19" s="2"/>
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AA19" s="3"/>
+      <c r="AB19" s="3"/>
+      <c r="AC19" s="3"/>
+      <c r="AD19" s="3"/>
       <c r="AE19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="AF19" s="4">
-        <f>SUM(AA19:AD19)</f>
-        <v>0</v>
-      </c>
-      <c r="AG19" s="2"/>
-      <c r="AH19" s="2"/>
-      <c r="AI19" s="2"/>
-      <c r="AJ19" s="2"/>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AG19" s="3"/>
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="3"/>
+      <c r="AJ19" s="3"/>
       <c r="AK19" s="9">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="AL19" s="4">
-        <f>SUM(AG19:AJ19)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM19" s="6" cm="1">
         <f t="array" ref="AM19">SUM(C19:F19+I19:L19+O19:R19+U19:X19+AA19:AD19+AG19:AJ19)</f>
-        <v>657</v>
+        <v>1426</v>
       </c>
       <c r="AN19" s="8">
-        <f>SUM(H19+N19+T19+Z19+AF19+AL19)</f>
-        <v>693</v>
+        <f t="shared" si="6"/>
+        <v>1446</v>
       </c>
       <c r="AO19">
         <v>200</v>
       </c>
       <c r="AP19" s="11">
-        <v>187.47</v>
+        <v>192.5</v>
       </c>
       <c r="AQ19" s="11">
-        <f>SUM((AO19-AP19)*0.7)</f>
-        <v>8.7710000000000008</v>
+        <f t="shared" si="7"/>
+        <v>5.25</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -2651,7 +2803,7 @@
         <v>84</v>
       </c>
       <c r="H20" s="4">
-        <f>SUM(C20:G20)</f>
+        <f t="shared" si="0"/>
         <v>84</v>
       </c>
       <c r="I20" s="2"/>
@@ -2662,7 +2814,7 @@
         <v>84</v>
       </c>
       <c r="N20" s="4">
-        <f>SUM(I20:L20)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O20" s="2"/>
@@ -2673,7 +2825,7 @@
         <v>84</v>
       </c>
       <c r="T20" s="4">
-        <f>SUM(O20:R20)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U20" s="2"/>
@@ -2684,7 +2836,7 @@
         <v>84</v>
       </c>
       <c r="Z20" s="4">
-        <f>SUM(U20:X20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA20" s="2"/>
@@ -2695,7 +2847,7 @@
         <v>84</v>
       </c>
       <c r="AF20" s="4">
-        <f>SUM(AA20:AD20)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG20" s="2"/>
@@ -2706,7 +2858,7 @@
         <v>84</v>
       </c>
       <c r="AL20" s="4">
-        <f>SUM(AG20:AJ20)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM20" s="6" cm="1">
@@ -2714,7 +2866,7 @@
         <v>0</v>
       </c>
       <c r="AN20" s="8">
-        <f>SUM(H20+N20+T20+Z20+AF20+AL20)</f>
+        <f t="shared" si="6"/>
         <v>84</v>
       </c>
       <c r="AO20">
@@ -2724,7 +2876,7 @@
         <v>169.88</v>
       </c>
       <c r="AQ20" s="11">
-        <f>SUM((AO20-AP20)*0.7)</f>
+        <f t="shared" si="7"/>
         <v>21.084000000000003</v>
       </c>
     </row>
@@ -2743,7 +2895,7 @@
         <v>68</v>
       </c>
       <c r="H21" s="4">
-        <f>SUM(C21:G21)</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="I21" s="2"/>
@@ -2754,7 +2906,7 @@
         <v>68</v>
       </c>
       <c r="N21" s="4">
-        <f>SUM(I21:L21)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O21" s="2"/>
@@ -2765,7 +2917,7 @@
         <v>68</v>
       </c>
       <c r="T21" s="4">
-        <f>SUM(O21:R21)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U21" s="2"/>
@@ -2776,7 +2928,7 @@
         <v>68</v>
       </c>
       <c r="Z21" s="4">
-        <f>SUM(U21:X21)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA21" s="2"/>
@@ -2787,7 +2939,7 @@
         <v>68</v>
       </c>
       <c r="AF21" s="4">
-        <f>SUM(AA21:AD21)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG21" s="2"/>
@@ -2798,7 +2950,7 @@
         <v>68</v>
       </c>
       <c r="AL21" s="4">
-        <f>SUM(AG21:AJ21)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM21" s="6" cm="1">
@@ -2806,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="AN21" s="8">
-        <f>SUM(H21+N21+T21+Z21+AF21+AL21)</f>
+        <f t="shared" si="6"/>
         <v>68</v>
       </c>
       <c r="AO21">
@@ -2816,7 +2968,7 @@
         <v>175.36</v>
       </c>
       <c r="AQ21" s="11">
-        <f>SUM((AO21-AP21)*0.7)</f>
+        <f t="shared" si="7"/>
         <v>17.24799999999999</v>
       </c>
     </row>
@@ -2832,21 +2984,21 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="H22" s="4">
-        <f>SUM(C22:G22)</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>28</v>
       </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="N22" s="4">
-        <f>SUM(I22:L22)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O22" s="3"/>
@@ -2854,10 +3006,10 @@
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
       <c r="S22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="T22" s="4">
-        <f>SUM(O22:R22)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U22" s="3"/>
@@ -2865,10 +3017,10 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
       <c r="Y22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="Z22" s="4">
-        <f>SUM(U22:X22)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA22" s="3"/>
@@ -2876,10 +3028,10 @@
       <c r="AC22" s="3"/>
       <c r="AD22" s="3"/>
       <c r="AE22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="AF22" s="4">
-        <f>SUM(AA22:AD22)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG22" s="3"/>
@@ -2887,10 +3039,10 @@
       <c r="AI22" s="3"/>
       <c r="AJ22" s="3"/>
       <c r="AK22" s="9">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="AL22" s="4">
-        <f>SUM(AG22:AJ22)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AM22" s="6" cm="1">
@@ -2898,18 +3050,18 @@
         <v>0</v>
       </c>
       <c r="AN22" s="8">
-        <f>SUM(H22+N22+T22+Z22+AF22+AL22)</f>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>28</v>
       </c>
       <c r="AO22">
         <v>200</v>
       </c>
       <c r="AP22" s="11">
-        <v>202.46</v>
+        <v>190.61</v>
       </c>
       <c r="AQ22" s="11">
-        <f>SUM((AO22-AP22)*0.7)</f>
-        <v>-1.7220000000000055</v>
+        <f t="shared" si="7"/>
+        <v>6.5729999999999897</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -2920,7 +3072,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="9"/>
       <c r="H23" s="4">
-        <f t="shared" ref="H23:H34" si="0">SUM(C23:G23)</f>
+        <f t="shared" ref="H23:H34" si="8">SUM(C23:G23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="2"/>
@@ -2929,7 +3081,7 @@
       <c r="L23" s="2"/>
       <c r="M23" s="9"/>
       <c r="N23" s="4">
-        <f t="shared" ref="N23:N34" si="1">SUM(I23:L23)</f>
+        <f t="shared" ref="N23:N34" si="9">SUM(I23:L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="2"/>
@@ -2938,7 +3090,7 @@
       <c r="R23" s="2"/>
       <c r="S23" s="9"/>
       <c r="T23" s="4">
-        <f t="shared" ref="T23:T34" si="2">SUM(O23:R23)</f>
+        <f t="shared" ref="T23:T34" si="10">SUM(O23:R23)</f>
         <v>0</v>
       </c>
       <c r="U23" s="2"/>
@@ -2947,7 +3099,7 @@
       <c r="X23" s="2"/>
       <c r="Y23" s="9"/>
       <c r="Z23" s="4">
-        <f t="shared" ref="Z23:Z34" si="3">SUM(U23:X23)</f>
+        <f t="shared" ref="Z23:Z34" si="11">SUM(U23:X23)</f>
         <v>0</v>
       </c>
       <c r="AA23" s="2"/>
@@ -2956,7 +3108,7 @@
       <c r="AD23" s="2"/>
       <c r="AE23" s="9"/>
       <c r="AF23" s="4">
-        <f t="shared" ref="AF23:AF34" si="4">SUM(AA23:AD23)</f>
+        <f t="shared" ref="AF23:AF34" si="12">SUM(AA23:AD23)</f>
         <v>0</v>
       </c>
       <c r="AG23" s="2"/>
@@ -2965,7 +3117,7 @@
       <c r="AJ23" s="2"/>
       <c r="AK23" s="9"/>
       <c r="AL23" s="4">
-        <f t="shared" ref="AL23:AL34" si="5">SUM(AG23:AJ23)</f>
+        <f t="shared" ref="AL23:AL34" si="13">SUM(AG23:AJ23)</f>
         <v>0</v>
       </c>
       <c r="AM23" s="6" cm="1">
@@ -2973,7 +3125,7 @@
         <v>0</v>
       </c>
       <c r="AN23" s="8">
-        <f t="shared" ref="AN23:AN34" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
+        <f t="shared" ref="AN23:AN34" si="14">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
         <v>0</v>
       </c>
       <c r="AO23">
@@ -2981,7 +3133,7 @@
       </c>
       <c r="AP23" s="11"/>
       <c r="AQ23" s="11">
-        <f t="shared" ref="AQ23:AQ34" si="7">SUM((AO23-AP23)*0.7)</f>
+        <f t="shared" ref="AQ23:AQ34" si="15">SUM((AO23-AP23)*0.7)</f>
         <v>140</v>
       </c>
     </row>
@@ -2993,7 +3145,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="9"/>
       <c r="H24" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I24" s="2"/>
@@ -3002,7 +3154,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="9"/>
       <c r="N24" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O24" s="2"/>
@@ -3011,7 +3163,7 @@
       <c r="R24" s="2"/>
       <c r="S24" s="9"/>
       <c r="T24" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U24" s="2"/>
@@ -3020,7 +3172,7 @@
       <c r="X24" s="2"/>
       <c r="Y24" s="9"/>
       <c r="Z24" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA24" s="2"/>
@@ -3029,7 +3181,7 @@
       <c r="AD24" s="2"/>
       <c r="AE24" s="9"/>
       <c r="AF24" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG24" s="2"/>
@@ -3038,7 +3190,7 @@
       <c r="AJ24" s="2"/>
       <c r="AK24" s="9"/>
       <c r="AL24" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM24" s="6" cm="1">
@@ -3046,7 +3198,7 @@
         <v>0</v>
       </c>
       <c r="AN24" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO24">
@@ -3054,7 +3206,7 @@
       </c>
       <c r="AP24" s="11"/>
       <c r="AQ24" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3066,7 +3218,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="9"/>
       <c r="H25" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I25" s="2"/>
@@ -3075,7 +3227,7 @@
       <c r="L25" s="2"/>
       <c r="M25" s="9"/>
       <c r="N25" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O25" s="2"/>
@@ -3084,7 +3236,7 @@
       <c r="R25" s="2"/>
       <c r="S25" s="9"/>
       <c r="T25" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U25" s="2"/>
@@ -3093,7 +3245,7 @@
       <c r="X25" s="2"/>
       <c r="Y25" s="9"/>
       <c r="Z25" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA25" s="2"/>
@@ -3102,7 +3254,7 @@
       <c r="AD25" s="2"/>
       <c r="AE25" s="9"/>
       <c r="AF25" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG25" s="2"/>
@@ -3111,7 +3263,7 @@
       <c r="AJ25" s="2"/>
       <c r="AK25" s="9"/>
       <c r="AL25" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM25" s="6" cm="1">
@@ -3119,7 +3271,7 @@
         <v>0</v>
       </c>
       <c r="AN25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO25">
@@ -3127,7 +3279,7 @@
       </c>
       <c r="AP25" s="11"/>
       <c r="AQ25" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3139,7 +3291,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="9"/>
       <c r="H26" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I26" s="2"/>
@@ -3148,7 +3300,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="9"/>
       <c r="N26" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O26" s="2"/>
@@ -3157,7 +3309,7 @@
       <c r="R26" s="2"/>
       <c r="S26" s="9"/>
       <c r="T26" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U26" s="2"/>
@@ -3166,7 +3318,7 @@
       <c r="X26" s="2"/>
       <c r="Y26" s="9"/>
       <c r="Z26" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA26" s="2"/>
@@ -3175,7 +3327,7 @@
       <c r="AD26" s="2"/>
       <c r="AE26" s="9"/>
       <c r="AF26" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG26" s="2"/>
@@ -3184,7 +3336,7 @@
       <c r="AJ26" s="2"/>
       <c r="AK26" s="9"/>
       <c r="AL26" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM26" s="6" cm="1">
@@ -3192,7 +3344,7 @@
         <v>0</v>
       </c>
       <c r="AN26" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO26">
@@ -3200,7 +3352,7 @@
       </c>
       <c r="AP26" s="11"/>
       <c r="AQ26" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3212,7 +3364,7 @@
       <c r="F27" s="2"/>
       <c r="G27" s="9"/>
       <c r="H27" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I27" s="2"/>
@@ -3221,7 +3373,7 @@
       <c r="L27" s="2"/>
       <c r="M27" s="9"/>
       <c r="N27" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O27" s="2"/>
@@ -3230,7 +3382,7 @@
       <c r="R27" s="2"/>
       <c r="S27" s="9"/>
       <c r="T27" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U27" s="2"/>
@@ -3239,7 +3391,7 @@
       <c r="X27" s="2"/>
       <c r="Y27" s="9"/>
       <c r="Z27" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA27" s="2"/>
@@ -3248,7 +3400,7 @@
       <c r="AD27" s="2"/>
       <c r="AE27" s="9"/>
       <c r="AF27" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG27" s="2"/>
@@ -3257,7 +3409,7 @@
       <c r="AJ27" s="2"/>
       <c r="AK27" s="9"/>
       <c r="AL27" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM27" s="6" cm="1">
@@ -3265,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="AN27" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO27">
@@ -3273,7 +3425,7 @@
       </c>
       <c r="AP27" s="11"/>
       <c r="AQ27" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3285,7 +3437,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="9"/>
       <c r="H28" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I28" s="2"/>
@@ -3294,7 +3446,7 @@
       <c r="L28" s="2"/>
       <c r="M28" s="9"/>
       <c r="N28" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O28" s="2"/>
@@ -3303,7 +3455,7 @@
       <c r="R28" s="2"/>
       <c r="S28" s="9"/>
       <c r="T28" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U28" s="2"/>
@@ -3312,7 +3464,7 @@
       <c r="X28" s="2"/>
       <c r="Y28" s="9"/>
       <c r="Z28" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA28" s="2"/>
@@ -3321,7 +3473,7 @@
       <c r="AD28" s="2"/>
       <c r="AE28" s="9"/>
       <c r="AF28" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG28" s="2"/>
@@ -3330,7 +3482,7 @@
       <c r="AJ28" s="2"/>
       <c r="AK28" s="9"/>
       <c r="AL28" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM28" s="6" cm="1">
@@ -3338,7 +3490,7 @@
         <v>0</v>
       </c>
       <c r="AN28" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO28">
@@ -3346,7 +3498,7 @@
       </c>
       <c r="AP28" s="11"/>
       <c r="AQ28" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3358,7 +3510,7 @@
       <c r="F29" s="2"/>
       <c r="G29" s="9"/>
       <c r="H29" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I29" s="2"/>
@@ -3367,7 +3519,7 @@
       <c r="L29" s="2"/>
       <c r="M29" s="9"/>
       <c r="N29" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O29" s="2"/>
@@ -3376,7 +3528,7 @@
       <c r="R29" s="2"/>
       <c r="S29" s="9"/>
       <c r="T29" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U29" s="2"/>
@@ -3385,7 +3537,7 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="9"/>
       <c r="Z29" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA29" s="2"/>
@@ -3394,7 +3546,7 @@
       <c r="AD29" s="2"/>
       <c r="AE29" s="9"/>
       <c r="AF29" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG29" s="2"/>
@@ -3403,7 +3555,7 @@
       <c r="AJ29" s="2"/>
       <c r="AK29" s="9"/>
       <c r="AL29" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM29" s="6" cm="1">
@@ -3411,7 +3563,7 @@
         <v>0</v>
       </c>
       <c r="AN29" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO29">
@@ -3419,7 +3571,7 @@
       </c>
       <c r="AP29" s="11"/>
       <c r="AQ29" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3431,7 +3583,7 @@
       <c r="F30" s="2"/>
       <c r="G30" s="9"/>
       <c r="H30" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I30" s="2"/>
@@ -3440,7 +3592,7 @@
       <c r="L30" s="2"/>
       <c r="M30" s="9"/>
       <c r="N30" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O30" s="2"/>
@@ -3449,7 +3601,7 @@
       <c r="R30" s="2"/>
       <c r="S30" s="9"/>
       <c r="T30" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U30" s="2"/>
@@ -3458,7 +3610,7 @@
       <c r="X30" s="2"/>
       <c r="Y30" s="9"/>
       <c r="Z30" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA30" s="2"/>
@@ -3467,7 +3619,7 @@
       <c r="AD30" s="2"/>
       <c r="AE30" s="9"/>
       <c r="AF30" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG30" s="2"/>
@@ -3476,7 +3628,7 @@
       <c r="AJ30" s="2"/>
       <c r="AK30" s="9"/>
       <c r="AL30" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM30" s="6" cm="1">
@@ -3484,7 +3636,7 @@
         <v>0</v>
       </c>
       <c r="AN30" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO30">
@@ -3492,7 +3644,7 @@
       </c>
       <c r="AP30" s="11"/>
       <c r="AQ30" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3504,7 +3656,7 @@
       <c r="F31" s="2"/>
       <c r="G31" s="9"/>
       <c r="H31" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I31" s="2"/>
@@ -3513,7 +3665,7 @@
       <c r="L31" s="2"/>
       <c r="M31" s="9"/>
       <c r="N31" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O31" s="2"/>
@@ -3522,7 +3674,7 @@
       <c r="R31" s="2"/>
       <c r="S31" s="9"/>
       <c r="T31" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U31" s="2"/>
@@ -3531,7 +3683,7 @@
       <c r="X31" s="2"/>
       <c r="Y31" s="9"/>
       <c r="Z31" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA31" s="2"/>
@@ -3540,7 +3692,7 @@
       <c r="AD31" s="2"/>
       <c r="AE31" s="9"/>
       <c r="AF31" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG31" s="2"/>
@@ -3549,7 +3701,7 @@
       <c r="AJ31" s="2"/>
       <c r="AK31" s="9"/>
       <c r="AL31" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM31" s="6" cm="1">
@@ -3557,7 +3709,7 @@
         <v>0</v>
       </c>
       <c r="AN31" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO31">
@@ -3565,7 +3717,7 @@
       </c>
       <c r="AP31" s="11"/>
       <c r="AQ31" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3577,7 +3729,7 @@
       <c r="F32" s="2"/>
       <c r="G32" s="9"/>
       <c r="H32" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I32" s="2"/>
@@ -3586,7 +3738,7 @@
       <c r="L32" s="2"/>
       <c r="M32" s="9"/>
       <c r="N32" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O32" s="2"/>
@@ -3595,7 +3747,7 @@
       <c r="R32" s="2"/>
       <c r="S32" s="9"/>
       <c r="T32" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U32" s="2"/>
@@ -3604,7 +3756,7 @@
       <c r="X32" s="2"/>
       <c r="Y32" s="9"/>
       <c r="Z32" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA32" s="2"/>
@@ -3613,7 +3765,7 @@
       <c r="AD32" s="2"/>
       <c r="AE32" s="9"/>
       <c r="AF32" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG32" s="2"/>
@@ -3622,7 +3774,7 @@
       <c r="AJ32" s="2"/>
       <c r="AK32" s="9"/>
       <c r="AL32" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM32" s="6" cm="1">
@@ -3630,7 +3782,7 @@
         <v>0</v>
       </c>
       <c r="AN32" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO32">
@@ -3638,7 +3790,7 @@
       </c>
       <c r="AP32" s="11"/>
       <c r="AQ32" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3650,7 +3802,7 @@
       <c r="F33" s="2"/>
       <c r="G33" s="9"/>
       <c r="H33" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I33" s="2"/>
@@ -3659,7 +3811,7 @@
       <c r="L33" s="2"/>
       <c r="M33" s="9"/>
       <c r="N33" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O33" s="2"/>
@@ -3668,7 +3820,7 @@
       <c r="R33" s="2"/>
       <c r="S33" s="9"/>
       <c r="T33" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U33" s="2"/>
@@ -3677,7 +3829,7 @@
       <c r="X33" s="2"/>
       <c r="Y33" s="9"/>
       <c r="Z33" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA33" s="2"/>
@@ -3686,7 +3838,7 @@
       <c r="AD33" s="2"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG33" s="2"/>
@@ -3695,7 +3847,7 @@
       <c r="AJ33" s="2"/>
       <c r="AK33" s="9"/>
       <c r="AL33" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM33" s="6" cm="1">
@@ -3703,7 +3855,7 @@
         <v>0</v>
       </c>
       <c r="AN33" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO33">
@@ -3711,7 +3863,7 @@
       </c>
       <c r="AP33" s="11"/>
       <c r="AQ33" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3723,7 +3875,7 @@
       <c r="F34" s="2"/>
       <c r="G34" s="9"/>
       <c r="H34" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I34" s="2"/>
@@ -3732,7 +3884,7 @@
       <c r="L34" s="2"/>
       <c r="M34" s="9"/>
       <c r="N34" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O34" s="2"/>
@@ -3741,7 +3893,7 @@
       <c r="R34" s="2"/>
       <c r="S34" s="9"/>
       <c r="T34" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U34" s="2"/>
@@ -3750,7 +3902,7 @@
       <c r="X34" s="2"/>
       <c r="Y34" s="9"/>
       <c r="Z34" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA34" s="2"/>
@@ -3759,7 +3911,7 @@
       <c r="AD34" s="2"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG34" s="2"/>
@@ -3768,7 +3920,7 @@
       <c r="AJ34" s="2"/>
       <c r="AK34" s="9"/>
       <c r="AL34" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM34" s="6" cm="1">
@@ -3776,7 +3928,7 @@
         <v>0</v>
       </c>
       <c r="AN34" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO34">
@@ -3784,12 +3936,12 @@
       </c>
       <c r="AP34" s="11"/>
       <c r="AQ34" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:AQ22">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:AN22">
     <sortCondition descending="1" ref="AN3:AN22"/>
   </sortState>
   <mergeCells count="7">

</xml_diff>

<commit_message>
data(tournament): added finals results of Donaubowler CM, extended frontend for sophisitcated 3 format finals
</commit_message>
<xml_diff>
--- a/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
+++ b/database/input/clubmeisterschaft_donaubowler/Clubpokal DB 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco\Dropbox\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED3AA194-3CB4-4BC4-A2C9-338D015EAFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D04B15-C3DF-41E7-906B-49FAE77A843B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D7BAE6BD-B2A4-4DD1-AF79-906BD29E778A}"/>
   </bookViews>
@@ -148,7 +148,7 @@
     <t>Richard Zorzi</t>
   </si>
   <si>
-    <t>Donaubowler Clubmeisterschaft 2026 / Stand 18.06.26</t>
+    <t>Donaubowler Clubmeisterschaft 2026 / Stand 09.07.26</t>
   </si>
 </sst>
 </file>
@@ -759,139 +759,139 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="D3" s="3">
-        <v>193</v>
+        <v>227</v>
       </c>
       <c r="E3" s="3">
         <v>205</v>
       </c>
       <c r="F3" s="3">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="G3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H3" s="4">
         <f>SUM(C3:G3)</f>
-        <v>815</v>
+        <v>843</v>
       </c>
       <c r="I3" s="3">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="J3" s="3">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="K3" s="3">
+        <v>183</v>
+      </c>
+      <c r="L3" s="3">
         <v>224</v>
       </c>
-      <c r="L3" s="3">
-        <v>189</v>
-      </c>
       <c r="M3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="N3" s="4">
         <f>SUM(I3:L3)</f>
-        <v>880</v>
+        <v>830</v>
       </c>
       <c r="O3" s="3">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="P3" s="3">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="Q3" s="3">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="R3" s="3">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="S3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="T3" s="4">
         <f>SUM(O3:R3)</f>
-        <v>881</v>
+        <v>875</v>
       </c>
       <c r="U3" s="3">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="V3" s="3">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="W3" s="3">
-        <v>228</v>
+        <v>193</v>
       </c>
       <c r="X3" s="3">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="Y3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Z3" s="4">
         <f>SUM(U3:X3)</f>
-        <v>865</v>
+        <v>776</v>
       </c>
       <c r="AA3" s="3">
-        <v>166</v>
+        <v>229</v>
       </c>
       <c r="AB3" s="3">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="AC3" s="3">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="AD3" s="3">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="AE3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AF3" s="4">
         <f>SUM(AA3:AD3)</f>
-        <v>657</v>
+        <v>820</v>
       </c>
       <c r="AG3" s="3">
-        <v>243</v>
+        <v>197</v>
       </c>
       <c r="AH3" s="3">
-        <v>248</v>
+        <v>202</v>
       </c>
       <c r="AI3" s="3">
-        <v>193</v>
+        <v>247</v>
       </c>
       <c r="AJ3" s="3">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AK3" s="9">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AL3" s="4">
         <f>SUM(AG3:AJ3)</f>
-        <v>890</v>
+        <v>850</v>
       </c>
       <c r="AM3" s="6" cm="1">
         <f t="array" ref="AM3">SUM(C3:F3+I3:L3+O3:R3+U3:X3+AA3:AD3+AG3:AJ3)</f>
-        <v>4968</v>
+        <v>4978</v>
       </c>
       <c r="AN3" s="8">
         <f>SUM(H3+N3+T3+Z3+AF3+AL3)</f>
-        <v>4988</v>
+        <v>4994</v>
       </c>
       <c r="AO3">
         <v>200</v>
       </c>
       <c r="AP3" s="11">
-        <v>193.33</v>
+        <v>193.83</v>
       </c>
       <c r="AQ3" s="11">
         <f>SUM((AO3-AP3)*0.7)</f>
-        <v>4.6689999999999907</v>
+        <v>4.3189999999999911</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -899,139 +899,139 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C4" s="3">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="D4" s="3">
-        <v>239</v>
+        <v>193</v>
       </c>
       <c r="E4" s="3">
-        <v>224</v>
+        <v>205</v>
       </c>
       <c r="F4" s="3">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H4" s="4">
         <f>SUM(C4:G4)</f>
-        <v>888</v>
+        <v>815</v>
       </c>
       <c r="I4" s="3">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="J4" s="3">
-        <v>194</v>
+        <v>242</v>
       </c>
       <c r="K4" s="3">
-        <v>190</v>
+        <v>224</v>
       </c>
       <c r="L4" s="3">
-        <v>216</v>
+        <v>189</v>
       </c>
       <c r="M4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N4" s="4">
         <f>SUM(I4:L4)</f>
-        <v>845</v>
+        <v>880</v>
       </c>
       <c r="O4" s="3">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="P4" s="3">
-        <v>179</v>
+        <v>218</v>
       </c>
       <c r="Q4" s="3">
-        <v>217</v>
+        <v>204</v>
       </c>
       <c r="R4" s="3">
-        <v>192</v>
+        <v>233</v>
       </c>
       <c r="S4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="T4" s="4">
         <f>SUM(O4:R4)</f>
-        <v>803</v>
+        <v>881</v>
       </c>
       <c r="U4" s="3">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="V4" s="3">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="W4" s="3">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="X4" s="3">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="Y4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="Z4" s="4">
         <f>SUM(U4:X4)</f>
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="AA4" s="3">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="AB4" s="3">
-        <v>191</v>
+        <v>172</v>
       </c>
       <c r="AC4" s="3">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="AD4" s="3">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="AE4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AF4" s="4">
         <f>SUM(AA4:AD4)</f>
-        <v>759</v>
+        <v>657</v>
       </c>
       <c r="AG4" s="3">
-        <v>180</v>
+        <v>243</v>
       </c>
       <c r="AH4" s="3">
-        <v>166</v>
+        <v>248</v>
       </c>
       <c r="AI4" s="3">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="AJ4" s="3">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="AK4" s="9">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AL4" s="4">
         <f>SUM(AG4:AJ4)</f>
-        <v>760</v>
+        <v>890</v>
       </c>
       <c r="AM4" s="6" cm="1">
         <f t="array" ref="AM4">SUM(C4:F4+I4:L4+O4:R4+U4:X4+AA4:AD4+AG4:AJ4)</f>
-        <v>4905</v>
+        <v>4968</v>
       </c>
       <c r="AN4" s="8">
         <f>SUM(H4+N4+T4+Z4+AF4+AL4)</f>
-        <v>4905</v>
+        <v>4988</v>
       </c>
       <c r="AO4">
         <v>200</v>
       </c>
       <c r="AP4" s="11">
-        <v>200</v>
+        <v>193.33</v>
       </c>
       <c r="AQ4" s="11">
         <f>SUM((AO4-AP4)*0.7)</f>
-        <v>0</v>
+        <v>4.6689999999999907</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -1039,139 +1039,139 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D5" s="3">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="E5" s="3">
-        <v>154</v>
+        <v>134</v>
       </c>
       <c r="F5" s="3">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="G5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="H5" s="4">
         <f>SUM(C5:G5)</f>
-        <v>746</v>
+        <v>737</v>
       </c>
       <c r="I5" s="3">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="J5" s="3">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="K5" s="3">
-        <v>132</v>
+        <v>220</v>
       </c>
       <c r="L5" s="3">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="M5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="N5" s="4">
         <f>SUM(I5:L5)</f>
-        <v>657</v>
+        <v>813</v>
       </c>
       <c r="O5" s="3">
-        <v>179</v>
+        <v>222</v>
       </c>
       <c r="P5" s="3">
-        <v>173</v>
+        <v>227</v>
       </c>
       <c r="Q5" s="3">
-        <v>169</v>
+        <v>228</v>
       </c>
       <c r="R5" s="3">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="S5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="T5" s="4">
         <f>SUM(O5:R5)</f>
-        <v>677</v>
+        <v>878</v>
       </c>
       <c r="U5" s="3">
-        <v>191</v>
+        <v>226</v>
       </c>
       <c r="V5" s="3">
-        <v>173</v>
+        <v>208</v>
       </c>
       <c r="W5" s="3">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="X5" s="3">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="Y5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="Z5" s="4">
         <f>SUM(U5:X5)</f>
-        <v>746</v>
+        <v>863</v>
       </c>
       <c r="AA5" s="3">
-        <v>155</v>
+        <v>247</v>
       </c>
       <c r="AB5" s="3">
-        <v>200</v>
+        <v>238</v>
       </c>
       <c r="AC5" s="3">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="AD5" s="3">
-        <v>176</v>
+        <v>216</v>
       </c>
       <c r="AE5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="AF5" s="4">
         <f>SUM(AA5:AD5)</f>
-        <v>712</v>
+        <v>896</v>
       </c>
       <c r="AG5" s="3">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="AH5" s="3">
-        <v>136</v>
+        <v>188</v>
       </c>
       <c r="AI5" s="3">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="AJ5" s="3">
-        <v>226</v>
+        <v>183</v>
       </c>
       <c r="AK5" s="9">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="AL5" s="4">
         <f>SUM(AG5:AJ5)</f>
-        <v>705</v>
+        <v>768</v>
       </c>
       <c r="AM5" s="6" cm="1">
         <f t="array" ref="AM5">SUM(C5:F5+I5:L5+O5:R5+U5:X5+AA5:AD5+AG5:AJ5)</f>
-        <v>4159</v>
+        <v>4939</v>
       </c>
       <c r="AN5" s="8">
         <f>SUM(H5+N5+T5+Z5+AF5+AL5)</f>
-        <v>4243</v>
+        <v>4955</v>
       </c>
       <c r="AO5">
         <v>200</v>
       </c>
       <c r="AP5" s="11">
-        <v>169.44</v>
+        <v>194.71</v>
       </c>
       <c r="AQ5" s="11">
         <f>SUM((AO5-AP5)*0.7)</f>
-        <v>21.391999999999999</v>
+        <v>3.7029999999999941</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -1179,139 +1179,139 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D6" s="3">
-        <v>214</v>
+        <v>239</v>
       </c>
       <c r="E6" s="3">
-        <v>167</v>
+        <v>224</v>
       </c>
       <c r="F6" s="3">
-        <v>171</v>
+        <v>209</v>
       </c>
       <c r="G6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4">
         <f>SUM(C6:G6)</f>
-        <v>823</v>
+        <v>888</v>
       </c>
       <c r="I6" s="3">
-        <v>179</v>
+        <v>245</v>
       </c>
       <c r="J6" s="3">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="K6" s="3">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="L6" s="3">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="M6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="N6" s="4">
         <f>SUM(I6:L6)</f>
-        <v>781</v>
+        <v>845</v>
       </c>
       <c r="O6" s="3">
-        <v>148</v>
+        <v>215</v>
       </c>
       <c r="P6" s="3">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="Q6" s="3">
-        <v>177</v>
+        <v>217</v>
       </c>
       <c r="R6" s="3">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="S6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="T6" s="4">
         <f>SUM(O6:R6)</f>
-        <v>656</v>
+        <v>803</v>
       </c>
       <c r="U6" s="3">
-        <v>148</v>
+        <v>214</v>
       </c>
       <c r="V6" s="3">
-        <v>156</v>
+        <v>227</v>
       </c>
       <c r="W6" s="3">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="X6" s="3">
-        <v>201</v>
+        <v>185</v>
       </c>
       <c r="Y6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="4">
         <f>SUM(U6:X6)</f>
-        <v>719</v>
+        <v>850</v>
       </c>
       <c r="AA6" s="3">
-        <v>123</v>
+        <v>181</v>
       </c>
       <c r="AB6" s="3">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="AC6" s="3">
-        <v>168</v>
+        <v>205</v>
       </c>
       <c r="AD6" s="3">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AE6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="4">
         <f>SUM(AA6:AD6)</f>
-        <v>675</v>
+        <v>759</v>
       </c>
       <c r="AG6" s="3">
-        <v>128</v>
+        <v>180</v>
       </c>
       <c r="AH6" s="3">
         <v>166</v>
       </c>
       <c r="AI6" s="3">
-        <v>160</v>
+        <v>201</v>
       </c>
       <c r="AJ6" s="3">
-        <v>117</v>
+        <v>213</v>
       </c>
       <c r="AK6" s="9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="AL6" s="4">
         <f>SUM(AG6:AJ6)</f>
-        <v>571</v>
+        <v>760</v>
       </c>
       <c r="AM6" s="6" cm="1">
         <f t="array" ref="AM6">SUM(C6:F6+I6:L6+O6:R6+U6:X6+AA6:AD6+AG6:AJ6)</f>
-        <v>4149</v>
+        <v>4905</v>
       </c>
       <c r="AN6" s="8">
         <f>SUM(H6+N6+T6+Z6+AF6+AL6)</f>
-        <v>4225</v>
+        <v>4905</v>
       </c>
       <c r="AO6">
         <v>200</v>
       </c>
       <c r="AP6" s="11">
-        <v>173.04</v>
+        <v>200</v>
       </c>
       <c r="AQ6" s="11">
         <f>SUM((AO6-AP6)*0.7)</f>
-        <v>18.872000000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -1319,131 +1319,139 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="C7" s="3">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="D7" s="3">
-        <v>227</v>
+        <v>190</v>
       </c>
       <c r="E7" s="3">
-        <v>205</v>
+        <v>188</v>
       </c>
       <c r="F7" s="3">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="G7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="H7" s="4">
         <f>SUM(C7:G7)</f>
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="I7" s="3">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="J7" s="3">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="K7" s="3">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="L7" s="3">
-        <v>224</v>
+        <v>185</v>
       </c>
       <c r="M7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="N7" s="4">
         <f>SUM(I7:L7)</f>
-        <v>830</v>
+        <v>817</v>
       </c>
       <c r="O7" s="3">
-        <v>214</v>
+        <v>194</v>
       </c>
       <c r="P7" s="3">
-        <v>203</v>
+        <v>148</v>
       </c>
       <c r="Q7" s="3">
-        <v>219</v>
+        <v>200</v>
       </c>
       <c r="R7" s="3">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="S7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="T7" s="4">
         <f>SUM(O7:R7)</f>
-        <v>875</v>
+        <v>801</v>
       </c>
       <c r="U7" s="3">
-        <v>204</v>
+        <v>170</v>
       </c>
       <c r="V7" s="3">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="W7" s="3">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="X7" s="3">
-        <v>176</v>
+        <v>202</v>
       </c>
       <c r="Y7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="Z7" s="4">
         <f>SUM(U7:X7)</f>
-        <v>776</v>
+        <v>788</v>
       </c>
       <c r="AA7" s="3">
-        <v>229</v>
+        <v>170</v>
       </c>
       <c r="AB7" s="3">
-        <v>212</v>
+        <v>257</v>
       </c>
       <c r="AC7" s="3">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="AD7" s="3">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="AE7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="AF7" s="4">
         <f>SUM(AA7:AD7)</f>
-        <v>820</v>
-      </c>
-      <c r="AG7" s="3"/>
-      <c r="AH7" s="3"/>
-      <c r="AI7" s="3"/>
-      <c r="AJ7" s="3"/>
+        <v>812</v>
+      </c>
+      <c r="AG7" s="3">
+        <v>191</v>
+      </c>
+      <c r="AH7" s="3">
+        <v>203</v>
+      </c>
+      <c r="AI7" s="3">
+        <v>145</v>
+      </c>
+      <c r="AJ7" s="3">
+        <v>193</v>
+      </c>
       <c r="AK7" s="9">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="AL7" s="4">
         <f>SUM(AG7:AJ7)</f>
-        <v>0</v>
+        <v>732</v>
       </c>
       <c r="AM7" s="6" cm="1">
         <f t="array" ref="AM7">SUM(C7:F7+I7:L7+O7:R7+U7:X7+AA7:AD7+AG7:AJ7)</f>
-        <v>4128</v>
+        <v>4750</v>
       </c>
       <c r="AN7" s="8">
         <f>SUM(H7+N7+T7+Z7+AF7+AL7)</f>
-        <v>4144</v>
+        <v>4790</v>
       </c>
       <c r="AO7">
         <v>200</v>
       </c>
       <c r="AP7" s="11">
-        <v>193.83</v>
+        <v>185.77</v>
       </c>
       <c r="AQ7" s="11">
         <f>SUM((AO7-AP7)*0.7)</f>
-        <v>4.3189999999999911</v>
+        <v>9.9609999999999914</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -1451,131 +1459,139 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C8" s="3">
-        <v>220</v>
+        <v>183</v>
       </c>
       <c r="D8" s="3">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="E8" s="3">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="F8" s="3">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="G8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H8" s="4">
         <f>SUM(C8:G8)</f>
-        <v>840</v>
+        <v>800</v>
       </c>
       <c r="I8" s="3">
-        <v>213</v>
+        <v>174</v>
       </c>
       <c r="J8" s="3">
-        <v>242</v>
+        <v>190</v>
       </c>
       <c r="K8" s="3">
-        <v>177</v>
+        <v>146</v>
       </c>
       <c r="L8" s="3">
-        <v>185</v>
+        <v>136</v>
       </c>
       <c r="M8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="N8" s="4">
         <f>SUM(I8:L8)</f>
-        <v>817</v>
+        <v>646</v>
       </c>
       <c r="O8" s="3">
-        <v>194</v>
+        <v>227</v>
       </c>
       <c r="P8" s="3">
-        <v>148</v>
+        <v>207</v>
       </c>
       <c r="Q8" s="3">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="R8" s="3">
-        <v>259</v>
+        <v>277</v>
       </c>
       <c r="S8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="T8" s="4">
         <f>SUM(O8:R8)</f>
-        <v>801</v>
+        <v>901</v>
       </c>
       <c r="U8" s="3">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="V8" s="3">
-        <v>225</v>
+        <v>178</v>
       </c>
       <c r="W8" s="3">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="X8" s="3">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="Z8" s="4">
         <f>SUM(U8:X8)</f>
-        <v>788</v>
+        <v>734</v>
       </c>
       <c r="AA8" s="3">
-        <v>170</v>
+        <v>202</v>
       </c>
       <c r="AB8" s="3">
-        <v>257</v>
+        <v>176</v>
       </c>
       <c r="AC8" s="3">
-        <v>191</v>
+        <v>149</v>
       </c>
       <c r="AD8" s="3">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="AE8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="AF8" s="4">
         <f>SUM(AA8:AD8)</f>
-        <v>812</v>
-      </c>
-      <c r="AG8" s="3"/>
-      <c r="AH8" s="3"/>
-      <c r="AI8" s="3"/>
-      <c r="AJ8" s="3"/>
+        <v>737</v>
+      </c>
+      <c r="AG8" s="3">
+        <v>203</v>
+      </c>
+      <c r="AH8" s="3">
+        <v>195</v>
+      </c>
+      <c r="AI8" s="3">
+        <v>178</v>
+      </c>
+      <c r="AJ8" s="3">
+        <v>174</v>
+      </c>
       <c r="AK8" s="9">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="AL8" s="4">
         <f>SUM(AG8:AJ8)</f>
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="AM8" s="6" cm="1">
         <f t="array" ref="AM8">SUM(C8:F8+I8:L8+O8:R8+U8:X8+AA8:AD8+AG8:AJ8)</f>
-        <v>4018</v>
+        <v>4548</v>
       </c>
       <c r="AN8" s="8">
         <f>SUM(H8+N8+T8+Z8+AF8+AL8)</f>
-        <v>4058</v>
+        <v>4568</v>
       </c>
       <c r="AO8">
         <v>200</v>
       </c>
       <c r="AP8" s="11">
-        <v>185.77</v>
+        <v>192.5</v>
       </c>
       <c r="AQ8" s="11">
         <f>SUM((AO8-AP8)*0.7)</f>
-        <v>9.9609999999999914</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -1583,131 +1599,139 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="D9" s="3">
+        <v>205</v>
+      </c>
+      <c r="E9" s="3">
         <v>192</v>
       </c>
-      <c r="E9" s="3">
-        <v>176</v>
-      </c>
       <c r="F9" s="3">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="G9" s="9">
         <v>44</v>
       </c>
       <c r="H9" s="4">
         <f>SUM(C9:G9)</f>
-        <v>857</v>
+        <v>825</v>
       </c>
       <c r="I9" s="3">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="J9" s="3">
-        <v>146</v>
+        <v>200</v>
       </c>
       <c r="K9" s="3">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="L9" s="3">
-        <v>178</v>
+        <v>147</v>
       </c>
       <c r="M9" s="9">
         <v>44</v>
       </c>
       <c r="N9" s="4">
         <f>SUM(I9:L9)</f>
-        <v>725</v>
+        <v>710</v>
       </c>
       <c r="O9" s="3">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="P9" s="3">
-        <v>181</v>
+        <v>149</v>
       </c>
       <c r="Q9" s="3">
-        <v>198</v>
+        <v>167</v>
       </c>
       <c r="R9" s="3">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="S9" s="9">
         <v>44</v>
       </c>
       <c r="T9" s="4">
         <f>SUM(O9:R9)</f>
-        <v>775</v>
+        <v>714</v>
       </c>
       <c r="U9" s="3">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="V9" s="3">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="W9" s="3">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="X9" s="3">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Y9" s="9">
         <v>44</v>
       </c>
       <c r="Z9" s="4">
         <f>SUM(U9:X9)</f>
-        <v>698</v>
+        <v>724</v>
       </c>
       <c r="AA9" s="3">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="AB9" s="3">
-        <v>223</v>
+        <v>173</v>
       </c>
       <c r="AC9" s="3">
-        <v>233</v>
+        <v>215</v>
       </c>
       <c r="AD9" s="3">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="AE9" s="9">
         <v>44</v>
       </c>
       <c r="AF9" s="4">
         <f>SUM(AA9:AD9)</f>
-        <v>807</v>
-      </c>
-      <c r="AG9" s="3"/>
-      <c r="AH9" s="3"/>
-      <c r="AI9" s="3"/>
-      <c r="AJ9" s="3"/>
+        <v>768</v>
+      </c>
+      <c r="AG9" s="3">
+        <v>190</v>
+      </c>
+      <c r="AH9" s="3">
+        <v>193</v>
+      </c>
+      <c r="AI9" s="3">
+        <v>208</v>
+      </c>
+      <c r="AJ9" s="3">
+        <v>194</v>
+      </c>
       <c r="AK9" s="9">
         <v>44</v>
       </c>
       <c r="AL9" s="4">
         <f>SUM(AG9:AJ9)</f>
-        <v>0</v>
+        <v>785</v>
       </c>
       <c r="AM9" s="6" cm="1">
         <f t="array" ref="AM9">SUM(C9:F9+I9:L9+O9:R9+U9:X9+AA9:AD9+AG9:AJ9)</f>
-        <v>3818</v>
+        <v>4482</v>
       </c>
       <c r="AN9" s="8">
         <f>SUM(H9+N9+T9+Z9+AF9+AL9)</f>
-        <v>3862</v>
+        <v>4526</v>
       </c>
       <c r="AO9">
         <v>200</v>
       </c>
       <c r="AP9" s="11">
-        <v>185</v>
+        <v>184.5</v>
       </c>
       <c r="AQ9" s="11">
         <f>SUM((AO9-AP9)*0.7)</f>
-        <v>10.5</v>
+        <v>10.85</v>
       </c>
     </row>
     <row r="10" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1715,131 +1739,139 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C10" s="3">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="D10" s="3">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="E10" s="3">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="F10" s="3">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="G10" s="9">
         <v>44</v>
       </c>
       <c r="H10" s="4">
         <f>SUM(C10:G10)</f>
-        <v>825</v>
+        <v>857</v>
       </c>
       <c r="I10" s="3">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="J10" s="3">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="K10" s="3">
-        <v>189</v>
+        <v>224</v>
       </c>
       <c r="L10" s="3">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="M10" s="9">
         <v>44</v>
       </c>
       <c r="N10" s="4">
         <f>SUM(I10:L10)</f>
-        <v>710</v>
+        <v>725</v>
       </c>
       <c r="O10" s="3">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="P10" s="3">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="Q10" s="3">
-        <v>167</v>
+        <v>198</v>
       </c>
       <c r="R10" s="3">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="S10" s="9">
         <v>44</v>
       </c>
       <c r="T10" s="4">
         <f>SUM(O10:R10)</f>
-        <v>714</v>
+        <v>775</v>
       </c>
       <c r="U10" s="3">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="V10" s="3">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="W10" s="3">
-        <v>191</v>
+        <v>156</v>
       </c>
       <c r="X10" s="3">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="Y10" s="9">
         <v>44</v>
       </c>
       <c r="Z10" s="4">
         <f>SUM(U10:X10)</f>
-        <v>724</v>
+        <v>698</v>
       </c>
       <c r="AA10" s="3">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="AB10" s="3">
-        <v>173</v>
+        <v>223</v>
       </c>
       <c r="AC10" s="3">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="AD10" s="3">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="AE10" s="9">
         <v>44</v>
       </c>
       <c r="AF10" s="4">
         <f>SUM(AA10:AD10)</f>
-        <v>768</v>
-      </c>
-      <c r="AG10" s="3"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
+        <v>807</v>
+      </c>
+      <c r="AG10" s="3">
+        <v>164</v>
+      </c>
+      <c r="AH10" s="3">
+        <v>160</v>
+      </c>
+      <c r="AI10" s="3">
+        <v>167</v>
+      </c>
+      <c r="AJ10" s="3">
+        <v>155</v>
+      </c>
       <c r="AK10" s="9">
         <v>44</v>
       </c>
       <c r="AL10" s="4">
         <f>SUM(AG10:AJ10)</f>
-        <v>0</v>
+        <v>646</v>
       </c>
       <c r="AM10" s="6" cm="1">
         <f t="array" ref="AM10">SUM(C10:F10+I10:L10+O10:R10+U10:X10+AA10:AD10+AG10:AJ10)</f>
-        <v>3697</v>
+        <v>4464</v>
       </c>
       <c r="AN10" s="8">
         <f>SUM(H10+N10+T10+Z10+AF10+AL10)</f>
-        <v>3741</v>
+        <v>4508</v>
       </c>
       <c r="AO10">
         <v>200</v>
       </c>
       <c r="AP10" s="11">
-        <v>184.5</v>
+        <v>185</v>
       </c>
       <c r="AQ10" s="11">
         <f>SUM((AO10-AP10)*0.7)</f>
-        <v>10.85</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -1847,131 +1879,139 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C11" s="3">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D11" s="3">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="E11" s="3">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="F11" s="3">
-        <v>192</v>
+        <v>136</v>
       </c>
       <c r="G11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="H11" s="4">
         <f>SUM(C11:G11)</f>
-        <v>801</v>
+        <v>714</v>
       </c>
       <c r="I11" s="3">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="J11" s="3">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="K11" s="3">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="L11" s="3">
-        <v>204</v>
+        <v>162</v>
       </c>
       <c r="M11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="N11" s="4">
         <f>SUM(I11:L11)</f>
-        <v>789</v>
+        <v>685</v>
       </c>
       <c r="O11" s="3">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="P11" s="3">
-        <v>142</v>
+        <v>174</v>
       </c>
       <c r="Q11" s="3">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="R11" s="3">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="S11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="T11" s="4">
         <f>SUM(O11:R11)</f>
-        <v>588</v>
+        <v>664</v>
       </c>
       <c r="U11" s="3">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="V11" s="3">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="W11" s="3">
-        <v>157</v>
+        <v>212</v>
       </c>
       <c r="X11" s="3">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="Y11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="Z11" s="4">
         <f>SUM(U11:X11)</f>
-        <v>727</v>
+        <v>740</v>
       </c>
       <c r="AA11" s="3">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="AB11" s="3">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="AC11" s="3">
-        <v>166</v>
+        <v>213</v>
       </c>
       <c r="AD11" s="3">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="AE11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="AF11" s="4">
         <f>SUM(AA11:AD11)</f>
-        <v>702</v>
-      </c>
-      <c r="AG11" s="3"/>
-      <c r="AH11" s="3"/>
-      <c r="AI11" s="3"/>
-      <c r="AJ11" s="3"/>
+        <v>798</v>
+      </c>
+      <c r="AG11" s="3">
+        <v>158</v>
+      </c>
+      <c r="AH11" s="3">
+        <v>165</v>
+      </c>
+      <c r="AI11" s="3">
+        <v>199</v>
+      </c>
+      <c r="AJ11" s="3">
+        <v>144</v>
+      </c>
       <c r="AK11" s="9">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="AL11" s="4">
         <f>SUM(AG11:AJ11)</f>
-        <v>0</v>
+        <v>666</v>
       </c>
       <c r="AM11" s="6" cm="1">
         <f t="array" ref="AM11">SUM(C11:F11+I11:L11+O11:R11+U11:X11+AA11:AD11+AG11:AJ11)</f>
-        <v>3511</v>
+        <v>4199</v>
       </c>
       <c r="AN11" s="8">
         <f>SUM(H11+N11+T11+Z11+AF11+AL11)</f>
-        <v>3607</v>
+        <v>4267</v>
       </c>
       <c r="AO11">
         <v>200</v>
       </c>
       <c r="AP11" s="11">
-        <v>166.36</v>
+        <v>175.62</v>
       </c>
       <c r="AQ11" s="11">
         <f>SUM((AO11-AP11)*0.7)</f>
-        <v>23.547999999999988</v>
+        <v>17.065999999999995</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -1979,131 +2019,139 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C12" s="3">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="D12" s="3">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="E12" s="3">
-        <v>198</v>
+        <v>154</v>
       </c>
       <c r="F12" s="3">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="G12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="H12" s="4">
         <f>SUM(C12:G12)</f>
-        <v>714</v>
+        <v>746</v>
       </c>
       <c r="I12" s="3">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="J12" s="3">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="K12" s="3">
-        <v>189</v>
+        <v>132</v>
       </c>
       <c r="L12" s="3">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="M12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="N12" s="4">
         <f>SUM(I12:L12)</f>
-        <v>685</v>
+        <v>657</v>
       </c>
       <c r="O12" s="3">
+        <v>179</v>
+      </c>
+      <c r="P12" s="3">
+        <v>173</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>169</v>
+      </c>
+      <c r="R12" s="3">
         <v>156</v>
       </c>
-      <c r="P12" s="3">
-        <v>174</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>150</v>
-      </c>
-      <c r="R12" s="3">
-        <v>184</v>
-      </c>
       <c r="S12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="T12" s="4">
         <f>SUM(O12:R12)</f>
-        <v>664</v>
+        <v>677</v>
       </c>
       <c r="U12" s="3">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="V12" s="3">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="W12" s="3">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="X12" s="3">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="Y12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="Z12" s="4">
         <f>SUM(U12:X12)</f>
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="AA12" s="3">
-        <v>203</v>
+        <v>155</v>
       </c>
       <c r="AB12" s="3">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="AC12" s="3">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="AD12" s="3">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AE12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="AF12" s="4">
         <f>SUM(AA12:AD12)</f>
-        <v>798</v>
-      </c>
-      <c r="AG12" s="3"/>
-      <c r="AH12" s="3"/>
-      <c r="AI12" s="3"/>
-      <c r="AJ12" s="3"/>
+        <v>712</v>
+      </c>
+      <c r="AG12" s="3">
+        <v>155</v>
+      </c>
+      <c r="AH12" s="3">
+        <v>136</v>
+      </c>
+      <c r="AI12" s="3">
+        <v>188</v>
+      </c>
+      <c r="AJ12" s="3">
+        <v>226</v>
+      </c>
       <c r="AK12" s="9">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="AL12" s="4">
         <f>SUM(AG12:AJ12)</f>
-        <v>0</v>
+        <v>705</v>
       </c>
       <c r="AM12" s="6" cm="1">
         <f t="array" ref="AM12">SUM(C12:F12+I12:L12+O12:R12+U12:X12+AA12:AD12+AG12:AJ12)</f>
-        <v>3533</v>
+        <v>4159</v>
       </c>
       <c r="AN12" s="8">
         <f>SUM(H12+N12+T12+Z12+AF12+AL12)</f>
-        <v>3601</v>
+        <v>4243</v>
       </c>
       <c r="AO12">
         <v>200</v>
       </c>
       <c r="AP12" s="11">
-        <v>175.62</v>
+        <v>169.44</v>
       </c>
       <c r="AQ12" s="11">
         <f>SUM((AO12-AP12)*0.7)</f>
-        <v>17.065999999999995</v>
+        <v>21.391999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -2111,131 +2159,139 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C13" s="3">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="D13" s="3">
-        <v>183</v>
+        <v>214</v>
       </c>
       <c r="E13" s="3">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="F13" s="3">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="H13" s="4">
         <f>SUM(C13:G13)</f>
-        <v>762</v>
+        <v>823</v>
       </c>
       <c r="I13" s="3">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="J13" s="3">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="K13" s="3">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="L13" s="3">
-        <v>163</v>
+        <v>194</v>
       </c>
       <c r="M13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="N13" s="4">
         <f>SUM(I13:L13)</f>
-        <v>705</v>
+        <v>781</v>
       </c>
       <c r="O13" s="3">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="P13" s="3">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="Q13" s="3">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="R13" s="3">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="S13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="T13" s="4">
         <f>SUM(O13:R13)</f>
-        <v>712</v>
+        <v>656</v>
       </c>
       <c r="U13" s="3">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="V13" s="3">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="W13" s="3">
-        <v>168</v>
+        <v>214</v>
       </c>
       <c r="X13" s="3">
-        <v>165</v>
+        <v>201</v>
       </c>
       <c r="Y13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="Z13" s="4">
         <f>SUM(U13:X13)</f>
-        <v>681</v>
+        <v>719</v>
       </c>
       <c r="AA13" s="3">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="AB13" s="3">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="AC13" s="3">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="AD13" s="3">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="AE13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AF13" s="4">
         <f>SUM(AA13:AD13)</f>
-        <v>659</v>
-      </c>
-      <c r="AG13" s="3"/>
-      <c r="AH13" s="3"/>
-      <c r="AI13" s="3"/>
-      <c r="AJ13" s="3"/>
+        <v>675</v>
+      </c>
+      <c r="AG13" s="3">
+        <v>128</v>
+      </c>
+      <c r="AH13" s="3">
+        <v>166</v>
+      </c>
+      <c r="AI13" s="3">
+        <v>160</v>
+      </c>
+      <c r="AJ13" s="3">
+        <v>117</v>
+      </c>
       <c r="AK13" s="9">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AL13" s="4">
         <f>SUM(AG13:AJ13)</f>
-        <v>0</v>
+        <v>571</v>
       </c>
       <c r="AM13" s="6" cm="1">
         <f t="array" ref="AM13">SUM(C13:F13+I13:L13+O13:R13+U13:X13+AA13:AD13+AG13:AJ13)</f>
-        <v>3427</v>
+        <v>4149</v>
       </c>
       <c r="AN13" s="8">
         <f>SUM(H13+N13+T13+Z13+AF13+AL13)</f>
-        <v>3519</v>
+        <v>4225</v>
       </c>
       <c r="AO13">
         <v>200</v>
       </c>
       <c r="AP13" s="11">
-        <v>167</v>
+        <v>173.04</v>
       </c>
       <c r="AQ13" s="11">
         <f>SUM((AO13-AP13)*0.7)</f>
-        <v>23.099999999999998</v>
+        <v>18.872000000000003</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -2243,131 +2299,139 @@
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C14" s="3">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="D14" s="3">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="E14" s="3">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="F14" s="3">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="G14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="H14" s="4">
         <f>SUM(C14:G14)</f>
-        <v>712</v>
+        <v>801</v>
       </c>
       <c r="I14" s="3">
-        <v>226</v>
+        <v>200</v>
       </c>
       <c r="J14" s="3">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="K14" s="3">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="L14" s="3">
         <v>204</v>
       </c>
       <c r="M14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="N14" s="4">
         <f>SUM(I14:L14)</f>
-        <v>813</v>
+        <v>789</v>
       </c>
       <c r="O14" s="3">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="P14" s="3">
-        <v>192</v>
+        <v>142</v>
       </c>
       <c r="Q14" s="3">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="R14" s="3">
-        <v>190</v>
+        <v>163</v>
       </c>
       <c r="S14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="T14" s="4">
         <f>SUM(O14:R14)</f>
-        <v>686</v>
+        <v>588</v>
       </c>
       <c r="U14" s="3">
+        <v>192</v>
+      </c>
+      <c r="V14" s="3">
+        <v>168</v>
+      </c>
+      <c r="W14" s="3">
         <v>157</v>
       </c>
-      <c r="V14" s="3">
-        <v>146</v>
-      </c>
-      <c r="W14" s="3">
-        <v>162</v>
-      </c>
       <c r="X14" s="3">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="Y14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="Z14" s="4">
         <f>SUM(U14:X14)</f>
-        <v>624</v>
+        <v>727</v>
       </c>
       <c r="AA14" s="3">
-        <v>159</v>
+        <v>188</v>
       </c>
       <c r="AB14" s="3">
-        <v>185</v>
+        <v>160</v>
       </c>
       <c r="AC14" s="3">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="AD14" s="3">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="AE14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="AF14" s="4">
         <f>SUM(AA14:AD14)</f>
-        <v>675</v>
-      </c>
-      <c r="AG14" s="3"/>
-      <c r="AH14" s="3"/>
-      <c r="AI14" s="3"/>
-      <c r="AJ14" s="3"/>
+        <v>702</v>
+      </c>
+      <c r="AG14" s="3">
+        <v>125</v>
+      </c>
+      <c r="AH14" s="3">
+        <v>122</v>
+      </c>
+      <c r="AI14" s="3">
+        <v>191</v>
+      </c>
+      <c r="AJ14" s="3">
+        <v>179</v>
+      </c>
       <c r="AK14" s="9">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="AL14" s="4">
         <f>SUM(AG14:AJ14)</f>
-        <v>0</v>
+        <v>617</v>
       </c>
       <c r="AM14" s="6" cm="1">
         <f t="array" ref="AM14">SUM(C14:F14+I14:L14+O14:R14+U14:X14+AA14:AD14+AG14:AJ14)</f>
-        <v>3402</v>
+        <v>4128</v>
       </c>
       <c r="AN14" s="8">
         <f>SUM(H14+N14+T14+Z14+AF14+AL14)</f>
-        <v>3510</v>
+        <v>4224</v>
       </c>
       <c r="AO14">
         <v>200</v>
       </c>
       <c r="AP14" s="11">
-        <v>161.47</v>
+        <v>166.36</v>
       </c>
       <c r="AQ14" s="11">
         <f>SUM((AO14-AP14)*0.7)</f>
-        <v>26.971</v>
+        <v>23.547999999999988</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -2375,123 +2439,139 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C15" s="3">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D15" s="3">
-        <v>199</v>
+        <v>183</v>
       </c>
       <c r="E15" s="3">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="F15" s="3">
-        <v>211</v>
+        <v>164</v>
       </c>
       <c r="G15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="H15" s="4">
         <f>SUM(C15:G15)</f>
-        <v>737</v>
+        <v>762</v>
       </c>
       <c r="I15" s="3">
-        <v>200</v>
+        <v>182</v>
       </c>
       <c r="J15" s="3">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="K15" s="3">
-        <v>220</v>
+        <v>158</v>
       </c>
       <c r="L15" s="3">
-        <v>203</v>
+        <v>163</v>
       </c>
       <c r="M15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="N15" s="4">
         <f>SUM(I15:L15)</f>
-        <v>813</v>
+        <v>705</v>
       </c>
       <c r="O15" s="3">
-        <v>222</v>
+        <v>155</v>
       </c>
       <c r="P15" s="3">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="Q15" s="3">
-        <v>228</v>
+        <v>180</v>
       </c>
       <c r="R15" s="3">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="S15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="T15" s="4">
         <f>SUM(O15:R15)</f>
-        <v>878</v>
+        <v>712</v>
       </c>
       <c r="U15" s="3">
-        <v>226</v>
+        <v>168</v>
       </c>
       <c r="V15" s="3">
-        <v>208</v>
+        <v>180</v>
       </c>
       <c r="W15" s="3">
-        <v>218</v>
+        <v>168</v>
       </c>
       <c r="X15" s="3">
-        <v>211</v>
+        <v>165</v>
       </c>
       <c r="Y15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="Z15" s="4">
         <f>SUM(U15:X15)</f>
-        <v>863</v>
-      </c>
-      <c r="AA15" s="3"/>
-      <c r="AB15" s="3"/>
-      <c r="AC15" s="3"/>
-      <c r="AD15" s="3"/>
+        <v>681</v>
+      </c>
+      <c r="AA15" s="3">
+        <v>135</v>
+      </c>
+      <c r="AB15" s="3">
+        <v>200</v>
+      </c>
+      <c r="AC15" s="3">
+        <v>158</v>
+      </c>
+      <c r="AD15" s="3">
+        <v>166</v>
+      </c>
       <c r="AE15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="AF15" s="4">
         <f>SUM(AA15:AD15)</f>
-        <v>0</v>
-      </c>
-      <c r="AG15" s="3"/>
-      <c r="AH15" s="3"/>
-      <c r="AI15" s="3"/>
-      <c r="AJ15" s="3"/>
+        <v>659</v>
+      </c>
+      <c r="AG15" s="3">
+        <v>158</v>
+      </c>
+      <c r="AH15" s="3">
+        <v>156</v>
+      </c>
+      <c r="AI15" s="3">
+        <v>158</v>
+      </c>
+      <c r="AJ15" s="3">
+        <v>191</v>
+      </c>
       <c r="AK15" s="9">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="AL15" s="4">
         <f>SUM(AG15:AJ15)</f>
-        <v>0</v>
+        <v>663</v>
       </c>
       <c r="AM15" s="6" cm="1">
         <f t="array" ref="AM15">SUM(C15:F15+I15:L15+O15:R15+U15:X15+AA15:AD15+AG15:AJ15)</f>
-        <v>3275</v>
+        <v>4090</v>
       </c>
       <c r="AN15" s="8">
         <f>SUM(H15+N15+T15+Z15+AF15+AL15)</f>
-        <v>3291</v>
+        <v>4182</v>
       </c>
       <c r="AO15">
         <v>200</v>
       </c>
       <c r="AP15" s="11">
-        <v>194.71</v>
+        <v>167</v>
       </c>
       <c r="AQ15" s="11">
         <f>SUM((AO15-AP15)*0.7)</f>
-        <v>3.7029999999999941</v>
+        <v>23.099999999999998</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -2499,131 +2579,139 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C16" s="3">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D16" s="3">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="E16" s="3">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="F16" s="3">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="G16" s="9">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="H16" s="4">
         <f>SUM(C16:G16)</f>
-        <v>780</v>
+        <v>712</v>
       </c>
       <c r="I16" s="3">
-        <v>145</v>
+        <v>226</v>
       </c>
       <c r="J16" s="3">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="K16" s="3">
-        <v>150</v>
+        <v>203</v>
       </c>
       <c r="L16" s="3">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="M16" s="9">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="N16" s="4">
         <f>SUM(I16:L16)</f>
-        <v>586</v>
+        <v>813</v>
       </c>
       <c r="O16" s="3">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="P16" s="3">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="Q16" s="3">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="R16" s="3">
-        <v>156</v>
+        <v>190</v>
       </c>
       <c r="S16" s="9">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="T16" s="4">
         <f>SUM(O16:R16)</f>
         <v>686</v>
       </c>
       <c r="U16" s="3">
-        <v>135</v>
+        <v>157</v>
       </c>
       <c r="V16" s="3">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="W16" s="3">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="X16" s="3">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="Y16" s="9">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="Z16" s="4">
         <f>SUM(U16:X16)</f>
-        <v>596</v>
+        <v>624</v>
       </c>
       <c r="AA16" s="3">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="AB16" s="3">
-        <v>121</v>
+        <v>185</v>
       </c>
       <c r="AC16" s="3">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="AD16" s="3">
+        <v>168</v>
+      </c>
+      <c r="AE16" s="9">
         <v>108</v>
-      </c>
-      <c r="AE16" s="9">
-        <v>132</v>
       </c>
       <c r="AF16" s="4">
         <f>SUM(AA16:AD16)</f>
-        <v>504</v>
-      </c>
-      <c r="AG16" s="3"/>
-      <c r="AH16" s="3"/>
-      <c r="AI16" s="3"/>
-      <c r="AJ16" s="3"/>
+        <v>675</v>
+      </c>
+      <c r="AG16" s="3">
+        <v>166</v>
+      </c>
+      <c r="AH16" s="3">
+        <v>152</v>
+      </c>
+      <c r="AI16" s="3">
+        <v>128</v>
+      </c>
+      <c r="AJ16" s="3">
+        <v>171</v>
+      </c>
       <c r="AK16" s="9">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="AL16" s="4">
         <f>SUM(AG16:AJ16)</f>
-        <v>0</v>
+        <v>617</v>
       </c>
       <c r="AM16" s="6" cm="1">
         <f t="array" ref="AM16">SUM(C16:F16+I16:L16+O16:R16+U16:X16+AA16:AD16+AG16:AJ16)</f>
-        <v>3020</v>
+        <v>4019</v>
       </c>
       <c r="AN16" s="8">
         <f>SUM(H16+N16+T16+Z16+AF16+AL16)</f>
-        <v>3152</v>
+        <v>4127</v>
       </c>
       <c r="AO16">
         <v>200</v>
       </c>
       <c r="AP16" s="11">
-        <v>152.86000000000001</v>
+        <v>161.47</v>
       </c>
       <c r="AQ16" s="11">
         <f>SUM((AO16-AP16)*0.7)</f>
-        <v>32.99799999999999</v>
+        <v>26.971</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -2631,123 +2719,139 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="C17" s="3">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="D17" s="3">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="E17" s="3">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="F17" s="3">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="G17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="H17" s="4">
         <f>SUM(C17:G17)</f>
-        <v>700</v>
+        <v>780</v>
       </c>
       <c r="I17" s="3">
-        <v>203</v>
+        <v>145</v>
       </c>
       <c r="J17" s="3">
-        <v>176</v>
+        <v>100</v>
       </c>
       <c r="K17" s="3">
-        <v>183</v>
+        <v>150</v>
       </c>
       <c r="L17" s="3">
-        <v>223</v>
+        <v>191</v>
       </c>
       <c r="M17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="N17" s="4">
         <f>SUM(I17:L17)</f>
-        <v>785</v>
+        <v>586</v>
       </c>
       <c r="O17" s="3">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P17" s="3">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="Q17" s="3">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="R17" s="3">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="S17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="T17" s="4">
         <f>SUM(O17:R17)</f>
-        <v>665</v>
+        <v>686</v>
       </c>
       <c r="U17" s="3">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="V17" s="3">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="W17" s="3">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="X17" s="3">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="Y17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="Z17" s="4">
         <f>SUM(U17:X17)</f>
-        <v>599</v>
-      </c>
-      <c r="AA17" s="3"/>
-      <c r="AB17" s="3"/>
-      <c r="AC17" s="3"/>
-      <c r="AD17" s="3"/>
+        <v>596</v>
+      </c>
+      <c r="AA17" s="3">
+        <v>114</v>
+      </c>
+      <c r="AB17" s="3">
+        <v>121</v>
+      </c>
+      <c r="AC17" s="3">
+        <v>161</v>
+      </c>
+      <c r="AD17" s="3">
+        <v>108</v>
+      </c>
       <c r="AE17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="AF17" s="4">
         <f>SUM(AA17:AD17)</f>
-        <v>0</v>
-      </c>
-      <c r="AG17" s="3"/>
-      <c r="AH17" s="3"/>
-      <c r="AI17" s="3"/>
-      <c r="AJ17" s="3"/>
+        <v>504</v>
+      </c>
+      <c r="AG17" s="3">
+        <v>138</v>
+      </c>
+      <c r="AH17" s="3">
+        <v>128</v>
+      </c>
+      <c r="AI17" s="3">
+        <v>126</v>
+      </c>
+      <c r="AJ17" s="3">
+        <v>153</v>
+      </c>
       <c r="AK17" s="9">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="AL17" s="4">
         <f>SUM(AG17:AJ17)</f>
-        <v>0</v>
+        <v>545</v>
       </c>
       <c r="AM17" s="6" cm="1">
         <f t="array" ref="AM17">SUM(C17:F17+I17:L17+O17:R17+U17:X17+AA17:AD17+AG17:AJ17)</f>
-        <v>2673</v>
+        <v>3565</v>
       </c>
       <c r="AN17" s="8">
         <f>SUM(H17+N17+T17+Z17+AF17+AL17)</f>
-        <v>2749</v>
+        <v>3697</v>
       </c>
       <c r="AO17">
         <v>200</v>
       </c>
       <c r="AP17" s="11">
-        <v>173.14</v>
+        <v>152.86000000000001</v>
       </c>
       <c r="AQ17" s="11">
         <f>SUM((AO17-AP17)*0.7)</f>
-        <v>18.802000000000007</v>
+        <v>32.99799999999999</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -2795,27 +2899,43 @@
         <f>SUM(I18:L18)</f>
         <v>806</v>
       </c>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
+      <c r="O18" s="3">
+        <v>202</v>
+      </c>
+      <c r="P18" s="3">
+        <v>158</v>
+      </c>
+      <c r="Q18" s="3">
+        <v>216</v>
+      </c>
+      <c r="R18" s="3">
+        <v>167</v>
+      </c>
       <c r="S18" s="9">
         <v>36</v>
       </c>
       <c r="T18" s="4">
         <f>SUM(O18:R18)</f>
-        <v>0</v>
-      </c>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
+        <v>743</v>
+      </c>
+      <c r="U18" s="3">
+        <v>179</v>
+      </c>
+      <c r="V18" s="3">
+        <v>183</v>
+      </c>
+      <c r="W18" s="3">
+        <v>212</v>
+      </c>
+      <c r="X18" s="3">
+        <v>212</v>
+      </c>
       <c r="Y18" s="9">
         <v>36</v>
       </c>
       <c r="Z18" s="4">
         <f>SUM(U18:X18)</f>
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="AA18" s="3"/>
       <c r="AB18" s="3"/>
@@ -2841,11 +2961,11 @@
       </c>
       <c r="AM18" s="6" cm="1">
         <f t="array" ref="AM18">SUM(C18:F18+I18:L18+O18:R18+U18:X18+AA18:AD18+AG18:AJ18)</f>
-        <v>1463</v>
+        <v>2992</v>
       </c>
       <c r="AN18" s="8">
         <f>SUM(H18+N18+T18+Z18+AF18+AL18)</f>
-        <v>1499</v>
+        <v>3028</v>
       </c>
       <c r="AO18">
         <v>200</v>
@@ -2863,74 +2983,90 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C19" s="3">
-        <v>183</v>
+        <v>148</v>
       </c>
       <c r="D19" s="3">
-        <v>174</v>
+        <v>134</v>
       </c>
       <c r="E19" s="3">
-        <v>207</v>
+        <v>164</v>
       </c>
       <c r="F19" s="3">
-        <v>216</v>
+        <v>178</v>
       </c>
       <c r="G19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="H19" s="4">
         <f>SUM(C19:G19)</f>
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="I19" s="3">
-        <v>174</v>
+        <v>203</v>
       </c>
       <c r="J19" s="3">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="K19" s="3">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="L19" s="3">
-        <v>136</v>
+        <v>223</v>
       </c>
       <c r="M19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="N19" s="4">
         <f>SUM(I19:L19)</f>
-        <v>646</v>
-      </c>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
+        <v>785</v>
+      </c>
+      <c r="O19" s="3">
+        <v>164</v>
+      </c>
+      <c r="P19" s="3">
+        <v>160</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>169</v>
+      </c>
+      <c r="R19" s="3">
+        <v>172</v>
+      </c>
       <c r="S19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="T19" s="4">
         <f>SUM(O19:R19)</f>
-        <v>0</v>
-      </c>
-      <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
+        <v>665</v>
+      </c>
+      <c r="U19" s="3">
+        <v>138</v>
+      </c>
+      <c r="V19" s="3">
+        <v>123</v>
+      </c>
+      <c r="W19" s="3">
+        <v>155</v>
+      </c>
+      <c r="X19" s="3">
+        <v>183</v>
+      </c>
       <c r="Y19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="Z19" s="4">
         <f>SUM(U19:X19)</f>
-        <v>0</v>
+        <v>599</v>
       </c>
       <c r="AA19" s="3"/>
       <c r="AB19" s="3"/>
       <c r="AC19" s="3"/>
       <c r="AD19" s="3"/>
       <c r="AE19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="AF19" s="4">
         <f>SUM(AA19:AD19)</f>
@@ -2941,7 +3077,7 @@
       <c r="AI19" s="3"/>
       <c r="AJ19" s="3"/>
       <c r="AK19" s="9">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="AL19" s="4">
         <f>SUM(AG19:AJ19)</f>
@@ -2949,21 +3085,21 @@
       </c>
       <c r="AM19" s="6" cm="1">
         <f t="array" ref="AM19">SUM(C19:F19+I19:L19+O19:R19+U19:X19+AA19:AD19+AG19:AJ19)</f>
-        <v>1426</v>
+        <v>2673</v>
       </c>
       <c r="AN19" s="8">
         <f>SUM(H19+N19+T19+Z19+AF19+AL19)</f>
-        <v>1446</v>
+        <v>2749</v>
       </c>
       <c r="AO19">
         <v>200</v>
       </c>
       <c r="AP19" s="11">
-        <v>192.5</v>
+        <v>173.14</v>
       </c>
       <c r="AQ19" s="11">
         <f>SUM((AO19-AP19)*0.7)</f>
-        <v>5.25</v>
+        <v>18.802000000000007</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -3258,7 +3394,7 @@
       <c r="F23" s="3"/>
       <c r="G23" s="9"/>
       <c r="H23" s="4">
-        <f t="shared" ref="H23:H34" si="0">SUM(C23:G23)</f>
+        <f t="shared" ref="H23:H24" si="0">SUM(C23:G23)</f>
         <v>0</v>
       </c>
       <c r="I23" s="3"/>
@@ -3267,7 +3403,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="9"/>
       <c r="N23" s="4">
-        <f t="shared" ref="N23:N34" si="1">SUM(I23:L23)</f>
+        <f t="shared" ref="N23:N24" si="1">SUM(I23:L23)</f>
         <v>0</v>
       </c>
       <c r="O23" s="3"/>
@@ -3276,7 +3412,7 @@
       <c r="R23" s="3"/>
       <c r="S23" s="9"/>
       <c r="T23" s="4">
-        <f t="shared" ref="T23:T34" si="2">SUM(O23:R23)</f>
+        <f t="shared" ref="T23:T24" si="2">SUM(O23:R23)</f>
         <v>0</v>
       </c>
       <c r="U23" s="3"/>
@@ -3285,7 +3421,7 @@
       <c r="X23" s="3"/>
       <c r="Y23" s="9"/>
       <c r="Z23" s="4">
-        <f t="shared" ref="Z23:Z34" si="3">SUM(U23:X23)</f>
+        <f t="shared" ref="Z23:Z24" si="3">SUM(U23:X23)</f>
         <v>0</v>
       </c>
       <c r="AA23" s="3"/>
@@ -3294,7 +3430,7 @@
       <c r="AD23" s="3"/>
       <c r="AE23" s="9"/>
       <c r="AF23" s="4">
-        <f t="shared" ref="AF23:AF34" si="4">SUM(AA23:AD23)</f>
+        <f t="shared" ref="AF23:AF24" si="4">SUM(AA23:AD23)</f>
         <v>0</v>
       </c>
       <c r="AG23" s="3"/>
@@ -3303,7 +3439,7 @@
       <c r="AJ23" s="3"/>
       <c r="AK23" s="9"/>
       <c r="AL23" s="4">
-        <f t="shared" ref="AL23:AL34" si="5">SUM(AG23:AJ23)</f>
+        <f t="shared" ref="AL23:AL24" si="5">SUM(AG23:AJ23)</f>
         <v>0</v>
       </c>
       <c r="AM23" s="6" cm="1">
@@ -3311,7 +3447,7 @@
         <v>0</v>
       </c>
       <c r="AN23" s="8">
-        <f t="shared" ref="AN23:AN34" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
+        <f t="shared" ref="AN23:AN24" si="6">SUM(H23+N23+T23+Z23+AF23+AL23)</f>
         <v>0</v>
       </c>
       <c r="AO23">
@@ -3319,7 +3455,7 @@
       </c>
       <c r="AP23" s="11"/>
       <c r="AQ23" s="11">
-        <f t="shared" ref="AQ23:AQ34" si="7">SUM((AO23-AP23)*0.7)</f>
+        <f t="shared" ref="AQ23:AQ24" si="7">SUM((AO23-AP23)*0.7)</f>
         <v>140</v>
       </c>
     </row>
@@ -3404,7 +3540,7 @@
       <c r="F25" s="3"/>
       <c r="G25" s="9"/>
       <c r="H25" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="H25:H34" si="8">SUM(C25:G25)</f>
         <v>0</v>
       </c>
       <c r="I25" s="3"/>
@@ -3413,7 +3549,7 @@
       <c r="L25" s="3"/>
       <c r="M25" s="9"/>
       <c r="N25" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="N25:N34" si="9">SUM(I25:L25)</f>
         <v>0</v>
       </c>
       <c r="O25" s="3"/>
@@ -3422,7 +3558,7 @@
       <c r="R25" s="3"/>
       <c r="S25" s="9"/>
       <c r="T25" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="T25:T34" si="10">SUM(O25:R25)</f>
         <v>0</v>
       </c>
       <c r="U25" s="3"/>
@@ -3431,7 +3567,7 @@
       <c r="X25" s="3"/>
       <c r="Y25" s="9"/>
       <c r="Z25" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="Z25:Z34" si="11">SUM(U25:X25)</f>
         <v>0</v>
       </c>
       <c r="AA25" s="3"/>
@@ -3440,7 +3576,7 @@
       <c r="AD25" s="3"/>
       <c r="AE25" s="9"/>
       <c r="AF25" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="AF25:AF34" si="12">SUM(AA25:AD25)</f>
         <v>0</v>
       </c>
       <c r="AG25" s="3"/>
@@ -3449,7 +3585,7 @@
       <c r="AJ25" s="3"/>
       <c r="AK25" s="9"/>
       <c r="AL25" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="AL25:AL34" si="13">SUM(AG25:AJ25)</f>
         <v>0</v>
       </c>
       <c r="AM25" s="6" cm="1">
@@ -3457,7 +3593,7 @@
         <v>0</v>
       </c>
       <c r="AN25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="AN25:AN34" si="14">SUM(H25+N25+T25+Z25+AF25+AL25)</f>
         <v>0</v>
       </c>
       <c r="AO25">
@@ -3465,7 +3601,7 @@
       </c>
       <c r="AP25" s="11"/>
       <c r="AQ25" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="AQ25:AQ34" si="15">SUM((AO25-AP25)*0.7)</f>
         <v>140</v>
       </c>
     </row>
@@ -3477,7 +3613,7 @@
       <c r="F26" s="3"/>
       <c r="G26" s="9"/>
       <c r="H26" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I26" s="3"/>
@@ -3486,7 +3622,7 @@
       <c r="L26" s="3"/>
       <c r="M26" s="9"/>
       <c r="N26" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O26" s="3"/>
@@ -3495,7 +3631,7 @@
       <c r="R26" s="3"/>
       <c r="S26" s="9"/>
       <c r="T26" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U26" s="3"/>
@@ -3504,7 +3640,7 @@
       <c r="X26" s="3"/>
       <c r="Y26" s="9"/>
       <c r="Z26" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA26" s="3"/>
@@ -3513,7 +3649,7 @@
       <c r="AD26" s="3"/>
       <c r="AE26" s="9"/>
       <c r="AF26" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG26" s="3"/>
@@ -3522,7 +3658,7 @@
       <c r="AJ26" s="3"/>
       <c r="AK26" s="9"/>
       <c r="AL26" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM26" s="6" cm="1">
@@ -3530,7 +3666,7 @@
         <v>0</v>
       </c>
       <c r="AN26" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO26">
@@ -3538,7 +3674,7 @@
       </c>
       <c r="AP26" s="11"/>
       <c r="AQ26" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3550,7 +3686,7 @@
       <c r="F27" s="3"/>
       <c r="G27" s="9"/>
       <c r="H27" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I27" s="3"/>
@@ -3559,7 +3695,7 @@
       <c r="L27" s="3"/>
       <c r="M27" s="9"/>
       <c r="N27" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O27" s="3"/>
@@ -3568,7 +3704,7 @@
       <c r="R27" s="3"/>
       <c r="S27" s="9"/>
       <c r="T27" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U27" s="3"/>
@@ -3577,7 +3713,7 @@
       <c r="X27" s="3"/>
       <c r="Y27" s="9"/>
       <c r="Z27" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA27" s="3"/>
@@ -3586,7 +3722,7 @@
       <c r="AD27" s="3"/>
       <c r="AE27" s="9"/>
       <c r="AF27" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG27" s="3"/>
@@ -3595,7 +3731,7 @@
       <c r="AJ27" s="3"/>
       <c r="AK27" s="9"/>
       <c r="AL27" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM27" s="6" cm="1">
@@ -3603,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="AN27" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO27">
@@ -3611,7 +3747,7 @@
       </c>
       <c r="AP27" s="11"/>
       <c r="AQ27" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3623,7 +3759,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="9"/>
       <c r="H28" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I28" s="3"/>
@@ -3632,7 +3768,7 @@
       <c r="L28" s="3"/>
       <c r="M28" s="9"/>
       <c r="N28" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O28" s="3"/>
@@ -3641,7 +3777,7 @@
       <c r="R28" s="3"/>
       <c r="S28" s="9"/>
       <c r="T28" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U28" s="3"/>
@@ -3650,7 +3786,7 @@
       <c r="X28" s="3"/>
       <c r="Y28" s="9"/>
       <c r="Z28" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA28" s="3"/>
@@ -3659,7 +3795,7 @@
       <c r="AD28" s="3"/>
       <c r="AE28" s="9"/>
       <c r="AF28" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG28" s="3"/>
@@ -3668,7 +3804,7 @@
       <c r="AJ28" s="3"/>
       <c r="AK28" s="9"/>
       <c r="AL28" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM28" s="6" cm="1">
@@ -3676,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="AN28" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO28">
@@ -3684,7 +3820,7 @@
       </c>
       <c r="AP28" s="11"/>
       <c r="AQ28" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3696,7 +3832,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="9"/>
       <c r="H29" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I29" s="3"/>
@@ -3705,7 +3841,7 @@
       <c r="L29" s="3"/>
       <c r="M29" s="9"/>
       <c r="N29" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O29" s="3"/>
@@ -3714,7 +3850,7 @@
       <c r="R29" s="3"/>
       <c r="S29" s="9"/>
       <c r="T29" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U29" s="3"/>
@@ -3723,7 +3859,7 @@
       <c r="X29" s="3"/>
       <c r="Y29" s="9"/>
       <c r="Z29" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA29" s="3"/>
@@ -3732,7 +3868,7 @@
       <c r="AD29" s="3"/>
       <c r="AE29" s="9"/>
       <c r="AF29" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG29" s="3"/>
@@ -3741,7 +3877,7 @@
       <c r="AJ29" s="3"/>
       <c r="AK29" s="9"/>
       <c r="AL29" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM29" s="6" cm="1">
@@ -3749,7 +3885,7 @@
         <v>0</v>
       </c>
       <c r="AN29" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO29">
@@ -3757,7 +3893,7 @@
       </c>
       <c r="AP29" s="11"/>
       <c r="AQ29" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3769,7 +3905,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="9"/>
       <c r="H30" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I30" s="3"/>
@@ -3778,7 +3914,7 @@
       <c r="L30" s="3"/>
       <c r="M30" s="9"/>
       <c r="N30" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O30" s="3"/>
@@ -3787,7 +3923,7 @@
       <c r="R30" s="3"/>
       <c r="S30" s="9"/>
       <c r="T30" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U30" s="3"/>
@@ -3796,7 +3932,7 @@
       <c r="X30" s="3"/>
       <c r="Y30" s="9"/>
       <c r="Z30" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA30" s="3"/>
@@ -3805,7 +3941,7 @@
       <c r="AD30" s="3"/>
       <c r="AE30" s="9"/>
       <c r="AF30" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG30" s="3"/>
@@ -3814,7 +3950,7 @@
       <c r="AJ30" s="3"/>
       <c r="AK30" s="9"/>
       <c r="AL30" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM30" s="6" cm="1">
@@ -3822,7 +3958,7 @@
         <v>0</v>
       </c>
       <c r="AN30" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO30">
@@ -3830,7 +3966,7 @@
       </c>
       <c r="AP30" s="11"/>
       <c r="AQ30" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3842,7 +3978,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="9"/>
       <c r="H31" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I31" s="3"/>
@@ -3851,7 +3987,7 @@
       <c r="L31" s="3"/>
       <c r="M31" s="9"/>
       <c r="N31" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O31" s="3"/>
@@ -3860,7 +3996,7 @@
       <c r="R31" s="3"/>
       <c r="S31" s="9"/>
       <c r="T31" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U31" s="3"/>
@@ -3869,7 +4005,7 @@
       <c r="X31" s="3"/>
       <c r="Y31" s="9"/>
       <c r="Z31" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA31" s="3"/>
@@ -3878,7 +4014,7 @@
       <c r="AD31" s="3"/>
       <c r="AE31" s="9"/>
       <c r="AF31" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG31" s="3"/>
@@ -3887,7 +4023,7 @@
       <c r="AJ31" s="3"/>
       <c r="AK31" s="9"/>
       <c r="AL31" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM31" s="6" cm="1">
@@ -3895,7 +4031,7 @@
         <v>0</v>
       </c>
       <c r="AN31" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO31">
@@ -3903,7 +4039,7 @@
       </c>
       <c r="AP31" s="11"/>
       <c r="AQ31" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3915,7 +4051,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="9"/>
       <c r="H32" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I32" s="3"/>
@@ -3924,7 +4060,7 @@
       <c r="L32" s="3"/>
       <c r="M32" s="9"/>
       <c r="N32" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O32" s="3"/>
@@ -3933,7 +4069,7 @@
       <c r="R32" s="3"/>
       <c r="S32" s="9"/>
       <c r="T32" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U32" s="3"/>
@@ -3942,7 +4078,7 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="9"/>
       <c r="Z32" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA32" s="3"/>
@@ -3951,7 +4087,7 @@
       <c r="AD32" s="3"/>
       <c r="AE32" s="9"/>
       <c r="AF32" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG32" s="3"/>
@@ -3960,7 +4096,7 @@
       <c r="AJ32" s="3"/>
       <c r="AK32" s="9"/>
       <c r="AL32" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM32" s="6" cm="1">
@@ -3968,7 +4104,7 @@
         <v>0</v>
       </c>
       <c r="AN32" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO32">
@@ -3976,7 +4112,7 @@
       </c>
       <c r="AP32" s="11"/>
       <c r="AQ32" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -3988,7 +4124,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="9"/>
       <c r="H33" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I33" s="3"/>
@@ -3997,7 +4133,7 @@
       <c r="L33" s="3"/>
       <c r="M33" s="9"/>
       <c r="N33" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O33" s="3"/>
@@ -4006,7 +4142,7 @@
       <c r="R33" s="3"/>
       <c r="S33" s="9"/>
       <c r="T33" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U33" s="3"/>
@@ -4015,7 +4151,7 @@
       <c r="X33" s="3"/>
       <c r="Y33" s="9"/>
       <c r="Z33" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA33" s="3"/>
@@ -4024,7 +4160,7 @@
       <c r="AD33" s="3"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG33" s="3"/>
@@ -4033,7 +4169,7 @@
       <c r="AJ33" s="3"/>
       <c r="AK33" s="9"/>
       <c r="AL33" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM33" s="6" cm="1">
@@ -4041,7 +4177,7 @@
         <v>0</v>
       </c>
       <c r="AN33" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO33">
@@ -4049,7 +4185,7 @@
       </c>
       <c r="AP33" s="11"/>
       <c r="AQ33" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>
@@ -4061,7 +4197,7 @@
       <c r="F34" s="3"/>
       <c r="G34" s="9"/>
       <c r="H34" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="I34" s="3"/>
@@ -4070,7 +4206,7 @@
       <c r="L34" s="3"/>
       <c r="M34" s="9"/>
       <c r="N34" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="O34" s="3"/>
@@ -4079,7 +4215,7 @@
       <c r="R34" s="3"/>
       <c r="S34" s="9"/>
       <c r="T34" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="U34" s="3"/>
@@ -4088,7 +4224,7 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="9"/>
       <c r="Z34" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="AA34" s="3"/>
@@ -4097,7 +4233,7 @@
       <c r="AD34" s="3"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG34" s="3"/>
@@ -4106,7 +4242,7 @@
       <c r="AJ34" s="3"/>
       <c r="AK34" s="9"/>
       <c r="AL34" s="4">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM34" s="6" cm="1">
@@ -4114,7 +4250,7 @@
         <v>0</v>
       </c>
       <c r="AN34" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="AO34">
@@ -4122,7 +4258,7 @@
       </c>
       <c r="AP34" s="11"/>
       <c r="AQ34" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="15"/>
         <v>140</v>
       </c>
     </row>

</xml_diff>